<commit_message>
v0.7.03: weapon tweaks, auto-pause, training dropdown, equip animation
- Compass returns at the same speed it was thrown
- Brush refunds only after two shots with no hits; stroke fx matches the hitbox
- Slower highlighter overheat cooldown
- Auto-pause when the tab is hidden or the window loses focus
- Touch settings: no panel fade, per-slider reset buttons
- Starting deck has one scatter
- Codex enemy and boss entries animate in and idle-bob
- Training menu weapon dropdown; refill toggle without wobble, whole cell toggles
- Light red hover on leave and summary buttons
- Equip animation in the weapon view

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -105,7 +105,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.02</t>
+      <t xml:space="preserve">beta v0.7.03</t>
     </r>
     <r>
       <rPr>
@@ -204,7 +204,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.02 </t>
+      <t xml:space="preserve">beta v0.7.03 </t>
     </r>
     <r>
       <rPr>
@@ -10807,24 +10807,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">次揮筆總命中 ≤ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">道時返還 </t>
+      <t xml:space="preserve">次揮筆都沒打中任何敵人時返還 </t>
     </r>
     <r>
       <rPr>
@@ -11026,7 +11009,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.35 </t>
+      <t xml:space="preserve">0.5 </t>
     </r>
     <r>
       <rPr>
@@ -11043,7 +11026,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
+      <t xml:space="preserve">8</t>
     </r>
     <r>
       <rPr>
@@ -11060,7 +11043,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2 </t>
+      <t xml:space="preserve">3 </t>
     </r>
     <r>
       <rPr>
@@ -11812,7 +11795,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" s="8" t="n">
         <v>2</v>
@@ -14421,7 +14404,7 @@
         <v>30</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
         <v>329</v>

</xml_diff>

<commit_message>
v0.7.05: fix touch controls drifting on mobile, compass rework
- Overlay canvas kept its scaled size after quality changes, stretching the canvas and pulling sticks toward the center; resize now reuses the real screen size and UI scale
- Compass: no reload, each compass refills ammo when it returns or expires
- Compass flies out and back at the same constant speed, including through the turn
- Compass passes through crates and ink barrels
- Changelog, README, stats sheet and version

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -105,7 +105,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.03</t>
+      <t xml:space="preserve">beta v0.7.05</t>
     </r>
     <r>
       <rPr>
@@ -204,7 +204,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.03 </t>
+      <t xml:space="preserve">beta v0.7.05 </t>
     </r>
     <r>
       <rPr>
@@ -11058,10 +11058,10 @@
     <t xml:space="preserve">圓規</t>
   </si>
   <si>
-    <t xml:space="preserve">回力鏢・穿透</t>
-  </si>
-  <si>
-    <t xml:space="preserve">回力鏢：飛出逐漸減速、到最遠處加速飛回手上，去回都穿透（可打兩次），撞牆彈回</t>
+    <t xml:space="preserve">回力鏢・飛回補彈</t>
+  </si>
+  <si>
+    <t xml:space="preserve">回力鏢：以固定速度飛出再飛回手上，去回都穿透（可打兩次），穿過紙箱與墨水桶，撞牆彈回；不需換彈，飛回即補回一發</t>
   </si>
 </sst>
 </file>
@@ -14424,7 +14424,7 @@
       </c>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>313</v>
       </c>
@@ -14456,7 +14456,7 @@
         <v>20</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>0.55</v>
+        <v>0.38</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
v0.7.06: easier normal rooms, dash i-frames, straight compass, touch skill-only casting
- Lower story room budgets and HP growth, no elite rooms in act 1, slower endless scaling; boss HP unchanged
- Brief invulnerability after dashing
- Compass flies straight out and straight back toward the player
- Touch: hand cards are view-only, skill buttons cast, no detail tooltip while casting, non-directional cards cast on tap
- Popups sized to content on small screens; larger training picker cards
- Default quality high on first launch

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -105,7 +105,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.05</t>
+      <t xml:space="preserve">beta v0.7.06</t>
     </r>
     <r>
       <rPr>
@@ -204,7 +204,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.05 </t>
+      <t xml:space="preserve">beta v0.7.06 </t>
     </r>
     <r>
       <rPr>
@@ -11061,7 +11061,7 @@
     <t xml:space="preserve">回力鏢・飛回補彈</t>
   </si>
   <si>
-    <t xml:space="preserve">回力鏢：以固定速度飛出再飛回手上，去回都穿透（可打兩次），穿過紙箱與墨水桶，撞牆彈回；不需換彈，飛回即補回一發</t>
+    <t xml:space="preserve">回力鏢：直線飛出、以同樣速度直線飛回手上，去回都穿透（可打兩次），穿過紙箱與墨水桶，撞牆彈回；不需換彈，飛回即補回一發</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
v0.7.07: device toast, effect timers, cast origin, card fixes, grade tooltip
- Replace the touch notice popup with a toast on every input-device switch
- Duration bar under the player for timed card effects (soonest to expire), clone bar on the clone
- Cards cast from the player position at the moment of pressing
- Summary grade shows points, formula and thresholds on hover or tap
- Eraser preview matches the swept sector; sweep line covers the whole cone
- Giant pen wider and stronger; pierce pen passes walls and ramps damage per enemy
- Stop player flicker while paused in the training picker; fit weapon card text

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -105,7 +105,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.06</t>
+      <t xml:space="preserve">beta v0.7.07</t>
     </r>
     <r>
       <rPr>
@@ -204,7 +204,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.06 </t>
+      <t xml:space="preserve">beta v0.7.07 </t>
     </r>
     <r>
       <rPr>
@@ -1028,7 +1028,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">34</t>
+      <t xml:space="preserve">34
+ramp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
     </r>
   </si>
   <si>
@@ -1069,17 +1089,37 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">36</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">射出巨型筆尖，貫穿路徑上所有敵人，造成 </t>
+      <t xml:space="preserve">36
+ramp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">射出巨型筆尖，穿過牆壁並貫穿路徑上所有敵人，造成 </t>
     </r>
     <r>
       <rPr>
@@ -1096,17 +1136,34 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">射出巨型筆尖，貫穿路徑上所有敵人，造成 </t>
+      <t xml:space="preserve">傷害；每貫穿一名敵人，傷害再提升 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">射出巨型筆尖，穿過牆壁並貫穿路徑上所有敵人，造成 </t>
     </r>
     <r>
       <rPr>
@@ -1123,7 +1180,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">傷害。</t>
+      <t xml:space="preserve">傷害；每貫穿一名敵人，傷害再提升 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
     </r>
   </si>
   <si>
@@ -7554,7 +7628,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150
+      <t xml:space="preserve">210
 </t>
     </r>
     <r>
@@ -7574,7 +7648,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.6</t>
+      <t xml:space="preserve">2.8</t>
     </r>
   </si>
   <si>
@@ -7595,7 +7669,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">200
+      <t xml:space="preserve">280
 </t>
     </r>
     <r>
@@ -7615,7 +7689,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.9</t>
+      <t xml:space="preserve">3.3</t>
     </r>
   </si>
   <si>
@@ -7634,7 +7708,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150 </t>
+      <t xml:space="preserve">210 </t>
     </r>
     <r>
       <rPr>
@@ -7661,7 +7735,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">200 </t>
+      <t xml:space="preserve">280 </t>
     </r>
     <r>
       <rPr>
@@ -11819,7 +11893,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
         <v>44</v>
       </c>

</xml_diff>

<commit_message>
v0.9.05: compass uses a cooldown instead of a magazine
- Compass has no ammo or reload; each throw starts a 1.2s cooldown (shortened by rapid-fire effects)
- Ammo ticks under the player become a cooldown bar for cooldown weapons
- Weapon screen shows damage and cooldown; removed the return-refill logic
- Stats sheet updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="370">
   <si>
     <r>
       <rPr>
@@ -11132,10 +11132,35 @@
     <t xml:space="preserve">圓規</t>
   </si>
   <si>
-    <t xml:space="preserve">回力鏢・飛回補彈</t>
-  </si>
-  <si>
-    <t xml:space="preserve">回力鏢：直線飛出、以同樣速度直線飛回手上，去回都穿透（可打兩次），穿過紙箱與墨水桶，撞牆彈回；不需換彈，飛回即補回一發</t>
+    <t xml:space="preserve">回力鏢・冷卻制</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回力鏢：直線飛出、以同樣速度直線飛回手上，去回都穿透（可打兩次），穿過紙箱與墨水桶，撞牆彈回
+冷卻制：沒有彈匣與換彈，每次丟出後冷卻 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒（射擊間隔欄填的是冷卻時間）</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -14498,7 +14523,7 @@
       </c>
       <c r="O6" s="10"/>
     </row>
-    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>313</v>
       </c>
@@ -14518,13 +14543,13 @@
         <v>1</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="I7" s="8" t="n">
-        <v>1</v>
+        <v>1.2</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>329</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -14537,7 +14562,7 @@
       </c>
       <c r="M7" s="7" t="n">
         <f aca="false">ROUND(E7*F7/G7,1)</f>
-        <v>36.4</v>
+        <v>16.7</v>
       </c>
       <c r="N7" s="7" t="s">
         <v>369</v>

</xml_diff>

<commit_message>
beta v0.9.07: notebook-style choice panel, varied peace layouts, brush distance tiers, compass cooldown 1.8s, weapon values beside bars, concise tutorial
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -10915,7 +10915,93 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">發</t>
+      <t xml:space="preserve">發
+距離分段傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">格內 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">格內 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，更遠 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（傷害欄填最遠的基礎值）</t>
     </r>
   </si>
   <si>
@@ -11151,7 +11237,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.2 </t>
+      <t xml:space="preserve">1.8 </t>
     </r>
     <r>
       <rPr>
@@ -14385,7 +14471,7 @@
       <c r="N3" s="7"/>
       <c r="O3" s="10"/>
     </row>
-    <row r="4" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
         <v>355</v>
       </c>
@@ -14543,7 +14629,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>329</v>
@@ -14562,7 +14648,7 @@
       </c>
       <c r="M7" s="7" t="n">
         <f aca="false">ROUND(E7*F7/G7,1)</f>
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
         <v>369</v>

</xml_diff>

<commit_message>
beta v0.9.09: training minigame test, picker home button, pencil buff, per-act timed progress bar, 10-level cap with level-up show, animated results under score, interact bells, touch nudges, unarmed peace rooms
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -3685,6 +3685,298 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">mark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">標記</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">標記目標附近的一名敵人，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內受到的傷害變為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">標記目標附近的一名敵人，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內受到的傷害變為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍。</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">haste</t>
   </si>
   <si>
@@ -3921,10 +4213,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">mark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">標記</t>
+    <t xml:space="preserve">inkMine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">墨水地雷</t>
   </si>
   <si>
     <r>
@@ -3954,55 +4246,38 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6
+      <t xml:space="preserve">傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.6
 </t>
     </r>
     <r>
@@ -4012,18 +4287,112 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍率：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
+      <t xml:space="preserve">傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">70</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在地上埋一顆地雷，敵人靠近時爆炸，半徑 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">內造成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在地上埋一顆地雷，敵人靠近時爆炸，半徑 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">內造成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">70 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">blot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">吸墨紙</t>
   </si>
   <si>
     <r>
@@ -4043,7 +4412,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3.5
+      <t xml:space="preserve">4
 </t>
     </r>
     <r>
@@ -4053,55 +4422,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8
+      <t xml:space="preserve">每次：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4
 </t>
     </r>
     <r>
@@ -4111,112 +4442,18 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍率：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">標記目標附近的一名敵人，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內受到的傷害變為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">倍。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">標記目標附近的一名敵人，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內受到的傷害變為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">倍。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">inkMine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">墨水地雷</t>
+      <t xml:space="preserve">上限：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4227,6 +4464,26 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每次：</t>
     </r>
     <r>
       <rPr>
@@ -4246,18 +4503,342 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
+      <t xml:space="preserve">上限：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">吸走身邊半徑 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">內的所有敵彈，每吸 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">發獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水（最多 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">吸走身邊半徑 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">內的所有敵彈，每吸 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">發獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水（最多 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">dualWield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">雙持</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內每次射擊都會同時射出兩發。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內每次射擊都會同時射出兩發。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">釘住</t>
   </si>
   <si>
     <r>
@@ -4277,7 +4858,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3.6
+      <t xml:space="preserve">3.2
 </t>
     </r>
     <r>
@@ -4287,112 +4868,56 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">70</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在地上埋一顆地雷，敵人靠近時爆炸，半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在地上埋一顆地雷，敵人靠近時爆炸，半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">70 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">blot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">吸墨紙</t>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.5</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4422,17 +4947,207 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">每次：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">把目標附近半徑 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">內的敵人釘在原地 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒（首領效果減為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">把目標附近半徑 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">內的敵人釘在原地 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒（首領效果減為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">chain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">連鎖墨線</t>
+  </si>
+  <si>
+    <t xml:space="preserve">連鎖跳躍</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">跳躍次數：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5
 </t>
     </r>
     <r>
@@ -4442,38 +5157,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">上限：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">半徑：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5.5
+      <t xml:space="preserve">傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25
 </t>
     </r>
     <r>
@@ -4483,17 +5177,38 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">每次：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3
+      <t xml:space="preserve">距離：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">跳躍次數：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7
 </t>
     </r>
     <r>
@@ -4503,362 +5218,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">上限：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">吸走身邊半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內的所有敵彈，每吸 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">發獲得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水（最多 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">吸走身邊半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5.5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內的所有敵彈，每吸 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">發獲得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水（最多 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">dualWield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">雙持</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內每次射擊都會同時射出兩發。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內每次射擊都會同時射出兩發。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">pin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">釘住</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">半徑：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.2
+      <t xml:space="preserve">傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30
 </t>
     </r>
     <r>
@@ -4868,256 +5238,105 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2.5</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">半徑：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.5</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">把目標附近半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內的敵人釘在原地 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2.5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒（首領效果減為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">把目標附近半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內的敵人釘在原地 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒（首領效果減為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）。</t>
+      <t xml:space="preserve">距離：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨線在敵人之間跳躍 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次，每次造成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨線在敵人之間跳躍 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次，每次造成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害。</t>
     </r>
   </si>
   <si>
@@ -5294,225 +5513,6 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">傷害，並切掉碰到的敵彈。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">chain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">連鎖墨線</t>
-  </si>
-  <si>
-    <t xml:space="preserve">連鎖跳躍</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">跳躍次數：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">距離：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">跳躍次數：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">距離：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨線在敵人之間跳躍 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次，每次造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨線在敵人之間跳躍 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次，每次造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
     </r>
   </si>
   <si>
@@ -11268,7 +11268,31 @@
     <t xml:space="preserve">音鈴指揮</t>
   </si>
   <si>
-    <t xml:space="preserve">我會依序敲響四個音鈴。看清楚順序後，走進音鈴腳下的圈圈，照同樣順序踩一遍！</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">我會依序敲響四個音鈴。看清楚順序後，走到音鈴旁按 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">F</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（觸控按互動鍵）照同樣順序敲一遍！</t>
+    </r>
   </si>
   <si>
     <r>
@@ -11346,27 +11370,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.2
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">踏板半徑：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1.1
+      <t xml:space="preserve">0.4
+reach</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.7
 </t>
     </r>
     <r>
@@ -18935,7 +18959,7 @@
       </c>
       <c r="P16" s="10"/>
     </row>
-    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>144</v>
       </c>
@@ -18949,14 +18973,16 @@
         <v>118</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G17" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>14</v>
+      </c>
       <c r="H17" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17" s="8" t="n">
         <v>0</v>
@@ -18973,15 +18999,15 @@
       <c r="M17" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="N17" s="6" t="s">
+      <c r="N17" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="O17" s="6" t="s">
+      <c r="O17" s="7" t="s">
         <v>149</v>
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
         <v>150</v>
       </c>
@@ -18995,14 +19021,12 @@
         <v>118</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G18" s="8" t="n">
-        <v>14</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G18" s="8"/>
       <c r="H18" s="8" t="n">
         <v>3</v>
       </c>
@@ -19021,10 +19045,10 @@
       <c r="M18" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="N18" s="7" t="s">
+      <c r="N18" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="O18" s="7" t="s">
+      <c r="O18" s="6" t="s">
         <v>155</v>
       </c>
       <c r="P18" s="10"/>
@@ -19052,7 +19076,7 @@
         <v>10</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I19" s="8" t="n">
         <v>0</v>
@@ -19098,7 +19122,7 @@
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I20" s="8" t="n">
         <v>0</v>
@@ -19144,7 +19168,7 @@
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I21" s="8" t="n">
         <v>0</v>
@@ -19192,7 +19216,7 @@
         <v>12</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I22" s="8" t="n">
         <v>0</v>
@@ -19217,7 +19241,7 @@
       </c>
       <c r="P22" s="10"/>
     </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
         <v>180</v>
       </c>
@@ -19231,16 +19255,14 @@
         <v>36</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>59</v>
+        <v>182</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>9</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G23" s="8"/>
       <c r="H23" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I23" s="8" t="n">
         <v>0</v>
@@ -19252,25 +19274,25 @@
         <v>2</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N23" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O23" s="7" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P23" s="10"/>
     </row>
-    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>35</v>
@@ -19279,14 +19301,16 @@
         <v>36</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>188</v>
+        <v>59</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G24" s="8"/>
+        <v>38</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>9</v>
+      </c>
       <c r="H24" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I24" s="8" t="n">
         <v>0</v>
@@ -19334,7 +19358,7 @@
         <v>12</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I25" s="8" t="n">
         <v>0</v>
@@ -19382,7 +19406,7 @@
         <v>9</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I26" s="8" t="n">
         <v>0</v>
@@ -19428,7 +19452,7 @@
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I27" s="8" t="n">
         <v>0</v>
@@ -19474,7 +19498,7 @@
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I28" s="8" t="n">
         <v>0</v>
@@ -19522,7 +19546,7 @@
         <v>10</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I29" s="8" t="n">
         <v>0</v>
@@ -19664,7 +19688,7 @@
         <v>16</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I32" s="13" t="n">
         <v>0</v>
@@ -19710,7 +19734,7 @@
       </c>
       <c r="G33" s="13"/>
       <c r="H33" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I33" s="13" t="n">
         <v>0</v>
@@ -19758,7 +19782,7 @@
         <v>12</v>
       </c>
       <c r="H34" s="13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I34" s="13" t="n">
         <v>0</v>
@@ -19804,7 +19828,7 @@
       </c>
       <c r="G35" s="13"/>
       <c r="H35" s="13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I35" s="13" t="n">
         <v>0</v>
@@ -19852,7 +19876,7 @@
         <v>22</v>
       </c>
       <c r="H36" s="13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I36" s="13" t="n">
         <v>0</v>
@@ -19898,7 +19922,7 @@
       </c>
       <c r="G37" s="13"/>
       <c r="H37" s="13" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I37" s="13" t="n">
         <v>0</v>
@@ -19944,7 +19968,7 @@
       </c>
       <c r="G38" s="13"/>
       <c r="H38" s="13" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I38" s="13" t="n">
         <v>0</v>
@@ -20712,7 +20736,7 @@
         <v>354</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>1</v>
@@ -20721,7 +20745,7 @@
         <v>0.09</v>
       </c>
       <c r="H3" s="8" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="I3" s="8" t="n">
         <v>1.4</v>
@@ -20737,7 +20761,7 @@
       </c>
       <c r="M3" s="7" t="n">
         <f aca="false">ROUND(E3*F3/G3,1)</f>
-        <v>50</v>
+        <v>55.6</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="10"/>
@@ -20796,7 +20820,7 @@
         <v>360</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>361</v>
@@ -20842,7 +20866,7 @@
         <v>364</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>365</v>
@@ -20888,7 +20912,7 @@
         <v>367</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>368</v>

</xml_diff>

<commit_message>
beta v0.9.11: shop shelves, brush sweep, echo/time-stop ults, summary drawer
- Gacha odds on separate lines; minigame host speaks win/lose lines
- Training settings: map preview no longer touches weapon dropdown
- Brush: horizontal sweep hitbox, 30/20/15 by distance; only brush and compass clear bullets
- Smooth random-weapon carousel centered in frame
- Stationery shop items displayed on stands, bought via interact
- Device-specific UI wording for touch vs mouse/keyboard
- Peace-room ink can overflow the cap once
- Echo recasts the last used ult with its cutin and fog vignette; time stop fully freezes bosses
- Summary details as a torn paper drawer grouped by act with damage dealt/taken and running total
- Shadow minigame leaves a red trail; training test room has three always-open doors

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -6947,7 +6947,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">免費重播本房間你上一張打出的卡（目標相同）；若還沒出過牌則獲得 </t>
+      <t xml:space="preserve">免費再施放一次你上一張使用的特殊卡（自動瞄準最近的敵人）；若還沒用過特殊卡則獲得 </t>
     </r>
     <r>
       <rPr>
@@ -7837,24 +7837,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒：所有敵人與敵彈完全靜止（首領效果減為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）。</t>
+      <t xml:space="preserve">秒：所有敵人與敵彈完全靜止，首領也不例外。</t>
     </r>
   </si>
   <si>
@@ -7881,24 +7864,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒：所有敵人與敵彈完全靜止（首領效果減為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）。</t>
+      <t xml:space="preserve">秒：所有敵人與敵彈完全靜止，首領也不例外。</t>
     </r>
   </si>
   <si>
@@ -10787,7 +10753,7 @@
     <t xml:space="preserve">毛筆</t>
   </si>
   <si>
-    <t xml:space="preserve">揮灑墨痕・近距離加傷</t>
+    <t xml:space="preserve">橫掃墨痕・可擦敵彈</t>
   </si>
   <si>
     <r>
@@ -10805,7 +10771,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">5 </t>
+      <t xml:space="preserve">1 </t>
     </r>
     <r>
       <rPr>
@@ -10831,42 +10797,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">揮筆擦除身前敵彈（半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4.2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">、角度 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">）
-距離分段傷害：</t>
+      <t xml:space="preserve">距離分段傷害：</t>
     </r>
     <r>
       <rPr>
@@ -10892,7 +10823,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">25</t>
+      <t xml:space="preserve">30</t>
     </r>
     <r>
       <rPr>
@@ -11283,15 +11214,15 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（觸控按互動鍵）照同樣順序敲一遍！</t>
+      <t xml:space="preserve">F </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">照同樣順序敲一遍！</t>
     </r>
   </si>
   <si>
@@ -14896,24 +14827,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">站在「丟」字發射台上瞄準垃圾桶，看準旁邊力道條的高度按 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（觸控按互動鍵）丟出。有三次機會！</t>
+      <t xml:space="preserve">站在「丟」字發射台上，用滑鼠瞄準垃圾桶，看準旁邊力道條的高度按 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">F </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">丟出。有三次機會！</t>
     </r>
   </si>
   <si>
@@ -16410,7 +16341,87 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.35</t>
+      <t xml:space="preserve">0.35
+trail</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90
+trailR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
+trailGap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.28
+trailLife</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
     </r>
   </si>
   <si>
@@ -20841,7 +20852,7 @@
       <c r="N3" s="7"/>
       <c r="O3" s="10"/>
     </row>
-    <row r="4" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
         <v>355</v>
       </c>
@@ -20858,7 +20869,7 @@
         <v>15</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>0.62</v>
@@ -20880,7 +20891,7 @@
       </c>
       <c r="M4" s="7" t="n">
         <f aca="false">ROUND(E4*F4/G4,1)</f>
-        <v>121</v>
+        <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
         <v>358</v>
@@ -21305,7 +21316,7 @@
       </c>
       <c r="F14" s="10"/>
     </row>
-    <row r="15" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>437</v>
       </c>

</xml_diff>

<commit_message>
beta v0.9.15: tutorial deck step and fixes, dual highlighter beams, blot range cast, deck scroll
- Tutorial: always pen, cancel-cast goal alongside card casting, new deck/details step, ult step waits for the hit, clear leftovers without damage numbers
- Boss death clears remaining enemies without 99999 damage popups
- Memory bells: random 4-6 rings, pendulum swing animation
- Touch deck view scrolls and only closes via the close button
- Reduced motion zeroes jitter and restores it when turned off
- Blot shows its radius and casts on slide-out (touch) or second press (keys)
- Compass miss cooldown cut is smaller
- Dual wield: 6 s, highlighter fires two parallel beams with aim between, refreshed codex animation
- Ink vortex deals 100 (140 upgraded) when it only hits one enemy
- Codex open/close animation

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="469">
   <si>
     <r>
       <rPr>
@@ -4293,6 +4293,9 @@
     <t xml:space="preserve">吸墨紙</t>
   </si>
   <si>
+    <t xml:space="preserve">自身範圍（滑出施放）</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -6708,18 +6711,18 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
+      <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
     </r>
     <r>
       <rPr>
@@ -6889,7 +6892,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">90</t>
+      <t xml:space="preserve">90
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">單體傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
     </r>
   </si>
   <si>
@@ -6988,7 +7011,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">120</t>
+      <t xml:space="preserve">120
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">單體傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">140</t>
     </r>
   </si>
   <si>
@@ -7049,6 +7092,40 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">傷害；只炸到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人時改為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">傷害。</t>
     </r>
   </si>
@@ -7103,6 +7180,40 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">120 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害；只炸到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人時改為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">140 </t>
     </r>
     <r>
       <rPr>
@@ -10956,7 +11067,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">40%
+      <t xml:space="preserve">70%
 </t>
     </r>
     <r>
@@ -11043,7 +11154,41 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">我會依序敲響四個音鈴。看清楚順序後，走到音鈴旁按 </t>
+      <t xml:space="preserve">我會在四個音鈴上連續敲 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">下。看清楚順序後，走到音鈴旁按 </t>
     </r>
     <r>
       <rPr>
@@ -11169,112 +11314,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">序列長度：第</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">幕 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／第</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">幕 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／第</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">幕 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5
+      <t xml:space="preserve">序列長度：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[4, 6]
 </t>
     </r>
     <r>
@@ -19569,7 +19619,7 @@
         <v>132</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>52</v>
+        <v>158</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8" t="n">
@@ -19585,25 +19635,25 @@
         <v>1</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O19" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>35</v>
@@ -19633,25 +19683,25 @@
         <v>2</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="N20" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="O20" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>35</v>
@@ -19660,7 +19710,7 @@
         <v>36</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>52</v>
@@ -19679,25 +19729,25 @@
         <v>2</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N21" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="O21" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>35</v>
@@ -19727,25 +19777,25 @@
         <v>2</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="M22" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="O22" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>35</v>
@@ -19754,7 +19804,7 @@
         <v>36</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>60</v>
@@ -19775,25 +19825,25 @@
         <v>3</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N23" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O23" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>35</v>
@@ -19823,25 +19873,25 @@
         <v>2</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N24" s="7" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O24" s="7" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>35</v>
@@ -19872,22 +19922,22 @@
         <v>114</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="N25" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O25" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>35</v>
@@ -19915,25 +19965,25 @@
         <v>1</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N26" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="O26" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="P26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>35</v>
@@ -19963,28 +20013,28 @@
         <v>3</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N27" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="O27" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="P27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>36</v>
@@ -20011,28 +20061,28 @@
         <v>4</v>
       </c>
       <c r="L28" s="14" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M28" s="14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N28" s="12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="O28" s="12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="P28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D29" s="12" t="s">
         <v>111</v>
@@ -20057,28 +20107,28 @@
         <v>2</v>
       </c>
       <c r="L29" s="14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="M29" s="14" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="N29" s="12" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O29" s="12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="P29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>36</v>
@@ -20105,28 +20155,28 @@
         <v>3</v>
       </c>
       <c r="L30" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="M30" s="14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="N30" s="12" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="O30" s="12" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="P30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>36</v>
@@ -20151,13 +20201,13 @@
         <v>2</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O31" s="12" t="s">
         <v>87</v>
@@ -20166,19 +20216,19 @@
     </row>
     <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>111</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>52</v>
@@ -20197,28 +20247,28 @@
         <v>2</v>
       </c>
       <c r="L32" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M32" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N32" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="O32" s="12" t="s">
         <v>87</v>
       </c>
       <c r="P32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D33" s="12" t="s">
         <v>36</v>
@@ -20245,28 +20295,28 @@
         <v>4</v>
       </c>
       <c r="L33" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="M33" s="14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="N33" s="12" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O33" s="12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="P33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>36</v>
@@ -20291,34 +20341,34 @@
         <v>3</v>
       </c>
       <c r="L34" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M34" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N34" s="11" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O34" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="P34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D35" s="12" t="s">
         <v>36</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F35" s="12" t="s">
         <v>38</v>
@@ -20339,28 +20389,28 @@
         <v>3</v>
       </c>
       <c r="L35" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M35" s="14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N35" s="12" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="O35" s="12" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="P35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>111</v>
@@ -20388,25 +20438,25 @@
         <v>114</v>
       </c>
       <c r="M36" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="N36" s="12" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="O36" s="12" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="P36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D37" s="12" t="s">
         <v>36</v>
@@ -20431,13 +20481,13 @@
         <v>3</v>
       </c>
       <c r="L37" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="M37" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="N37" s="12" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="O37" s="12" t="s">
         <v>87</v>
@@ -20481,13 +20531,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B1" s="15" t="n">
         <v>2.5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D1" s="15" t="n">
         <v>2</v>
@@ -20504,40 +20554,40 @@
         <v>20</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>32</v>
@@ -20545,13 +20595,13 @@
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>38</v>
@@ -20573,7 +20623,7 @@
         <v>10</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>1</v>
@@ -20586,22 +20636,22 @@
         <v>1</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="P4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>52</v>
@@ -20634,22 +20684,22 @@
         <v>2</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="P5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>46</v>
@@ -20671,7 +20721,7 @@
         <v>8.5</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K6" s="8" t="n">
         <v>1.5</v>
@@ -20684,22 +20734,22 @@
         <v>2</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="P6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>44</v>
@@ -20728,22 +20778,22 @@
         <v>2</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="P7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>26</v>
@@ -20772,22 +20822,22 @@
         <v>1</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="P8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>58</v>
@@ -20809,7 +20859,7 @@
         <v>6</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="K9" s="8" t="n">
         <v>1.5</v>
@@ -20822,22 +20872,22 @@
         <v>2</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="P9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>90</v>
@@ -20866,22 +20916,22 @@
         <v>2</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="P10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>14</v>
@@ -20911,25 +20961,25 @@
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="P11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="176.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D12" s="13" t="n">
         <v>900</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F12" s="13" t="n">
         <v>0.8</v>
@@ -20948,32 +20998,32 @@
         <v>4</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="12" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="O12" s="11" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="P12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F13" s="13" t="n">
         <v>2.2</v>
@@ -20992,32 +21042,32 @@
         <v>4</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="12" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="P13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>1300</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>0</v>
@@ -21036,14 +21086,14 @@
         <v>4</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="12" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="P14" s="10"/>
     </row>
@@ -21093,37 +21143,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>274</v>
-      </c>
       <c r="K1" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -21131,16 +21181,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -21175,16 +21225,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -21219,16 +21269,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -21259,22 +21309,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -21305,22 +21355,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -21338,10 +21388,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -21351,22 +21401,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -21378,10 +21428,10 @@
         <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -21397,7 +21447,7 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -21429,19 +21479,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -21449,289 +21499,289 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="189.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -21766,13 +21816,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -21780,13 +21830,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -21796,13 +21846,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -21812,13 +21862,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -21828,13 +21878,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -21844,13 +21894,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -21860,13 +21910,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -21876,13 +21926,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -21892,13 +21942,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -21908,13 +21958,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -21924,13 +21974,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -21940,13 +21990,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -21956,13 +22006,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -21972,13 +22022,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -21988,13 +22038,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -22004,13 +22054,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -22020,13 +22070,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -22036,13 +22086,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -22052,13 +22102,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -22068,13 +22118,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>

</xml_diff>

<commit_message>
beta v0.9.16: wall-blocked brush and compass, minigame thumbnails, first-launch tutorial
- Compass collides with walls and pillars (still passes crates and barrels); a returning compass hitting a wall is caught
- Brush swing and its ink stroke stop at walls
- Training minigame chooser shows animated thumbnails
- First launch goes straight into the tutorial stage
- Maze hides wall footprints until the game starts
- Ink Rain speeds up over time and clears the field when it ends
- Tutorial: done stamp no longer overlaps progress pips; remove stray control box in deck illustration
- Reduced motion keeps ult cut-in background motifs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -14950,7 +14950,47 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.35
+      <t xml:space="preserve">0.55
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">後段預警縮短：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.45
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">後段雙滴增加：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3
 </t>
     </r>
     <r>
@@ -21641,7 +21681,7 @@
       </c>
       <c r="F9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="189.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>406</v>
       </c>

</xml_diff>

<commit_message>
beta v0.9.17: English language option, random bosses, new enemies and bosses, endless acts
- Language dropdown in settings (繁體中文 / English) with a full English
  translation; first launch asks for the language before the tutorial
- Endless mode: 5 pages per act, card rewards on pages 1, 3 and 5
- New enemies: rubber stamper and scissor minions (with elites)
- New bosses: exam overlord and the final ink-stained tome; bosses are
  drawn at random and scale tempo, HP and minion summons by stage
- Scissors dash trail bullets linger, then fire perpendicular to the dash
- Brush refunds only after two swings with zero damage
- No resume countdown outside combat and timed minigames
- At most 3 normal enemy types per page, rotating between pages

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="485">
   <si>
     <r>
       <rPr>
@@ -8766,6 +8766,410 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">stampSoldier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">橡皮印章兵</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【跳躍蓋章】預判你的位置跳過去，落點先畫出紅圈；落地時圈內受到傷害並留下減速墨印，之後會硬直一下。
+【連續蓋章（精英）】精英會連跳兩次、硬直更短，每次落地都向四周彈出一圈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">發子彈。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">range</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[4, 8]
+strafe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
+stampEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[2.6, 3.6]
+firstStamp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1.6, 2.4]
+crouch</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3
+jumpTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.85
+jumpRange</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6.5
+jumpHeight</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.4
+lead</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35
+stampRadius</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.8
+stampDamage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+landStun</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.75
+eliteLandStun</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35
+eliteHops</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+eliteRing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8
+bulletLife</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.2
+puddleRadius</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.5
+puddleTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.5
+puddleSlow</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+knockMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">inkCloud</t>
   </si>
   <si>
@@ -9290,6 +9694,302 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">scissorMinion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">剪刀小兵</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【左右夾擊】一隻準備衝刺時，附近的同伴也會一起畫紅線，從兩側同時剪過來。精英衝刺結束後會再朝你射出 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">發子彈。
+【暴走】同伴被打倒時，剩下的剪刀小兵會變紅暴走：移動、出招與衝刺都更快。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">range</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[4.5, 7]
+strafe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.9
+snipEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[2.6, 3.6]
+firstSnip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1.4, 2.2]
+telegraph</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.7
+telegraphLength</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9
+dashSpeed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15
+dashTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.42
+recover</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.45
+pairRange</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14
+rage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'speed': 1.4, 'tele': 0.7, 'every': 0.6, 'dash': 1.15}
+eliteShots</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+eliteSpread</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.45
+bulletLife</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
     </r>
   </si>
   <si>
@@ -10220,7 +10920,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【衝刺剪擊】預判你的位置畫出紅線後高速衝刺，沿路留下紅色切痕。撞牆會卡住，此時受到 </t>
+      <t xml:space="preserve">【衝刺剪擊】預判你的位置畫出紅線後高速衝刺，沿路留下一排子彈；子彈停留一下後會朝衝刺路線的左右兩側射出。撞牆會卡住，此時受到 </t>
     </r>
     <r>
       <rPr>
@@ -10340,6 +11040,24 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.5
+trail</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'every': 0.09, 'linger': 1.3, 'stagger': 0.02, 'speed': 6.5, 'life': 3}
 bulletLife</t>
     </r>
     <r>
@@ -10531,6 +11249,439 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">exam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">考卷魔王</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【選擇題】在你腳下和周圍畫出紅圈，一段時間後依序引爆並向外炸出子彈。
+【安靜作答】這段時間只要你開火，它就會喊「作弊！」並朝你射出一排子彈。
+【紅筆批改】畫出好幾條紅線，接著沿著紅線連續射出子彈。
+【答對了】每道題目結束時如果你沒被打中，它會攤開休息，這時受到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍傷害；被打中就沒有休息。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">knockMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0
+weakMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+keep</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8
+questionGap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1.1, 1.6]
+askTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.1
+restTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.3
+wrongTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.7
+zone</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'count': 4, 'count2': 6, 'r': 1.9, 'spread': 5.5, 'delay': 1.1, 'stagger': 0.18, 'ring': 8, 'speed': 4.5, 'life': 2.4}
+quiet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'time': 2.8, 'cool': 0.35, 'shots': 3, 'shots2': 5, 'spread': 0.5}
+grade</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'lines': 4, 'lines2': 6, 'spread': 2.4, 'tele': 0.8, 'time': 1.3, 'every': 0.07}
+toss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'volleys': 3, 'volleys2': 4, 'count': 5, 'spread': 0.9, 'every': 0.5, 'speed': 6}
+bulletLife</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">bookFinal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">墨跡之書・終章</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【翻頁】連續翻頁震出好幾圈子彈，章節越後面圈數越多。
+【仿寫】模仿你的技能：在你身邊標記紅圈後引爆（爆墨），或連射扇形子彈（散射）。
+【攤開休息】每次攻擊後攤開休息，受到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍傷害。也會使用墨跡之書的彈幕牆、墨水雨、重擊與召喚。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">knockMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0
+weakMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+restTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.5
+flip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'rings': 3, 'count': 20, 'every': 0.4, 'speeds': [5, 7.5]}
+mimicScatter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'volleys': 3, 'count': 7, 'spread': 0.9, 'every': 0.45, 'speed': 8}
+mimicBomb</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'count': 4, 'count2': 6, 'r': 1.8, 'delay': 0.9, 'stagger': 0.15, 'ring': 10, 'speed': 5, 'life': 2.4}
+bulletLife</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">特色</t>
   </si>
   <si>
@@ -10728,7 +11879,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">低傷返還：連續 </t>
+      <t xml:space="preserve">落空返還：連續 </t>
     </r>
     <r>
       <rPr>
@@ -10745,24 +11896,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">次揮筆造成的傷害都 ≤ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">時返還 </t>
+      <t xml:space="preserve">次揮筆都沒有造成任何傷害時返還 </t>
     </r>
     <r>
       <rPr>
@@ -20552,7 +21686,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -20781,7 +21915,7 @@
       </c>
       <c r="P6" s="10"/>
     </row>
-    <row r="7" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="270.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>297</v>
       </c>
@@ -20789,23 +21923,27 @@
         <v>298</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>299</v>
+        <v>284</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="E7" s="7" t="n">
         <f aca="false">ROUND(D7*$B$1,0)</f>
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
+        <v>1</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>6</v>
+      </c>
       <c r="J7" s="8"/>
       <c r="K7" s="8" t="n">
         <v>1.5</v>
@@ -20818,48 +21956,48 @@
         <v>2</v>
       </c>
       <c r="N7" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>300</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>301</v>
       </c>
       <c r="P7" s="10"/>
     </row>
-    <row r="8" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>303</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>299</v>
-      </c>
       <c r="D8" s="8" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="E8" s="7" t="n">
         <f aca="false">ROUND(D8*$B$1,0)</f>
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>6.5</v>
+        <v>2.6</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
       <c r="K8" s="8" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">K8*$D$1</f>
+        <v>3</v>
+      </c>
+      <c r="M8" s="8" t="n">
         <v>2</v>
-      </c>
-      <c r="M8" s="8" t="n">
-        <v>1</v>
       </c>
       <c r="N8" s="7" t="s">
         <v>304</v>
@@ -20869,7 +22007,7 @@
       </c>
       <c r="P8" s="10"/>
     </row>
-    <row r="9" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>306</v>
       </c>
@@ -20877,240 +22015,244 @@
         <v>307</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="E9" s="7" t="n">
         <f aca="false">ROUND(D9*$B$1,0)</f>
-        <v>145</v>
+        <v>65</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>2.2</v>
+        <v>6.5</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8" t="n">
         <v>1</v>
-      </c>
-      <c r="I9" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>308</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>1.5</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">K9*$D$1</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N9" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="O9" s="6" t="s">
         <v>309</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>310</v>
       </c>
       <c r="P9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="202.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>311</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>312</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>284</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">ROUND(D10*$B$1,0)</f>
-        <v>225</v>
+        <v>75</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
+      <c r="H10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>9</v>
+      </c>
       <c r="J10" s="8"/>
       <c r="K10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">K10*$D$1</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="N10" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="O10" s="6" t="s">
         <v>313</v>
-      </c>
-      <c r="O10" s="6" t="s">
-        <v>314</v>
       </c>
       <c r="P10" s="10"/>
     </row>
-    <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>315</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>289</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>316</v>
+        <v>284</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">ROUND(D11*$B$1,0)</f>
-        <v>35</v>
+        <v>145</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>4.2</v>
+        <v>2.2</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="H11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>316</v>
+      </c>
       <c r="K11" s="8" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">K11*$D$1</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N11" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="N11" s="7" t="s">
+        <v>317</v>
+      </c>
       <c r="O11" s="6" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="P11" s="10"/>
     </row>
-    <row r="12" customFormat="false" ht="176.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>318</v>
-      </c>
-      <c r="B12" s="12" t="s">
+    <row r="12" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="B12" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="D12" s="13" t="n">
-        <v>900</v>
-      </c>
-      <c r="E12" s="12" t="s">
+      <c r="C12" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <f aca="false">ROUND(D12*$B$1,0)</f>
+        <v>225</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <f aca="false">K12*$D$1</f>
+        <v>4</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" s="7" t="s">
         <v>321</v>
       </c>
-      <c r="F12" s="13" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G12" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" s="11" t="s">
+      <c r="O12" s="6" t="s">
         <v>322</v>
-      </c>
-      <c r="M12" s="13"/>
-      <c r="N12" s="12" t="s">
-        <v>323</v>
-      </c>
-      <c r="O12" s="11" t="s">
-        <v>324</v>
       </c>
       <c r="P12" s="10"/>
     </row>
-    <row r="13" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <f aca="false">ROUND(D13*$B$1,0)</f>
+        <v>35</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <f aca="false">K13*$D$1</f>
+        <v>1</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="7"/>
+      <c r="O13" s="6" t="s">
         <v>325</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>326</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>320</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>321</v>
-      </c>
-      <c r="F13" s="13" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>322</v>
-      </c>
-      <c r="M13" s="13"/>
-      <c r="N13" s="12" t="s">
-        <v>327</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>328</v>
       </c>
       <c r="P13" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="176.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>900</v>
+      </c>
+      <c r="E14" s="12" t="s">
         <v>329</v>
       </c>
-      <c r="B14" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>320</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>1300</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>321</v>
-      </c>
       <c r="F14" s="13" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G14" s="13" t="n">
         <v>1</v>
@@ -21119,14 +22261,14 @@
         <v>1</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="J14" s="13"/>
       <c r="K14" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="12" t="s">
@@ -21136,6 +22278,182 @@
         <v>332</v>
       </c>
       <c r="P14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="108.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="M15" s="13"/>
+      <c r="N15" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="O15" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="P15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="M16" s="13"/>
+      <c r="N16" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="O16" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="P16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="226.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>341</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>342</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="M17" s="13"/>
+      <c r="N17" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="O17" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="P17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="133.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>328</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="M18" s="13"/>
+      <c r="N18" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="O18" s="11" t="s">
+        <v>348</v>
+      </c>
+      <c r="P18" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -21183,37 +22501,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>333</v>
+        <v>349</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>335</v>
+        <v>351</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>276</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>336</v>
+        <v>352</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>337</v>
+        <v>353</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>275</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -21221,16 +22539,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -21265,16 +22583,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -21309,16 +22627,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>348</v>
+        <v>364</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>350</v>
+        <v>366</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -21349,22 +22667,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>351</v>
+        <v>367</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -21395,22 +22713,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>356</v>
+        <v>372</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -21428,10 +22746,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -21441,22 +22759,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -21468,10 +22786,10 @@
         <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -21487,7 +22805,7 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>362</v>
+        <v>378</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -21519,19 +22837,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>363</v>
+        <v>379</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -21539,289 +22857,289 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>367</v>
+        <v>383</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>369</v>
+        <v>385</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>370</v>
+        <v>386</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>373</v>
+        <v>389</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>374</v>
+        <v>390</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>376</v>
+        <v>392</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>377</v>
+        <v>393</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>378</v>
+        <v>394</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>379</v>
+        <v>395</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>380</v>
+        <v>396</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>381</v>
+        <v>397</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>382</v>
+        <v>398</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>384</v>
+        <v>400</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>385</v>
+        <v>401</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>391</v>
+        <v>407</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>400</v>
+        <v>416</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>401</v>
+        <v>417</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>403</v>
+        <v>419</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>404</v>
+        <v>420</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>405</v>
+        <v>421</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>406</v>
+        <v>422</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>407</v>
+        <v>423</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>408</v>
+        <v>424</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>409</v>
+        <v>425</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>410</v>
+        <v>426</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>411</v>
+        <v>427</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>432</v>
+        <v>448</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>440</v>
+        <v>456</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>441</v>
+        <v>457</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>443</v>
+        <v>459</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>444</v>
+        <v>460</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -21856,13 +23174,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>445</v>
+        <v>461</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>446</v>
+        <v>462</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>447</v>
+        <v>463</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -21870,13 +23188,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>449</v>
+        <v>465</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -21886,13 +23204,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -21902,13 +23220,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>451</v>
+        <v>467</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -21918,13 +23236,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>452</v>
+        <v>468</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -21934,13 +23252,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>453</v>
+        <v>469</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -21950,13 +23268,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>454</v>
+        <v>470</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -21966,13 +23284,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>455</v>
+        <v>471</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -21982,13 +23300,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>456</v>
+        <v>472</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -21998,13 +23316,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>457</v>
+        <v>473</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -22014,13 +23332,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>458</v>
+        <v>474</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -22030,13 +23348,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>459</v>
+        <v>475</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -22046,13 +23364,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -22062,13 +23380,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>462</v>
+        <v>478</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -22078,13 +23396,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>463</v>
+        <v>479</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -22094,13 +23412,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>464</v>
+        <v>480</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -22110,13 +23428,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>465</v>
+        <v>481</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -22126,13 +23444,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>466</v>
+        <v>482</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -22142,13 +23460,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>467</v>
+        <v>483</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -22158,13 +23476,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>460</v>
+        <v>476</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>468</v>
+        <v>484</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>

</xml_diff>

<commit_message>
beta v0.9.18: training boss dropdown, final tome rework, scissor minion pincer, stamp prints
- Training: boss picker is a dropdown (None first, one boss at a time),
  enemy/boss config resets to defaults on entry, boss HP bar in training
- Final tome: fewer bullets, new ruled-line, page-sweep and bookmark-seal
  mechanics (immune until bookmarks break, then knocked down)
- Scissor minions: paired thread pincer; lone minions throw a returning blade
- Stamp soldier prints match the landing circle, last ~12s, halve speed
- No touch-switch toast on the first touch; animated language dropdown

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="488">
   <si>
     <r>
       <rPr>
@@ -8778,7 +8778,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【跳躍蓋章】預判你的位置跳過去，落點先畫出紅圈；落地時圈內受到傷害並留下減速墨印，之後會硬直一下。
+      <t xml:space="preserve">【跳躍蓋章】預判你的位置跳過去，落點先畫出紅圈；落地時圈內受到傷害，並留下和紅圈一樣大的墨印（踩到會減速一半），之後會硬直一下。墨印大約到它再跳兩次時才開始慢慢變淡。
 【連續蓋章（精英）】精英會連跳兩次、硬直更短，每次落地都向四周彈出一圈 </t>
     </r>
     <r>
@@ -9095,7 +9095,7 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.2
-puddleRadius</t>
+puddleTime</t>
     </r>
     <r>
       <rPr>
@@ -9112,8 +9112,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.5
-puddleTime</t>
+      <t xml:space="preserve">12
+puddleFade</t>
     </r>
     <r>
       <rPr>
@@ -9130,7 +9130,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3.5
+      <t xml:space="preserve">3
 puddleSlow</t>
     </r>
     <r>
@@ -9148,7 +9148,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.6
+      <t xml:space="preserve">0.5
 knockMult</t>
     </r>
     <r>
@@ -9703,32 +9703,8 @@
     <t xml:space="preserve">剪刀小兵</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">【左右夾擊】一隻準備衝刺時，附近的同伴也會一起畫紅線，從兩側同時剪過來。精英衝刺結束後會再朝你射出 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">發子彈。
-【暴走】同伴被打倒時，剩下的剪刀小兵會變紅暴走：移動、出招與衝刺都更快。</t>
-    </r>
+    <t xml:space="preserve">【剪合】兩隻剪刀小兵繞到你的兩側，在彼此之間拉起紅線，接著同時往中間衝刺剪合——站在線上就會被剪到，往旁邊走開就安全。精英剪合時會在交會點噴出一圈子彈。
+【飛刃（落單）】同伴被打倒（或本來就落單）時會變紅暴走，改為朝你丟出半片刀刃：沿紅線飛出，到底後原路飛回。精英一次丟兩片。</t>
   </si>
   <si>
     <r>
@@ -9773,8 +9749,152 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">0.8
+snipEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[3, 4.2]
+firstSnip</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1.8, 2.8]
+pairRange</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16
+flank</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.6
+orbit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+readyDist</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.4
+readyWait</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.5
+threadTele</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">0.9
-snipEvery</t>
+threadWidth</t>
     </r>
     <r>
       <rPr>
@@ -9791,8 +9911,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[2.6, 3.6]
-firstSnip</t>
+      <t xml:space="preserve">0.35
+snipDamage</t>
     </r>
     <r>
       <rPr>
@@ -9809,8 +9929,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[1.4, 2.2]
-telegraph</t>
+      <t xml:space="preserve">1
+dashSpeed</t>
     </r>
     <r>
       <rPr>
@@ -9827,8 +9947,44 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">13
+dashTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+recover</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">0.7
-telegraphLength</t>
+throwRange</t>
     </r>
     <r>
       <rPr>
@@ -9845,8 +10001,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">9
-dashSpeed</t>
+      <t xml:space="preserve">7.5
+throwTele</t>
     </r>
     <r>
       <rPr>
@@ -9863,8 +10019,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">15
-dashTime</t>
+      <t xml:space="preserve">0.65
+throwSpeed</t>
     </r>
     <r>
       <rPr>
@@ -9881,8 +10037,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.42
-recover</t>
+      <t xml:space="preserve">11
+bladeDots</t>
     </r>
     <r>
       <rPr>
@@ -9899,8 +10055,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.45
-pairRange</t>
+      <t xml:space="preserve">3
+bladeGap</t>
     </r>
     <r>
       <rPr>
@@ -9917,7 +10073,43 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">14
+      <t xml:space="preserve">0.32
+eliteThrowSpread</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+eliteRing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8
 rage</t>
     </r>
     <r>
@@ -9935,43 +10127,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'speed': 1.4, 'tele': 0.7, 'every': 0.6, 'dash': 1.15}
-eliteShots</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3
-eliteSpread</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.45
+      <t xml:space="preserve">{'speed': 1.35, 'tele': 0.7, 'every': 0.6, 'dash': 1.2}
 bulletLife</t>
     </r>
     <r>
@@ -11523,8 +11679,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【翻頁】連續翻頁震出好幾圈子彈，章節越後面圈數越多。
-【仿寫】模仿你的技能：在你身邊標記紅圈後引爆（爆墨），或連射扇形子彈（散射）。
+      <t xml:space="preserve">【畫線】在場上拉出幾條橫豎紅線（一定有一條穿過你），紅線畫完後變成粗墨線，站在上面就會受傷。章節越後面線越多。
+【仿寫】模仿你的技能：在你身邊標記紅圈後引爆（爆墨，終章才會噴子彈），或射出少量扇形子彈（散射）。
 【攤開休息】每次攻擊後攤開休息，受到 </t>
     </r>
     <r>
@@ -11542,7 +11698,77 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍傷害。也會使用墨跡之書的彈幕牆、墨水雨、重擊與召喚。</t>
+      <t xml:space="preserve">倍傷害。第二章起也會使用有缺口的彈幕牆。
+【書籤封印】每翻到新章節就闔上書、刀槍不入，並在四周插上 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">根書籤（紅線連到書）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內打斷所有書籤，它會倒下休息 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒並受到三倍傷害；來不及就會回復一些血量。
+【翻頁橫掃】一大頁紙從書旁掃過半個場地，起點和終點都會先畫出紅線。貼近書本（掃不到的內圈）或衝刺穿過都能躲開。</t>
     </r>
   </si>
   <si>
@@ -11606,8 +11832,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.5
-flip</t>
+      <t xml:space="preserve">1.6
+lines</t>
     </r>
     <r>
       <rPr>
@@ -11624,7 +11850,43 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'rings': 3, 'count': 20, 'every': 0.4, 'speeds': [5, 7.5]}
+      <t xml:space="preserve">{'count': [2, 3, 4], 'warn': 1.1, 'live': 0.5, 'fade': 0.35, 'width': 0.55, 'stagger': 0.25, 'spread': 5}
+sweep</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'arc': 2.6, 'inner': 3.4, 'outer': 17, 'width': 0.5, 'warn': 1, 'dur': 1.9, 'fade': 0.3}
+seal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'marks': [3, 4], 'radius': 7.5, 'time': 14, 'heal': 0.06, 'stun': 4, 'attackEvery': 3.2, 'lines': 2}
 mimicScatter</t>
     </r>
     <r>
@@ -11642,7 +11904,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'volleys': 3, 'count': 7, 'spread': 0.9, 'every': 0.45, 'speed': 8}
+      <t xml:space="preserve">{'volleys': 2, 'count': 5, 'spread': 0.8, 'every': 0.5, 'speed': 8}
 mimicBomb</t>
     </r>
     <r>
@@ -11660,7 +11922,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'count': 4, 'count2': 6, 'r': 1.8, 'delay': 0.9, 'stagger': 0.15, 'ring': 10, 'speed': 5, 'life': 2.4}
+      <t xml:space="preserve">{'count': [3, 4, 5], 'r': 1.8, 'delay': 1, 'stagger': 0.2, 'ring': 6, 'speed': 4.5, 'life': 2.2}
 bulletLife</t>
     </r>
     <r>
@@ -11679,6 +11941,40 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">bookmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">書籤</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">knockMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
     </r>
   </si>
   <si>
@@ -21686,7 +21982,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -22051,7 +22347,7 @@
       </c>
       <c r="P9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="202.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="336.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>310</v>
       </c>
@@ -22411,7 +22707,7 @@
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="133.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="185.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>345</v>
       </c>
@@ -22454,6 +22750,48 @@
         <v>348</v>
       </c>
       <c r="P18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <f aca="false">ROUND(D19*$B$1,0)</f>
+        <v>113</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <f aca="false">K19*$D$1</f>
+        <v>1</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="7"/>
+      <c r="O19" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="P19" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -22501,37 +22839,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>276</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>275</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -22539,16 +22877,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -22583,16 +22921,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -22627,16 +22965,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -22667,22 +23005,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -22713,22 +23051,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -22759,7 +23097,7 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="O6" s="10"/>
     </row>
@@ -22768,13 +23106,13 @@
         <v>314</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -22805,7 +23143,7 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -22837,19 +23175,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -22857,289 +23195,289 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -23174,13 +23512,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -23188,13 +23526,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -23204,13 +23542,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -23220,13 +23558,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -23236,13 +23574,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -23252,13 +23590,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -23268,13 +23606,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -23284,13 +23622,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -23300,13 +23638,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -23316,13 +23654,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -23332,13 +23670,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -23348,13 +23686,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -23364,13 +23702,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -23380,13 +23718,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -23396,13 +23734,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -23412,13 +23750,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -23428,13 +23766,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -23444,13 +23782,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -23460,13 +23798,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -23476,13 +23814,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>

</xml_diff>

<commit_message>
beta v0.9.19: boss evolution forms, Quill Tyrant, exam questions, cut-along-the-line scissor imps
- Bosses lock HP at a threshold, play an evolution animation and enter a
  second form with new moves: ink bottle rolling charge, scissors circling
  snips, book pouncing press, exam essay/trick questions, quill writing dash
- Weak-point bonus is now x2 for all bosses except the Quill Tyrant (x3)
- Exam: red-pen rate matches the codex demo; new true/false and
  fill-in-the-blank questions
- Final boss renamed to Quill Tyrant with a new pen model, 1400 HP, a
  single cartridge seal, and joins the regular 5-boss random pool
- Scissor imps rebuilt: they cut along a dotted box around you, pairs split
  the cut, and interrupting the cutter cancels it
- Slow and field zones show a countdown ring on their inner edge
- Training bosses spawn at the arena center

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -9703,8 +9703,8 @@
     <t xml:space="preserve">剪刀小兵</t>
   </si>
   <si>
-    <t xml:space="preserve">【剪合】兩隻剪刀小兵繞到你的兩側，在彼此之間拉起紅線，接著同時往中間衝刺剪合——站在線上就會被剪到，往旁邊走開就安全。精英剪合時會在交會點噴出一圈子彈。
-【飛刃（落單）】同伴被打倒（或本來就落單）時會變紅暴走，改為朝你丟出半片刀刃：沿紅線飛出，到底後原路飛回。精英一次丟兩片。</t>
+    <t xml:space="preserve">【分頭剪】附近有另一隻剪刀小兵時，兩隻會從對角分頭剪，一人剪半圈，框收得更快。同伴被打倒時剩下的會暴走變紅、剪得更快。精英的框更大，剪完時四個角會朝內射出子彈。
+【沿虛線剪下】在你周圍畫出紅色虛線方框，跑到角落後沿著虛線一路剪過去（剪過的地方變成實線）；整圈剪完時框內的紙片會被剪掉，還站在裡面就會受傷。打倒或擊暈正在剪的小兵可以中斷。</t>
   </si>
   <si>
     <r>
@@ -9731,7 +9731,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[4.5, 7]
+      <t xml:space="preserve">[4.5, 7.5]
 strafe</t>
     </r>
     <r>
@@ -9767,7 +9767,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[3, 4.2]
+      <t xml:space="preserve">[3.4, 4.6]
 firstSnip</t>
     </r>
     <r>
@@ -9785,7 +9785,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[1.8, 2.8]
+      <t xml:space="preserve">[1.6, 2.6]
 pairRange</t>
     </r>
     <r>
@@ -9804,7 +9804,7 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">16
-flank</t>
+rect</t>
     </r>
     <r>
       <rPr>
@@ -9821,8 +9821,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4.6
-orbit</t>
+      <t xml:space="preserve">[2.6, 2]
+eliteRect</t>
     </r>
     <r>
       <rPr>
@@ -9839,8 +9839,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.5
-readyDist</t>
+      <t xml:space="preserve">[3.4, 2.6]
+runSpeed</t>
     </r>
     <r>
       <rPr>
@@ -9857,8 +9857,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.4
-readyWait</t>
+      <t xml:space="preserve">10
+markMin</t>
     </r>
     <r>
       <rPr>
@@ -9875,8 +9875,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.5
-threadTele</t>
+      <t xml:space="preserve">0.55
+markMax</t>
     </r>
     <r>
       <rPr>
@@ -9893,8 +9893,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.9
-threadWidth</t>
+      <t xml:space="preserve">1.6
+cutSpeed</t>
     </r>
     <r>
       <rPr>
@@ -9911,8 +9911,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.35
-snipDamage</t>
+      <t xml:space="preserve">7
+cutDamage</t>
     </r>
     <r>
       <rPr>
@@ -9930,7 +9930,7 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1
-dashSpeed</t>
+dash</t>
     </r>
     <r>
       <rPr>
@@ -9947,8 +9947,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">13
-dashTime</t>
+      <t xml:space="preserve">0.7
+pieceTime</t>
     </r>
     <r>
       <rPr>
@@ -9983,8 +9983,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.7
-throwRange</t>
+      <t xml:space="preserve">0.6
+eliteSpread</t>
     </r>
     <r>
       <rPr>
@@ -10001,8 +10001,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">7.5
-throwTele</t>
+      <t xml:space="preserve">0.3
+rage</t>
     </r>
     <r>
       <rPr>
@@ -10019,115 +10019,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.65
-throwSpeed</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">11
-bladeDots</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3
-bladeGap</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.32
-eliteThrowSpread</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.5
-eliteRing</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8
-rage</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{'speed': 1.35, 'tele': 0.7, 'every': 0.6, 'dash': 1.2}
+      <t xml:space="preserve">{'speed': 1.4, 'every': 0.6}
 bulletLife</t>
     </r>
     <r>
@@ -10658,7 +10550,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【螺旋彈幕】原地旋轉，從瓶身噴出 </t>
+      <t xml:space="preserve">【翻滾衝撞（第二型態）】血量剩一半時鎖血進化。進化後會倒下沿紅線翻滾衝撞兩次，沿路灑下會倒數消失的減速墨漬，滾完會暈一下。
+【螺旋彈幕】原地旋轉，從瓶身噴出 </t>
     </r>
     <r>
       <rPr>
@@ -10808,7 +10701,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3 </t>
+      <t xml:space="preserve">2 </t>
     </r>
     <r>
       <rPr>
@@ -10880,7 +10773,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3
+      <t xml:space="preserve">2
 spinSpeed</t>
     </r>
     <r>
@@ -11060,7 +10953,43 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.48</t>
+      <t xml:space="preserve">0.48
+evolve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'at': 0.5, 'time': 2.4}
+roll</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'tele': 0.85, 'tele2': 0.5, 'speed': 11, 'time': 1.5, 'drop': 0.22, 'dropR': 1.2, 'dropTime': 4, 'count': 2, 'dizzy': 1.1, 'damage': 1}</t>
     </r>
   </si>
   <si>
@@ -11076,7 +11005,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【衝刺剪擊】預判你的位置畫出紅線後高速衝刺，沿路留下一排子彈；子彈停留一下後會朝衝刺路線的左右兩側射出。撞牆會卡住，此時受到 </t>
+      <t xml:space="preserve">【繞圈剪擊（第二型態）】血量剩一半時鎖血進化。進化後會繞著你高速轉圈，每隔一下朝你射出 </t>
     </r>
     <r>
       <rPr>
@@ -11086,6 +11015,24 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">發子彈；衝刺也會連衝三次。
+【衝刺剪擊】預判你的位置畫出紅線後高速衝刺，沿路留下一排子彈；子彈停留一下後會朝衝刺路線的左右兩側射出。撞牆會卡住，此時受到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
     </r>
     <r>
       <rPr>
@@ -11141,7 +11088,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3
+      <t xml:space="preserve">2
 dashSpeed</t>
     </r>
     <r>
@@ -11196,6 +11143,42 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.5
+evolve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'at': 0.5, 'time': 2.2}
+orbit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'tele': 0.6, 'r': 5.5, 'turn': 1.5, 'speed': 13, 'time': 3, 'every': 0.5, 'count': 3, 'spread': 0.35}
 trail</t>
     </r>
     <r>
@@ -11247,7 +11230,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【彈幕牆】射出一整排子彈牆，只留下一個缺口，找到缺口鑽過去。
+      <t xml:space="preserve">【飛撲重壓（第二型態）】血量剩一半時鎖血進化。進化後會飛起來撲向紅圈標記的位置連壓兩次，落地時圈內受傷並震出一圈子彈，壓完會攤開休息。
+【彈幕牆】射出一整排子彈牆，只留下一個缺口，找到缺口鑽過去。
 【墨水雨】在地上標記紅圈，稍後墨水落下並向四周炸出子彈，快離開紅圈。
 【重擊】把書重重闔上，震出 </t>
     </r>
@@ -11311,7 +11295,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3 </t>
+      <t xml:space="preserve">2 </t>
     </r>
     <r>
       <rPr>
@@ -11365,7 +11349,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3
+      <t xml:space="preserve">2
 restTime</t>
     </r>
     <r>
@@ -11384,6 +11368,42 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.8
+evolve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'at': 0.5, 'time': 2.4}
+glide</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'tele': 0.9, 'time': 0.75, 'height': 3, 'r': 3, 'ring': 12, 'speed': 5, 'hops': 2}
 bulletLife</t>
     </r>
     <r>
@@ -11429,15 +11449,52 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">倍傷害；被打中就沒有休息。</t>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍傷害；被打中就沒有休息。
+【申論題（第二型態）】進化後才會出的題目：考卷一邊追著你一邊寫字，留下的筆跡過一下會變成粗墨線，碰到就受傷。
+【填空題】在你周圍畫出 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3×3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">的格子，只有畫 ○ 的格子是正確答案；其他格子會一格一格被墨水填滿，站在裡面就會受傷。進化後只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">格安全。
+【是非題】用紅線把場地切成兩半，一半畫上 ✗、一半畫上 ○；時間到時 ✗ 那半邊整片被劃掉，站在那邊就會受傷。進化後有一半機率在中途換邊（陷阱題）。</t>
     </r>
   </si>
   <si>
@@ -11483,7 +11540,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3
+      <t xml:space="preserve">2
 keep</t>
     </r>
     <r>
@@ -11627,7 +11684,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'lines': 4, 'lines2': 6, 'spread': 2.4, 'tele': 0.8, 'time': 1.3, 'every': 0.07}
+      <t xml:space="preserve">{'lines': 4, 'lines2': 5, 'spread': 2.4, 'tele': 0.8, 'time': 1.2, 'every': 0.16}
 toss</t>
     </r>
     <r>
@@ -11646,6 +11703,78 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">{'volleys': 3, 'volleys2': 4, 'count': 5, 'spread': 0.9, 'every': 0.5, 'speed': 6}
+evolve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'at': 0.5, 'time': 2.4}
+tf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'ask': 1.9, 'ask2': 2.3, 'swapAt': 0.55, 'swapChance': 0.5, 'live': 0.55, 'hatch': 6}
+blank</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'cell': 2.6, 'safe': 2, 'safe2': 1, 'every': 0.2, 'fill': 0.7}
+essay</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'time': 3.4, 'speed': 4.4, 'drop': 0.2, 'arm': 0.5, 'live': 2.6, 'width': 0.45}
 bulletLife</t>
     </r>
     <r>
@@ -11670,18 +11799,18 @@
     <t xml:space="preserve">bookFinal</t>
   </si>
   <si>
-    <t xml:space="preserve">墨跡之書・終章</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">【畫線】在場上拉出幾條橫豎紅線（一定有一條穿過你），紅線畫完後變成粗墨線，站在上面就會受傷。章節越後面線越多。
-【仿寫】模仿你的技能：在你身邊標記紅圈後引爆（爆墨，終章才會噴子彈），或射出少量扇形子彈（散射）。
-【攤開休息】每次攻擊後攤開休息，受到 </t>
+    <t xml:space="preserve">巨筆暴君</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【畫線】在場上拉出幾條橫豎紅線（一定有一條穿過你），紅線畫完後變成粗墨線，站在上面就會受傷。越後期線越多。
+【仿寫】模仿你的技能：在你身邊標記紅圈後引爆（爆墨，進化後才會噴子彈），或射出少量扇形子彈（散射）。
+【喘息】每次攻擊後筆尖插地喘息，受到 </t>
     </r>
     <r>
       <rPr>
@@ -11698,25 +11827,77 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍傷害。第二章起也會使用有缺口的彈幕牆。
-【書籤封印】每翻到新章節就闔上書、刀槍不入，並在四周插上 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">～</t>
+      <t xml:space="preserve">倍傷害。也會使用有缺口的彈幕牆。
+【書寫衝刺（第二型態）】血量剩三分之一時鎖血進化。進化後會沿紅線高速衝刺 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次，經過的路線留下約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒的粗墨線，碰到就受傷。
+【墨水管封印】血量剩三分之二時刀槍不入，並在四周插上 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">根墨水管（紅線連到本體）。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內打斷所有墨水管，它會倒下 </t>
     </r>
     <r>
       <rPr>
@@ -11733,42 +11914,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">根書籤（紅線連到書）。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">14 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內打斷所有書籤，它會倒下休息 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">秒並受到三倍傷害；來不及就會回復一些血量。
-【翻頁橫掃】一大頁紙從書旁掃過半個場地，起點和終點都會先畫出紅線。貼近書本（掃不到的內圈）或衝刺穿過都能躲開。</t>
+【筆桿橫掃】倒下筆桿掃過半個場地，起點和終點都會先畫出紅線。貼近筆尖（掃不到的內圈）或衝刺穿過都能躲開。</t>
     </r>
   </si>
   <si>
@@ -11886,7 +12033,43 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'marks': [3, 4], 'radius': 7.5, 'time': 14, 'heal': 0.06, 'stun': 4, 'attackEvery': 3.2, 'lines': 2}
+      <t xml:space="preserve">{'marks': [3], 'radius': 7.5, 'time': 14, 'heal': 0.06, 'stun': 4, 'attackEvery': 3.2, 'lines': 2}
+evolve</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'at': 0.34, 'time': 2.6}
+scribble</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'count': 3, 'tele': 0.7, 'tele2': 0.45, 'speed': 15, 'time': 0.85, 'live': 2.2}
 mimicScatter</t>
     </r>
     <r>
@@ -11947,7 +12130,7 @@
     <t xml:space="preserve">bookmark</t>
   </si>
   <si>
-    <t xml:space="preserve">書籤</t>
+    <t xml:space="preserve">墨水管</t>
   </si>
   <si>
     <r>
@@ -22347,7 +22530,7 @@
       </c>
       <c r="P9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="336.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>310</v>
       </c>
@@ -22531,7 +22714,7 @@
       </c>
       <c r="P13" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="176.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>326</v>
       </c>
@@ -22575,7 +22758,7 @@
       </c>
       <c r="P14" s="10"/>
     </row>
-    <row r="15" customFormat="false" ht="108.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="147.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
         <v>333</v>
       </c>
@@ -22619,7 +22802,7 @@
       </c>
       <c r="P15" s="10"/>
     </row>
-    <row r="16" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>337</v>
       </c>
@@ -22663,7 +22846,7 @@
       </c>
       <c r="P16" s="10"/>
     </row>
-    <row r="17" customFormat="false" ht="226.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="317.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
         <v>341</v>
       </c>
@@ -22707,7 +22890,7 @@
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="185.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>345</v>
       </c>
@@ -22718,7 +22901,7 @@
         <v>328</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1700</v>
+        <v>1400</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>329</v>

</xml_diff>

<commit_message>
beta v0.9.20: quill tyrant redesign and cartridge guard, exam tweaks, detail-based quality levels
- Remove scissor imps from levels, endless, training and codex for now
- Quill Tyrant: shorter, lighter, more detailed model; thrown ink
  cartridges halve damage taken while it keeps attacking; the x3 rest
  window only comes after every third attack
- Exam: grading and paper balls no longer count as questions; true/false
  deals 2 damage; fill-in-the-blank grid covers the whole arena
- Countdown rings only on the trap circle and stamp prints
- Training keeps map and toggles for the session, resets enemies per entry
- Codex list drops the "tap to view" hint line
- Graphics quality no longer lowers resolution; low/mid cut edge samples,
  wobble, grain, outlines, shadows, particles and decals; UI stays crisp

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="484">
   <si>
     <r>
       <rPr>
@@ -9694,350 +9694,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">scissorMinion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">剪刀小兵</t>
-  </si>
-  <si>
-    <t xml:space="preserve">【分頭剪】附近有另一隻剪刀小兵時，兩隻會從對角分頭剪，一人剪半圈，框收得更快。同伴被打倒時剩下的會暴走變紅、剪得更快。精英的框更大，剪完時四個角會朝內射出子彈。
-【沿虛線剪下】在你周圍畫出紅色虛線方框，跑到角落後沿著虛線一路剪過去（剪過的地方變成實線）；整圈剪完時框內的紙片會被剪掉，還站在裡面就會受傷。打倒或擊暈正在剪的小兵可以中斷。</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">range</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[4.5, 7.5]
-strafe</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.8
-snipEvery</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[3.4, 4.6]
-firstSnip</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[1.6, 2.6]
-pairRange</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">16
-rect</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[2.6, 2]
-eliteRect</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[3.4, 2.6]
-runSpeed</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10
-markMin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.55
-markMax</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1.6
-cutSpeed</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7
-cutDamage</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1
-dash</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.7
-pieceTime</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.6
-recover</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.6
-eliteSpread</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.3
-rage</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{'speed': 1.4, 'every': 0.6}
-bulletLife</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
     </r>
   </si>
   <si>
@@ -11439,7 +11095,7 @@
       </rPr>
       <t xml:space="preserve">【選擇題】在你腳下和周圍畫出紅圈，一段時間後依序引爆並向外炸出子彈。
 【安靜作答】這段時間只要你開火，它就會喊「作弊！」並朝你射出一排子彈。
-【紅筆批改】畫出好幾條紅線，接著沿著紅線連續射出子彈。
+【紅筆批改】畫出好幾條紅線，接著沿著紅線連續射出子彈。單純攻擊，不算題目。
 【答對了】每道題目結束時如果你沒被打中，它會攤開休息，這時受到 </t>
     </r>
     <r>
@@ -11457,44 +11113,78 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍傷害；被打中就沒有休息。
+      <t xml:space="preserve">倍傷害；被打中就沒有休息。紅筆批改與丟紙團不算題目。
 【申論題（第二型態）】進化後才會出的題目：考卷一邊追著你一邊寫字，留下的筆跡過一下會變成粗墨線，碰到就受傷。
-【填空題】在你周圍畫出 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3×3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">的格子，只有畫 ○ 的格子是正確答案；其他格子會一格一格被墨水填滿，站在裡面就會受傷。進化後只剩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">格安全。
-【是非題】用紅線把場地切成兩半，一半畫上 ✗、一半畫上 ○；時間到時 ✗ 那半邊整片被劃掉，站在那邊就會受傷。進化後有一半機率在中途換邊（陷阱題）。</t>
+【填空題】把整個場地切成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4×3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">格，只有畫 ○ 的 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">格是正確答案（進化後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">格）；其他格子會一格一格被墨水填滿，站在裡面就會受傷。
+【是非題】用紅線把場地切成兩半，一半畫上 ✗、一半畫上 ○；時間到時 ✗ 那半邊整片被劃掉，站在那邊受到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點傷害。進化後有一半機率在中途換邊（陷阱題）。</t>
     </r>
   </si>
   <si>
@@ -11738,7 +11428,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'ask': 1.9, 'ask2': 2.3, 'swapAt': 0.55, 'swapChance': 0.5, 'live': 0.55, 'hatch': 6}
+      <t xml:space="preserve">{'ask': 1.9, 'ask2': 2.3, 'swapAt': 0.55, 'swapChance': 0.5, 'live': 0.55, 'hatch': 6, 'damage': 2}
 blank</t>
     </r>
     <r>
@@ -11756,7 +11446,25 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'cell': 2.6, 'safe': 2, 'safe2': 1, 'every': 0.2, 'fill': 0.7}
+      <t xml:space="preserve">{'cols': 4, 'rows': 3, 'safe': 3, 'safe2': 2, 'ask': 2.4, 'ask2': 2.1, 'every': 0.22, 'fill': 0.7}
+plain</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">['grade', 'toss']
 essay</t>
     </r>
     <r>
@@ -11810,7 +11518,7 @@
       </rPr>
       <t xml:space="preserve">【畫線】在場上拉出幾條橫豎紅線（一定有一條穿過你），紅線畫完後變成粗墨線，站在上面就會受傷。越後期線越多。
 【仿寫】模仿你的技能：在你身邊標記紅圈後引爆（爆墨，進化後才會噴子彈），或射出少量扇形子彈（散射）。
-【喘息】每次攻擊後筆尖插地喘息，受到 </t>
+【喘息】每三次攻擊才會筆尖插地喘息一次，這時受到 </t>
     </r>
     <r>
       <rPr>
@@ -11827,7 +11535,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍傷害。也會使用有缺口的彈幕牆。
+      <t xml:space="preserve">倍傷害；其他攻擊後只會短暫停頓。也會使用有缺口的彈幕牆。
 【書寫衝刺（第二型態）】血量剩三分之一時鎖血進化。進化後會沿紅線高速衝刺 </t>
     </r>
     <r>
@@ -11863,7 +11571,7 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">秒的粗墨線，碰到就受傷。
-【墨水管封印】血量剩三分之二時刀槍不入，並在四周插上 </t>
+【墨水管護盾】血量剩三分之二、以及進化完成時，會把 </t>
     </r>
     <r>
       <rPr>
@@ -11880,41 +11588,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">根墨水管（紅線連到本體）。</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">14 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內打斷所有墨水管，它會倒下 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒並受到三倍傷害；來不及就會回復一些血量。
+      <t xml:space="preserve">根墨水管丟到場上（紅線連到本體）。墨水管全部打掉之前，它只受到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害，而且照常攻擊。
 【筆桿橫掃】倒下筆桿掃過半個場地，起點和終點都會先畫出紅線。貼近筆尖（掃不到的內圈）或衝刺穿過都能躲開。</t>
     </r>
   </si>
@@ -11980,6 +11671,42 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.6
+restEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+pauseTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.7
 lines</t>
     </r>
     <r>
@@ -12033,7 +11760,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'marks': [3], 'radius': 7.5, 'time': 14, 'heal': 0.06, 'stun': 4, 'attackEvery': 3.2, 'lines': 2}
+      <t xml:space="preserve">{'marks': 3, 'radius': 7.5, 'guard': 0.5, 'flight': 0.8, 'arc': 4}
 evolve</t>
     </r>
     <r>
@@ -22165,7 +21892,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -22530,7 +22257,7 @@
       </c>
       <c r="P9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>310</v>
       </c>
@@ -22541,14 +22268,14 @@
         <v>284</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">ROUND(D10*$B$1,0)</f>
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>3.2</v>
+        <v>2.2</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>1</v>
@@ -22557,65 +22284,61 @@
         <v>1</v>
       </c>
       <c r="I10" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="J10" s="8"/>
+        <v>6</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>312</v>
+      </c>
       <c r="K10" s="8" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">K10*$D$1</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="P10" s="10"/>
     </row>
-    <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>284</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">ROUND(D11*$B$1,0)</f>
-        <v>145</v>
+        <v>225</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>316</v>
-      </c>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
       <c r="K11" s="8" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">K11*$D$1</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M11" s="8" t="n">
         <v>2</v>
@@ -22628,25 +22351,25 @@
       </c>
       <c r="P11" s="10"/>
     </row>
-    <row r="12" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
         <v>319</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>320</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>284</v>
-      </c>
       <c r="D12" s="8" t="n">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">ROUND(D12*$B$1,0)</f>
-        <v>225</v>
+        <v>35</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>1</v>
@@ -22655,83 +22378,83 @@
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
       <c r="K12" s="8" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">K12*$D$1</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="N12" s="7"/>
+      <c r="O12" s="6" t="s">
         <v>321</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>322</v>
       </c>
       <c r="P12" s="10"/>
     </row>
-    <row r="13" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+    <row r="13" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>322</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>289</v>
-      </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="12" t="s">
         <v>324</v>
       </c>
-      <c r="D13" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <f aca="false">ROUND(D13*$B$1,0)</f>
-        <v>35</v>
-      </c>
-      <c r="F13" s="8" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="G13" s="8" t="n">
+      <c r="D13" s="13" t="n">
+        <v>900</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>325</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G13" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L13" s="7" t="n">
-        <f aca="false">K13*$D$1</f>
+      <c r="H13" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="M13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="7"/>
-      <c r="O13" s="6" t="s">
-        <v>325</v>
+      <c r="I13" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="M13" s="13"/>
+      <c r="N13" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="O13" s="11" t="s">
+        <v>328</v>
       </c>
       <c r="P13" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="147.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.8</v>
+        <v>2.2</v>
       </c>
       <c r="G14" s="13" t="n">
         <v>1</v>
@@ -22740,14 +22463,14 @@
         <v>1</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J14" s="13"/>
       <c r="K14" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="12" t="s">
@@ -22758,7 +22481,7 @@
       </c>
       <c r="P14" s="10"/>
     </row>
-    <row r="15" customFormat="false" ht="147.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
         <v>333</v>
       </c>
@@ -22766,16 +22489,16 @@
         <v>334</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>1000</v>
+        <v>1300</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="G15" s="13" t="n">
         <v>1</v>
@@ -22784,14 +22507,14 @@
         <v>1</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="J15" s="13"/>
       <c r="K15" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="12" t="s">
@@ -22802,7 +22525,7 @@
       </c>
       <c r="P15" s="10"/>
     </row>
-    <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="331.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>337</v>
       </c>
@@ -22810,16 +22533,16 @@
         <v>338</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1300</v>
+        <v>1100</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>1</v>
@@ -22828,14 +22551,14 @@
         <v>1</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="12" t="s">
@@ -22846,7 +22569,7 @@
       </c>
       <c r="P16" s="10"/>
     </row>
-    <row r="17" customFormat="false" ht="317.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="252.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
         <v>341</v>
       </c>
@@ -22854,16 +22577,16 @@
         <v>342</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F17" s="13" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>1</v>
@@ -22876,10 +22599,10 @@
       </c>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="12" t="s">
@@ -22890,91 +22613,47 @@
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="7" t="s">
         <v>346</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="D18" s="13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>329</v>
-      </c>
-      <c r="F18" s="13" t="n">
+      <c r="C18" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <f aca="false">ROUND(D18*$B$1,0)</f>
+        <v>113</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="13" t="n">
+      <c r="G18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <f aca="false">K18*$D$1</f>
         <v>1</v>
       </c>
-      <c r="H18" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>330</v>
-      </c>
-      <c r="M18" s="13"/>
-      <c r="N18" s="12" t="s">
+      <c r="M18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="7"/>
+      <c r="O18" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="O18" s="11" t="s">
-        <v>348</v>
-      </c>
       <c r="P18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>350</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="D19" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <f aca="false">ROUND(D19*$B$1,0)</f>
-        <v>113</v>
-      </c>
-      <c r="F19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L19" s="7" t="n">
-        <f aca="false">K19*$D$1</f>
-        <v>1</v>
-      </c>
-      <c r="M19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="7"/>
-      <c r="O19" s="6" t="s">
-        <v>351</v>
-      </c>
-      <c r="P19" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -23022,37 +22701,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>276</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>275</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -23060,16 +22739,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -23104,16 +22783,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -23148,16 +22827,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -23188,22 +22867,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -23234,22 +22913,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -23267,10 +22946,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -23280,22 +22959,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -23307,10 +22986,10 @@
         <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -23326,7 +23005,7 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -23358,19 +23037,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -23378,289 +23057,289 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>386</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>387</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>389</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>390</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>388</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>391</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>392</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>393</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>394</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>395</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>395</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>396</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>397</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>400</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>405</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>406</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>407</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>409</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>406</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>410</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>412</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>413</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>414</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>415</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>416</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>417</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>419</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>419</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>420</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>421</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>422</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>423</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>424</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>425</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>426</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>427</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>428</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>429</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>430</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>431</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>432</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>433</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>434</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>438</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>439</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>440</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>442</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>443</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>442</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>444</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>445</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>446</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>447</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>448</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
+        <v>445</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>449</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>450</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>451</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>452</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>453</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>451</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>453</v>
+      </c>
+      <c r="E16" s="9" t="s">
         <v>454</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>455</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>456</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>457</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>458</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>459</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>460</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>461</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>462</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>463</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -23695,13 +23374,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -23709,13 +23388,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -23725,13 +23404,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -23741,13 +23420,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -23757,13 +23436,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -23773,13 +23452,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -23789,13 +23468,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -23805,13 +23484,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -23821,13 +23500,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -23837,13 +23516,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -23853,13 +23532,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -23869,13 +23548,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -23885,13 +23564,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -23901,13 +23580,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -23917,13 +23596,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -23933,13 +23612,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -23949,13 +23628,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -23965,13 +23644,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -23981,13 +23660,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -23997,13 +23676,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>

</xml_diff>

<commit_message>
v0.9.24: Red Ink Execution base damage 300 -> 230
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -6248,7 +6248,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">300
+      <t xml:space="preserve">230
 </t>
     </r>
     <r>
@@ -6328,7 +6328,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">300 </t>
+      <t xml:space="preserve">230 </t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
v0.9.25: drop unused upgrade params from ultimate cards
Ultimate (rare) card upgrades only lower the cost; the params stored in
their upgraded blocks were never applied, so remove them. Fix the
v0.9.24 changelog line that mentioned the unused 400 damage.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="563">
   <si>
     <r>
       <rPr>
@@ -6275,31 +6275,44 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">400
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">半徑：</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">對目標附近最近的敵人造成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">230 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點毀滅性傷害。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">redraw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">重畫</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水：</t>
     </r>
     <r>
       <rPr>
@@ -6319,108 +6332,6 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">對目標附近最近的敵人造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">230 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點毀滅性傷害。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">對目標附近最近的敵人造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">400 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點毀滅性傷害。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">redraw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">重畫</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">重新繪製整個房間：畫面從白紙重新畫出，清除所有敵彈、把被擦掉的掩體畫回來，並獲得 </t>
     </r>
     <r>
@@ -6431,33 +6342,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">重新繪製整個房間：畫面從白紙重新畫出，清除所有敵彈、把被擦掉的掩體畫回來，並獲得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
     </r>
     <r>
       <rPr>
@@ -6539,67 +6423,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">寬度：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">9
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">長度：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -6613,33 +6436,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">60 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害並沖走敵彈。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">掀起一道墨浪橫掃前方，對所有敵人造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80 </t>
     </r>
     <r>
       <rPr>
@@ -6920,125 +6716,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">半徑：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2.5
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">120
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">單體傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">140</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -7120,101 +6797,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">100 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在目標處形成漩渦，把半徑 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">內的敵人吸過來，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2.5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒後爆炸造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">120 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害；只炸到 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人時改為 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">140 </t>
     </r>
     <r>
       <rPr>
@@ -7334,105 +6916,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.5
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">14
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">數量：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">44</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -7472,59 +6955,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內連續放出 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">44 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">支追蹤筆，每支造成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">14 </t>
     </r>
     <r>
       <rPr>
@@ -7589,47 +7019,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">280
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">寬度：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -7654,33 +7043,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用巨筆朝指定方向劃過整個房間，路徑上所有敵人受到 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">280 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">傷害。</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">freezeAll</t>
   </si>
   <si>
@@ -7690,65 +7052,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -7762,33 +7065,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒：所有敵人與敵彈完全靜止，首領也不例外。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">畫面定格 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
     </r>
     <r>
       <rPr>
@@ -22451,23 +21727,21 @@
       <c r="L28" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="M28" s="14" t="s">
+      <c r="M28" s="13"/>
+      <c r="N28" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="N28" s="12" t="s">
-        <v>217</v>
-      </c>
       <c r="O28" s="12" t="s">
-        <v>218</v>
+        <v>87</v>
       </c>
       <c r="P28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>214</v>
@@ -22495,25 +21769,23 @@
         <v>2</v>
       </c>
       <c r="L29" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="M29" s="14" t="s">
-        <v>222</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="M29" s="13"/>
       <c r="N29" s="12" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="O29" s="12" t="s">
-        <v>224</v>
+        <v>87</v>
       </c>
       <c r="P29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>214</v>
@@ -22543,25 +21815,23 @@
         <v>3</v>
       </c>
       <c r="L30" s="14" t="s">
-        <v>227</v>
-      </c>
-      <c r="M30" s="14" t="s">
-        <v>228</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="M30" s="13"/>
       <c r="N30" s="12" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="O30" s="12" t="s">
-        <v>230</v>
+        <v>87</v>
       </c>
       <c r="P30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C31" s="12" t="s">
         <v>214</v>
@@ -22589,13 +21859,11 @@
         <v>2</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>233</v>
-      </c>
-      <c r="M31" s="14" t="s">
-        <v>233</v>
-      </c>
+        <v>227</v>
+      </c>
+      <c r="M31" s="13"/>
       <c r="N31" s="11" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="O31" s="12" t="s">
         <v>87</v>
@@ -22604,10 +21872,10 @@
     </row>
     <row r="32" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>214</v>
@@ -22616,7 +21884,7 @@
         <v>111</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>52</v>
@@ -22635,13 +21903,11 @@
         <v>2</v>
       </c>
       <c r="L32" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="M32" s="14" t="s">
-        <v>238</v>
-      </c>
+        <v>232</v>
+      </c>
+      <c r="M32" s="13"/>
       <c r="N32" s="12" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="O32" s="12" t="s">
         <v>87</v>
@@ -22650,10 +21916,10 @@
     </row>
     <row r="33" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>214</v>
@@ -22683,25 +21949,23 @@
         <v>4</v>
       </c>
       <c r="L33" s="14" t="s">
-        <v>242</v>
-      </c>
-      <c r="M33" s="14" t="s">
-        <v>243</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="M33" s="13"/>
       <c r="N33" s="12" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="O33" s="12" t="s">
-        <v>245</v>
+        <v>87</v>
       </c>
       <c r="P33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="C34" s="12" t="s">
         <v>214</v>
@@ -22729,25 +21993,23 @@
         <v>3</v>
       </c>
       <c r="L34" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="M34" s="14" t="s">
-        <v>249</v>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="M34" s="13"/>
       <c r="N34" s="11" t="s">
-        <v>250</v>
-      </c>
-      <c r="O34" s="11" t="s">
-        <v>251</v>
+        <v>241</v>
+      </c>
+      <c r="O34" s="12" t="s">
+        <v>87</v>
       </c>
       <c r="P34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>214</v>
@@ -22756,7 +22018,7 @@
         <v>36</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="F35" s="12" t="s">
         <v>38</v>
@@ -22777,25 +22039,23 @@
         <v>3</v>
       </c>
       <c r="L35" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="M35" s="14" t="s">
-        <v>256</v>
-      </c>
+        <v>245</v>
+      </c>
+      <c r="M35" s="13"/>
       <c r="N35" s="12" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="O35" s="12" t="s">
-        <v>258</v>
+        <v>87</v>
       </c>
       <c r="P35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>214</v>
@@ -22825,23 +22085,21 @@
       <c r="L36" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="M36" s="14" t="s">
-        <v>261</v>
-      </c>
+      <c r="M36" s="13"/>
       <c r="N36" s="12" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="O36" s="12" t="s">
-        <v>263</v>
+        <v>87</v>
       </c>
       <c r="P36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>214</v>
@@ -22869,13 +22127,11 @@
         <v>3</v>
       </c>
       <c r="L37" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="M37" s="14" t="s">
-        <v>266</v>
-      </c>
+        <v>252</v>
+      </c>
+      <c r="M37" s="13"/>
       <c r="N37" s="12" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="O37" s="12" t="s">
         <v>87</v>
@@ -22919,13 +22175,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="B1" s="15" t="n">
         <v>2.5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="D1" s="15" t="n">
         <v>2</v>
@@ -22942,40 +22198,40 @@
         <v>20</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>279</v>
+        <v>265</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>280</v>
+        <v>266</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>281</v>
+        <v>267</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>32</v>
@@ -22983,13 +22239,13 @@
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>282</v>
+        <v>268</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>283</v>
+        <v>269</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>38</v>
@@ -23011,7 +22267,7 @@
         <v>10</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>1</v>
@@ -23024,22 +22280,22 @@
         <v>1</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="P4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>52</v>
@@ -23072,22 +22328,22 @@
         <v>2</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="P5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>46</v>
@@ -23109,7 +22365,7 @@
         <v>8.5</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="K6" s="8" t="n">
         <v>1.5</v>
@@ -23122,22 +22378,22 @@
         <v>2</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>295</v>
+        <v>281</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="P6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="270.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>64</v>
@@ -23170,22 +22426,22 @@
         <v>2</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>299</v>
+        <v>285</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="P7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>301</v>
+        <v>287</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>44</v>
@@ -23214,22 +22470,22 @@
         <v>2</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>304</v>
+        <v>290</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="P8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>306</v>
+        <v>292</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>307</v>
+        <v>293</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>26</v>
@@ -23258,22 +22514,22 @@
         <v>1</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
       <c r="P9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>310</v>
+        <v>296</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>58</v>
@@ -23295,7 +22551,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>312</v>
+        <v>298</v>
       </c>
       <c r="K10" s="8" t="n">
         <v>1.5</v>
@@ -23308,22 +22564,22 @@
         <v>2</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>313</v>
+        <v>299</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>314</v>
+        <v>300</v>
       </c>
       <c r="P10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>315</v>
+        <v>301</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>316</v>
+        <v>302</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>90</v>
@@ -23352,22 +22608,22 @@
         <v>2</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>317</v>
+        <v>303</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="P11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>319</v>
+        <v>305</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>14</v>
@@ -23397,25 +22653,25 @@
       </c>
       <c r="N12" s="7"/>
       <c r="O12" s="6" t="s">
-        <v>321</v>
+        <v>307</v>
       </c>
       <c r="P12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>322</v>
+        <v>308</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>323</v>
+        <v>309</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>900</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="F13" s="13" t="n">
         <v>0.8</v>
@@ -23434,32 +22690,32 @@
         <v>4</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="12" t="s">
-        <v>327</v>
+        <v>313</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>328</v>
+        <v>314</v>
       </c>
       <c r="P13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="147.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>2.2</v>
@@ -23478,32 +22734,32 @@
         <v>4</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="12" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
       <c r="P14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1300</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>0</v>
@@ -23522,32 +22778,32 @@
         <v>4</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="12" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
       <c r="P15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="331.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>337</v>
+        <v>323</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>338</v>
+        <v>324</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1100</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>1.4</v>
@@ -23566,32 +22822,32 @@
         <v>4</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="12" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>340</v>
+        <v>326</v>
       </c>
       <c r="P16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="252.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>341</v>
+        <v>327</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1400</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>0</v>
@@ -23610,26 +22866,26 @@
         <v>5</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="12" t="s">
-        <v>343</v>
+        <v>329</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="P17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>346</v>
+        <v>332</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>45</v>
@@ -23659,7 +22915,7 @@
       </c>
       <c r="N18" s="7"/>
       <c r="O18" s="6" t="s">
-        <v>347</v>
+        <v>333</v>
       </c>
       <c r="P18" s="10"/>
     </row>
@@ -23709,37 +22965,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>348</v>
+        <v>334</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>349</v>
+        <v>335</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>351</v>
+        <v>337</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>352</v>
+        <v>338</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>353</v>
+        <v>339</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>354</v>
+        <v>340</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>355</v>
+        <v>341</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>356</v>
+        <v>342</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -23747,16 +23003,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>357</v>
+        <v>343</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>358</v>
+        <v>344</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>359</v>
+        <v>345</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -23791,16 +23047,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>360</v>
+        <v>346</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>361</v>
+        <v>347</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>362</v>
+        <v>348</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -23835,16 +23091,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>363</v>
+        <v>349</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>365</v>
+        <v>351</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -23875,22 +23131,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>368</v>
+        <v>354</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>369</v>
+        <v>355</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -23921,22 +23177,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>370</v>
+        <v>356</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>371</v>
+        <v>357</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>372</v>
+        <v>358</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -23954,10 +23210,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -23967,22 +23223,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>310</v>
+        <v>296</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>375</v>
+        <v>361</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>376</v>
+        <v>362</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -23994,10 +23250,10 @@
         <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -24013,7 +23269,7 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>377</v>
+        <v>363</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -24045,19 +23301,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>378</v>
+        <v>364</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>379</v>
+        <v>365</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>380</v>
+        <v>366</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>381</v>
+        <v>367</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -24065,289 +23321,289 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>382</v>
+        <v>368</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>383</v>
+        <v>369</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>385</v>
+        <v>371</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>390</v>
+        <v>376</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>391</v>
+        <v>377</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>392</v>
+        <v>378</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>393</v>
+        <v>379</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>394</v>
+        <v>380</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>405</v>
+        <v>391</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>417</v>
+        <v>403</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>418</v>
+        <v>404</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>420</v>
+        <v>406</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>422</v>
+        <v>408</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>423</v>
+        <v>409</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>424</v>
+        <v>410</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>425</v>
+        <v>411</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>426</v>
+        <v>412</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>427</v>
+        <v>413</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>428</v>
+        <v>414</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>429</v>
+        <v>415</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>430</v>
+        <v>416</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>431</v>
+        <v>417</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>432</v>
+        <v>418</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>432</v>
+        <v>418</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>433</v>
+        <v>419</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>434</v>
+        <v>420</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>435</v>
+        <v>421</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>436</v>
+        <v>422</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>437</v>
+        <v>423</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>438</v>
+        <v>424</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>439</v>
+        <v>425</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>440</v>
+        <v>426</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>441</v>
+        <v>427</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>442</v>
+        <v>428</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>443</v>
+        <v>429</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>444</v>
+        <v>430</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>445</v>
+        <v>431</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>446</v>
+        <v>432</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>447</v>
+        <v>433</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>448</v>
+        <v>434</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>449</v>
+        <v>435</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>450</v>
+        <v>436</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>451</v>
+        <v>437</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>452</v>
+        <v>438</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>453</v>
+        <v>439</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>454</v>
+        <v>440</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>455</v>
+        <v>441</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>456</v>
+        <v>442</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>457</v>
+        <v>443</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>458</v>
+        <v>444</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>459</v>
+        <v>445</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -24382,13 +23638,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>460</v>
+        <v>446</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>461</v>
+        <v>447</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -24396,13 +23652,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>464</v>
+        <v>450</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -24412,13 +23668,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>465</v>
+        <v>451</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -24428,13 +23684,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>466</v>
+        <v>452</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -24444,13 +23700,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>467</v>
+        <v>453</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -24460,13 +23716,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>468</v>
+        <v>454</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -24476,13 +23732,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>469</v>
+        <v>455</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -24492,13 +23748,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>470</v>
+        <v>456</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -24508,13 +23764,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>471</v>
+        <v>457</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -24524,13 +23780,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>472</v>
+        <v>458</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -24540,13 +23796,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>473</v>
+        <v>459</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -24556,13 +23812,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>474</v>
+        <v>460</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -24572,13 +23828,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>476</v>
+        <v>462</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -24588,13 +23844,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>477</v>
+        <v>463</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -24604,13 +23860,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>478</v>
+        <v>464</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -24620,13 +23876,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>479</v>
+        <v>465</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -24636,13 +23892,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>480</v>
+        <v>466</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -24652,13 +23908,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>481</v>
+        <v>467</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -24668,13 +23924,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>482</v>
+        <v>468</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -24684,13 +23940,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>475</v>
+        <v>461</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>483</v>
+        <v>469</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>
@@ -24726,16 +23982,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>484</v>
+        <v>470</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>485</v>
+        <v>471</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>486</v>
+        <v>472</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -24743,13 +23999,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>487</v>
+        <v>473</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>488</v>
+        <v>474</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>489</v>
+        <v>475</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -24758,13 +24014,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>487</v>
+        <v>473</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>490</v>
+        <v>476</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>491</v>
+        <v>477</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -24773,13 +24029,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>487</v>
+        <v>473</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>492</v>
+        <v>478</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>493</v>
+        <v>479</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
@@ -24788,13 +24044,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>494</v>
+        <v>480</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>495</v>
+        <v>481</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>496</v>
+        <v>482</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -24803,13 +24059,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>494</v>
+        <v>480</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>497</v>
+        <v>483</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>498</v>
+        <v>484</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -24818,13 +24074,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>494</v>
+        <v>480</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>499</v>
+        <v>485</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>500</v>
+        <v>486</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -24833,13 +24089,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>502</v>
+        <v>488</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>503</v>
+        <v>489</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -24848,13 +24104,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>504</v>
+        <v>490</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>505</v>
+        <v>491</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -24863,13 +24119,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>506</v>
+        <v>492</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>507</v>
+        <v>493</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -24878,13 +24134,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>508</v>
+        <v>494</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>509</v>
+        <v>495</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -24893,13 +24149,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>510</v>
+        <v>496</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>509</v>
+        <v>495</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -24908,28 +24164,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>501</v>
+        <v>487</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>511</v>
+        <v>497</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>512</v>
+        <v>498</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>513</v>
+        <v>499</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>487</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>500</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>501</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>514</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>515</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>1</v>
@@ -24938,13 +24194,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>517</v>
+        <v>503</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>518</v>
+        <v>504</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>1</v>
@@ -24953,13 +24209,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>519</v>
+        <v>505</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>520</v>
+        <v>506</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>10</v>
@@ -24968,13 +24224,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>521</v>
+        <v>507</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>522</v>
+        <v>508</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>100</v>
@@ -24983,13 +24239,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>523</v>
+        <v>509</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>524</v>
+        <v>510</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>200</v>
@@ -24998,13 +24254,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>525</v>
+        <v>511</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>526</v>
+        <v>512</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>1</v>
@@ -25013,13 +24269,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>527</v>
+        <v>513</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>528</v>
+        <v>514</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>30</v>
@@ -25028,13 +24284,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
+        <v>502</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>516</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>529</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>530</v>
       </c>
       <c r="D21" s="8" t="n">
         <v>5</v>
@@ -25043,13 +24299,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>531</v>
+        <v>517</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>532</v>
+        <v>518</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>10</v>
@@ -25058,13 +24314,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>533</v>
+        <v>519</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>534</v>
+        <v>520</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>10</v>
@@ -25073,13 +24329,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>535</v>
+        <v>521</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>536</v>
+        <v>522</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>5</v>
@@ -25088,13 +24344,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>537</v>
+        <v>523</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>538</v>
+        <v>524</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>10</v>
@@ -25103,13 +24359,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>539</v>
+        <v>525</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>540</v>
+        <v>526</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>25</v>
@@ -25118,13 +24374,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>541</v>
+        <v>527</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>542</v>
+        <v>528</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>10</v>
@@ -25133,13 +24389,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>543</v>
+        <v>529</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>544</v>
+        <v>530</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>100</v>
@@ -25148,13 +24404,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>545</v>
+        <v>531</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>546</v>
+        <v>532</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>1</v>
@@ -25163,13 +24419,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>547</v>
+        <v>533</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>548</v>
+        <v>534</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>10</v>
@@ -25178,13 +24434,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>549</v>
+        <v>535</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>550</v>
+        <v>536</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>1</v>
@@ -25193,13 +24449,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>551</v>
+        <v>537</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>10</v>
@@ -25208,13 +24464,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>553</v>
+        <v>539</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>554</v>
+        <v>540</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>4</v>
@@ -25223,13 +24479,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>555</v>
+        <v>541</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>556</v>
+        <v>542</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>1000</v>
@@ -25238,13 +24494,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>557</v>
+        <v>543</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>558</v>
+        <v>544</v>
       </c>
       <c r="D35" s="8" t="n">
         <v>1</v>
@@ -25253,13 +24509,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>559</v>
+        <v>545</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>560</v>
+        <v>546</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>10</v>
@@ -25268,13 +24524,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>561</v>
+        <v>547</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>562</v>
+        <v>548</v>
       </c>
       <c r="D37" s="8" t="n">
         <v>1</v>
@@ -25283,13 +24539,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>563</v>
+        <v>549</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>564</v>
+        <v>550</v>
       </c>
       <c r="D38" s="8" t="n">
         <v>13</v>
@@ -25298,13 +24554,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>565</v>
+        <v>551</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="D39" s="8" t="n">
         <v>1</v>
@@ -25313,13 +24569,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>567</v>
+        <v>553</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>568</v>
+        <v>554</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>1000</v>
@@ -25328,13 +24584,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>569</v>
+        <v>555</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>570</v>
+        <v>556</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>5</v>
@@ -25343,13 +24599,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>571</v>
+        <v>557</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>572</v>
+        <v>558</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>25</v>
@@ -25358,13 +24614,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>573</v>
+        <v>559</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>574</v>
+        <v>560</v>
       </c>
       <c r="D43" s="8" t="n">
         <v>10</v>
@@ -25373,13 +24629,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>516</v>
+        <v>502</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>575</v>
+        <v>561</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>576</v>
+        <v>562</v>
       </c>
       <c r="D44" s="8" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
v0.9.27: tutorial reminders and rewards page, exam cheat spin, resume countdown toggle
- Tutorial: re-show a step's intro (marked as a refresher) after 30 s
  without finishing, keeping progress; new "rewards & outfits" info page
  with chest/outfit animation; no idle skill-button shake in tutorial
- Touch cancel hints now say to drag onto the red X
- Exam boss cheat: spins a full turn while spraying a bullet ring;
  codex animation and description updated
- Settings: "resume countdown" toggle (default on)
- Custom outfit wear/overwrite halves sit inside the slot frame

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -10371,7 +10371,7 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">【選擇題】在你腳下和周圍畫出紅圈，一段時間後依序引爆並向外炸出子彈。
-【安靜作答】這段時間只要你開火，它就會喊「作弊！」並朝你射出一排子彈。
+【安靜作答】這段時間只要你開火，它就會喊「作弊！」並原地轉一圈，朝四面八方射出一圈子彈。
 【紅筆批改】畫出好幾條紅線，接著沿著紅線連續射出子彈。單純攻擊，不算題目。
 【答對了】每道題目結束時如果你沒被打中，它會攤開休息，這時受到 </t>
     </r>
@@ -10633,7 +10633,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'time': 2.8, 'cool': 0.35, 'shots': 3, 'shots2': 5, 'spread': 0.5}
+      <t xml:space="preserve">{'time': 2.8, 'cool': 0.5, 'spinTime': 0.7, 'ring': 12, 'ring2': 18, 'speed': 1.1}
 grade</t>
     </r>
     <r>

</xml_diff>

<commit_message>
v0.9.29: eraser card applies instantly, deals 5 damage and knocks back
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -2075,7 +2075,47 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.4</t>
+      <t xml:space="preserve">1.4
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊退力：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">14</t>
     </r>
   </si>
   <si>
@@ -2120,7 +2160,31 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">朝指定方向揮動橡皮擦，擦掉扇形範圍內所有敵彈。</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">朝指定方向揮動橡皮擦，立刻擦掉扇形範圍內所有敵彈，並對範圍內的敵人造成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">傷害並擊退。</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">（同基本）</t>
@@ -20748,7 +20812,7 @@
       </c>
       <c r="P7" s="10"/>
     </row>
-    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
         <v>81</v>
       </c>

</xml_diff>

<commit_message>
v0.9.31: redraw makes normal cards free, ult unlock reshuffle, smaller vortex
- Redraw: normal cards cost no ink for 5.5 s (red 0 cost, HUD timer);
  old bullet wipe / cover restore / ink gain removed with its dead code
- Level 1 ults: execute, tsunami, dual wield; redraw moves to level 5
- Ink vortex radius 7 -> 5.5
- Outfit wear/overwrite split closes when tapping anywhere else

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -6363,57 +6363,87 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">redraw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">重畫</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">重新繪製整個房間：畫面從白紙重新畫出，清除所有敵彈、把被擦掉的掩體畫回來，並獲得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨水。</t>
+    <t xml:space="preserve">dualWield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">雙持</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內左手也拿起一把同樣的武器，每次攻擊兩把一起發射；時間到時會把左手的武器甩掉收起。</t>
     </r>
   </si>
   <si>
@@ -6511,10 +6541,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">dualWield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">雙持</t>
+    <t xml:space="preserve">redraw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">重畫</t>
   </si>
   <si>
     <r>
@@ -6572,26 +6602,34 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">6</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內左手也拿起一把同樣的武器，每次攻擊兩把一起發射；時間到時會把左手的武器甩掉收起。</t>
+      <t xml:space="preserve">5.5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">重新提筆：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內施放一般卡都不消耗墨水（特殊技仍需墨水）。</t>
     </r>
   </si>
   <si>
@@ -6675,7 +6713,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">7
+      <t xml:space="preserve">5.5
 </t>
     </r>
     <r>
@@ -6792,7 +6830,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">7 </t>
+      <t xml:space="preserve">5.5 </t>
     </r>
     <r>
       <rPr>
@@ -21811,10 +21849,10 @@
         <v>214</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>111</v>
+        <v>36</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="F29" s="12" t="s">
         <v>52</v>
@@ -21836,7 +21874,7 @@
         <v>219</v>
       </c>
       <c r="M29" s="13"/>
-      <c r="N29" s="12" t="s">
+      <c r="N29" s="11" t="s">
         <v>220</v>
       </c>
       <c r="O29" s="12" t="s">
@@ -21867,7 +21905,7 @@
         <v>16</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I30" s="13" t="n">
         <v>0</v>
@@ -21901,10 +21939,10 @@
         <v>214</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>36</v>
+        <v>111</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>52</v>
@@ -21926,7 +21964,7 @@
         <v>227</v>
       </c>
       <c r="M31" s="13"/>
-      <c r="N31" s="11" t="s">
+      <c r="N31" s="12" t="s">
         <v>228</v>
       </c>
       <c r="O31" s="12" t="s">

</xml_diff>

<commit_message>
v0.9.34: course timetable mode, relics, mode info popups, dots rewards, AI notice
- Endless mode renamed to Timetable mode; acts of 4 distinct courses + boss page
- 5 courses (math, P.E., computer, study hall, cram) with intro popup, challenge bar, reward, HUD icon
- Relics tab in weapon view (4 relics, bought with ink dots, one per run)
- Ink dots from boss kills and as chest tiles
- (i) buttons and first-play popups for both modes
- AI-generated notice in privacy popup

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -15,6 +15,8 @@
     <sheet name="小遊戲" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="小遊戲獎懲" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="成就與墨點" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="遺物" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="課程" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">卡牌!$A$1:$P$37</definedName>
@@ -79,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="620">
   <si>
     <r>
       <rPr>
@@ -108,7 +110,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.07</t>
+      <t xml:space="preserve">beta v0.9.34</t>
     </r>
     <r>
       <rPr>
@@ -207,7 +209,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">beta v0.7.07 </t>
+      <t xml:space="preserve">beta v0.9.34 </t>
     </r>
     <r>
       <rPr>
@@ -18985,7 +18987,7 @@
     <t xml:space="preserve">筆記本：擊敗頭目</t>
   </si>
   <si>
-    <t xml:space="preserve">無盡：到達頁數</t>
+    <t xml:space="preserve">課表模式：到達頁數</t>
   </si>
   <si>
     <r>
@@ -19057,6 +19059,58 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">墨點</t>
+  </si>
+  <si>
+    <t xml:space="preserve">寶箱掉落墨點機率</t>
+  </si>
+  <si>
+    <t xml:space="preserve">寶箱每格抽到墨點（其餘為顏色或配飾）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">寶箱墨點數量</t>
+  </si>
+  <si>
+    <t xml:space="preserve">每次抽到墨點的數量（最少～最多）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗頭目獲得墨點</t>
+  </si>
+  <si>
+    <t xml:space="preserve">筆記本與課表模式</t>
+  </si>
+  <si>
     <t xml:space="preserve">等級獎勵</t>
   </si>
   <si>
@@ -19117,7 +19171,7 @@
     <t xml:space="preserve">第一頁</t>
   </si>
   <si>
-    <t xml:space="preserve">完成第一局冒險（筆記本或無盡）</t>
+    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
   </si>
   <si>
     <t xml:space="preserve">擦身而過</t>
@@ -19517,7 +19571,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">無盡模式抵達第 </t>
+      <t xml:space="preserve">課表模式抵達第 </t>
     </r>
     <r>
       <rPr>
@@ -19781,7 +19835,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">無盡模式抵達第 </t>
+      <t xml:space="preserve">課表模式抵達第 </t>
     </r>
     <r>
       <rPr>
@@ -19851,6 +19905,1345 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">遺物</t>
+  </si>
+  <si>
+    <t xml:space="preserve">價格（墨點）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">參數</t>
+  </si>
+  <si>
+    <t xml:space="preserve">備用筆芯</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">依武器增加彈匣容量：鋼筆 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、鉛筆 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、刷子 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、釘書機 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、螢光筆 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（圓規沒有彈匣，不受影響）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pen</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+pencil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4
+brush</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+stapler</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+highlighter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">立可白</t>
+  </si>
+  <si>
+    <t xml:space="preserve">每局第一次受到傷害時，完全抵銷這次傷害。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">guards</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+invuln</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">換彈時間縮短 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">reload</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.88</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">急救貼布</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每擊敗一隻頭目，回復 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回復：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">課程</t>
+  </si>
+  <si>
+    <t xml:space="preserve">挑戰</t>
+  </si>
+  <si>
+    <t xml:space="preserve">完成獎勵</t>
+  </si>
+  <si>
+    <t xml:space="preserve">數學課</t>
+  </si>
+  <si>
+    <t xml:space="preserve">老師在黑板上寫滿了數字，所有敵人都被編了號。要照順序來，不能亂跳！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 每隻敵人頭上有編號，紅色的是目前輪到的號碼。
+• 還沒輪到的敵人，受到的傷害減少 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{off}%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 依照編號由小到大，連續擊倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{goal} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">隻敵人。
+• 打錯順序（擊倒不是當前號碼的敵人）會讓連續紀錄歸零。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本頁加分：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">800
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水補滿：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">off</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
+goal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">體育課</t>
+  </si>
+  <si>
+    <t xml:space="preserve">操場上大家都在跑，連敵人也不例外。跑快一點，在時間內結束戰鬥！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 你的移動速度提高 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{speed}%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。
+• 敵人的行動與子彈速度也提高 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{foe}%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 在 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{time} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內清除本頁所有敵人。
+• 進度條代表已擊倒的敵人比例，右側顯示剩餘時間。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本頁加分：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1000
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨點：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">speed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2
+foe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2
+time</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">資訊課</t>
+  </si>
+  <si>
+    <t xml:space="preserve">電腦教室裡有人亂按了「複製貼上」，敵人會不斷分身。找出本尊！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{every} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒，場上會有一隻敵人複製自己，同時最多存在 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{max} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個副本。
+• 副本只有 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{hp}% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">的生命，頭上有「副本」標記；擊倒本尊會讓它的副本一起消失。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 擊倒本頁所有的本尊。
+• 副本不計入進度，也不給分數與墨水。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本頁加分：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">800
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回復生命：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">every</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6
+max</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4
+hp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">自習課</t>
+  </si>
+  <si>
+    <t xml:space="preserve">教室裡很安靜，敵人都趴在桌上睡著了。小聲一點，別吵醒大家！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 敵人睡著時不會移動，也不會攻擊。
+• 開槍的聲音與靠得太近都會提高警覺值，警覺滿了全班會一起醒來。
+• 睡著的敵人被打到會醒來，但受到的傷害變成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{sleep} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 在全班醒來之前，擊倒本頁所有敵人。
+• 畫面上方的「警覺」會即時顯示目前的警覺值。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本頁加分：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">800
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回復生命：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水補滿：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">shot</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.05
+near</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.2
+radius</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5
+decay</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.05
+sleep</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">補習班</t>
+  </si>
+  <si>
+    <t xml:space="preserve">放學後的補習班，題目又多又難。撐過去，收穫也加倍。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 敵人數量增加 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{budget}%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。
+• 敵人生命提高 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{hpUp}%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。
+• 本頁擊倒敵人的分數變成 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{score} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 清除本頁所有敵人，而且不能受傷。
+• 受到傷害就會挑戰失敗，但本頁仍可繼續打完。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本頁加分：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1600
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨點：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">budget</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.4
+hp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.15
+score</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">（每幕）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁為一幕：前 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁各抽一堂不同的課（同一幕不重複），第 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁為頭目、不套用課程。</t>
     </r>
   </si>
 </sst>
@@ -24072,7 +25465,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -24281,22 +25674,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>487</v>
+        <v>500</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="E14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>503</v>
@@ -24304,140 +25697,140 @@
       <c r="C15" s="7" t="s">
         <v>504</v>
       </c>
-      <c r="D15" s="8" t="n">
-        <v>1</v>
+      <c r="D15" s="8" t="s">
+        <v>505</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>502</v>
+        <v>487</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="E18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="E20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="E21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>5</v>
@@ -24446,13 +25839,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>10</v>
@@ -24461,73 +25854,73 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="E28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>10</v>
@@ -24536,213 +25929,529 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="E31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D44" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" s="10"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>565</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>566</v>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E45" s="10"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>568</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E46" s="10"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>570</v>
+      </c>
+      <c r="D47" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="10"/>
+      <c r="E47" s="10"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>574</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="E2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>577</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>582</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="E5" s="10"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>585</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>587</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>589</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>592</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>593</v>
+      </c>
+      <c r="G2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>595</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>597</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>599</v>
+      </c>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>602</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="G4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>610</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>611</v>
+      </c>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>616</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="G6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>618</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
v0.9.35: calmer achievements, modes guide in settings, weapons & relics UI polish, relic unlock lv3, harder timetable mode
- Achievement tiles fade in gently instead of bouncing
- Remove (i) buttons from main menu; add Guide button in settings
- Bigger, shorter guide/privacy popups with larger edge margins
- Weapons & Relics: tab slide animation, relic equip animation, relics unlock at level 3, larger text
- Timetable mode: new enemy types every 2 pages, higher enemy budget

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -20283,17 +20283,17 @@
     <t xml:space="preserve">數學課</t>
   </si>
   <si>
-    <t xml:space="preserve">老師在黑板上寫滿了數字，所有敵人都被編了號。要照順序來，不能亂跳！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 每隻敵人頭上有編號，紅色的是目前輪到的號碼。
-• 還沒輪到的敵人，受到的傷害減少 </t>
+    <t xml:space="preserve">黑板上全是數字，敵人也被編了號。照順序來！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 敵人頭上有編號，紅色是現在輪到的
+• 沒輪到的敵人，受到的傷害 −</t>
     </r>
     <r>
       <rPr>
@@ -20304,23 +20304,15 @@
       </rPr>
       <t xml:space="preserve">{off}%</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 依照編號由小到大，連續擊倒 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 依編號由小到大，連續擊倒 </t>
     </r>
     <r>
       <rPr>
@@ -20337,8 +20329,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">隻敵人。
-• 打錯順序（擊倒不是當前號碼的敵人）會讓連續紀錄歸零。</t>
+      <t xml:space="preserve">隻
+• 打錯順序，連續紀錄歸零</t>
     </r>
   </si>
   <si>
@@ -20433,79 +20425,63 @@
     <t xml:space="preserve">體育課</t>
   </si>
   <si>
-    <t xml:space="preserve">操場上大家都在跑，連敵人也不例外。跑快一點，在時間內結束戰鬥！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 你的移動速度提高 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{speed}%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。
-• 敵人的行動與子彈速度也提高 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{foe}%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 在 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{time} </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內清除本頁所有敵人。
-• 進度條代表已擊倒的敵人比例，右側顯示剩餘時間。</t>
+    <t xml:space="preserve">操場上大家都在跑。快一點，趕在時間內結束！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 你的移動速度 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+{speed}%
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">敵人與敵彈的速度也 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+{foe}%</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">• {time} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內清除全部敵人
+• 進度條是擊倒比例，右側顯示剩餘時間</t>
     </r>
   </si>
   <si>
@@ -20620,7 +20596,7 @@
     <t xml:space="preserve">資訊課</t>
   </si>
   <si>
-    <t xml:space="preserve">電腦教室裡有人亂按了「複製貼上」，敵人會不斷分身。找出本尊！</t>
+    <t xml:space="preserve">有人亂按「複製貼上」，敵人不斷分身。找出本尊！</t>
   </si>
   <si>
     <r>
@@ -20646,7 +20622,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒，場上會有一隻敵人複製自己，同時最多存在 </t>
+      <t xml:space="preserve">秒，一隻敵人複製自己（最多 </t>
     </r>
     <r>
       <rPr>
@@ -20663,7 +20639,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">個副本。
+      <t xml:space="preserve">個副本）
 • 副本只有 </t>
     </r>
     <r>
@@ -20681,12 +20657,12 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">的生命，頭上有「副本」標記；擊倒本尊會讓它的副本一起消失。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">• 擊倒本頁所有的本尊。
-• 副本不計入進度，也不給分數與墨水。</t>
+      <t xml:space="preserve">生命；擊倒本尊，副本一起消失</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 擊倒所有本尊
+• 副本不計進度，也沒有分數與墨水</t>
   </si>
   <si>
     <r>
@@ -20800,18 +20776,18 @@
     <t xml:space="preserve">自習課</t>
   </si>
   <si>
-    <t xml:space="preserve">教室裡很安靜，敵人都趴在桌上睡著了。小聲一點，別吵醒大家！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 敵人睡著時不會移動，也不會攻擊。
-• 開槍的聲音與靠得太近都會提高警覺值，警覺滿了全班會一起醒來。
-• 睡著的敵人被打到會醒來，但受到的傷害變成 </t>
+    <t xml:space="preserve">教室很安靜，敵人都睡著了。小聲一點！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 敵人睡著，不動也不攻擊
+• 開槍聲與靠近會提高警覺，滿了全班醒來
+• 睡著的敵人被打到會醒，但受到 </t>
     </r>
     <r>
       <rPr>
@@ -20828,12 +20804,12 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">倍。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">• 在全班醒來之前，擊倒本頁所有敵人。
-• 畫面上方的「警覺」會即時顯示目前的警覺值。</t>
+      <t xml:space="preserve">倍傷害</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 全班醒來前，清除所有敵人
+• 畫面上方顯示目前的警覺值</t>
   </si>
   <si>
     <r>
@@ -21005,74 +20981,66 @@
     <t xml:space="preserve">補習班</t>
   </si>
   <si>
-    <t xml:space="preserve">放學後的補習班，題目又多又難。撐過去，收穫也加倍。</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 敵人數量增加 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{budget}%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。
-• 敵人生命提高 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{hpUp}%</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。
-• 本頁擊倒敵人的分數變成 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{score} </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">倍。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">• 清除本頁所有敵人，而且不能受傷。
-• 受到傷害就會挑戰失敗，但本頁仍可繼續打完。</t>
+    <t xml:space="preserve">放學後的補習班：題目又多又難，收穫也加倍。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 敵人數量 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+{budget}%
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">敵人生命 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+{hpUp}%
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊倒分數 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×{score}</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 清除所有敵人，而且不能受傷
+• 受傷就失敗，但仍可繼續打完</t>
   </si>
   <si>
     <r>
@@ -26335,7 +26303,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
         <v>588</v>
       </c>
@@ -26366,7 +26334,7 @@
       <c r="C3" s="7" t="s">
         <v>596</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>597</v>
       </c>
       <c r="E3" s="7" t="s">
@@ -26377,7 +26345,7 @@
       </c>
       <c r="G3" s="10"/>
     </row>
-    <row r="4" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
         <v>600</v>
       </c>

</xml_diff>

<commit_message>
v0.9.39: new courses (discipline, music), remove study hall and cram, dizzy achievement, slower scissors summons
- Courses: math, P.E., computer, discipline hour (dodge chalk), music (step into circles)
- Simplified course briefing text
- Achievement dizzy: spin in place 10 turns
- Scissors boss summons 30% slower

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="622">
   <si>
     <r>
       <rPr>
@@ -10090,7 +10090,25 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">knockMult</t>
+      <t xml:space="preserve">summonMult</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.3
+knockMult</t>
     </r>
     <r>
       <rPr>
@@ -19908,6 +19926,36 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">頭暈目眩</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">連續原地旋轉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">圈（中間可停一下）</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">遺物</t>
   </si>
   <si>
@@ -20283,17 +20331,17 @@
     <t xml:space="preserve">數學課</t>
   </si>
   <si>
-    <t xml:space="preserve">黑板上全是數字，敵人也被編了號。照順序來！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 敵人頭上有編號，紅色是現在輪到的
-• 沒輪到的敵人，受到的傷害 −</t>
+    <t xml:space="preserve">照編號順序打！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 敵人有編號，紅色的先打
+• 沒輪到的敵人，傷害 −</t>
     </r>
     <r>
       <rPr>
@@ -20312,7 +20360,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">• 依編號由小到大，連續擊倒 </t>
+      <t xml:space="preserve">• 依序連續擊倒 </t>
     </r>
     <r>
       <rPr>
@@ -20329,8 +20377,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">隻
-• 打錯順序，連續紀錄歸零</t>
+      <t xml:space="preserve">隻（打錯歸零）</t>
     </r>
   </si>
   <si>
@@ -20425,16 +20472,16 @@
     <t xml:space="preserve">體育課</t>
   </si>
   <si>
-    <t xml:space="preserve">操場上大家都在跑。快一點，趕在時間內結束！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 你的移動速度 </t>
+    <t xml:space="preserve">跑起來，趕在時間內結束！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 你的速度 </t>
     </r>
     <r>
       <rPr>
@@ -20452,7 +20499,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">敵人與敵彈的速度也 </t>
+      <t xml:space="preserve">敵人與敵彈也 </t>
     </r>
     <r>
       <rPr>
@@ -20480,8 +20527,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒內清除全部敵人
-• 進度條是擊倒比例，右側顯示剩餘時間</t>
+      <t xml:space="preserve">秒內清場</t>
     </r>
   </si>
   <si>
@@ -20596,7 +20642,7 @@
     <t xml:space="preserve">資訊課</t>
   </si>
   <si>
-    <t xml:space="preserve">有人亂按「複製貼上」，敵人不斷分身。找出本尊！</t>
+    <t xml:space="preserve">敵人會分身，找出本尊！</t>
   </si>
   <si>
     <r>
@@ -20622,7 +20668,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒，一隻敵人複製自己（最多 </t>
+      <t xml:space="preserve">秒複製一隻（最多 </t>
     </r>
     <r>
       <rPr>
@@ -20639,7 +20685,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">個副本）
+      <t xml:space="preserve">個）
 • 副本只有 </t>
     </r>
     <r>
@@ -20657,12 +20703,11 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">生命；擊倒本尊，副本一起消失</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">• 擊倒所有本尊
-• 副本不計進度，也沒有分數與墨水</t>
+      <t xml:space="preserve">血，本尊倒下就消失</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">• 擊倒所有本尊</t>
   </si>
   <si>
     <r>
@@ -20773,43 +20818,74 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">自習課</t>
-  </si>
-  <si>
-    <t xml:space="preserve">教室很安靜，敵人都睡著了。小聲一點！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 敵人睡著，不動也不攻擊
-• 開槍聲與靠近會提高警覺，滿了全班醒來
-• 睡著的敵人被打到會醒，但受到 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{sleep} </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">倍傷害</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">• 全班醒來前，清除所有敵人
-• 畫面上方顯示目前的警覺值</t>
+    <t xml:space="preserve">訓導課</t>
+  </si>
+  <si>
+    <t xml:space="preserve">老師氣得丟粉筆，看準時機閃過去！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{every} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒飛來一顆粉筆
+• 衝刺冷卻 −</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{dash}%</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 衝刺閃過子彈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{goal} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
   </si>
   <si>
     <r>
@@ -20827,7 +20903,256 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">800
+      <t xml:space="preserve">900
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨點：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">every</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.6
+first</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.5
+speed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9
+life</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+spread</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.12
+dashCd</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+goal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">音樂課</t>
+  </si>
+  <si>
+    <t xml:space="preserve">跟著節奏，踩進地上的圈圈！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 戰鬥時地上不時出現圈圈
+• 圈圈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{life} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒後消失</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 踩中 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{goal} </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個圈圈</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本頁加分：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">900
 </t>
     </r>
     <r>
@@ -20875,7 +21200,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">shot</t>
+      <t xml:space="preserve">every</t>
     </r>
     <r>
       <rPr>
@@ -20894,8 +21219,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.05
-near</t>
+      <t xml:space="preserve">2
+first</t>
     </r>
     <r>
       <rPr>
@@ -20914,7 +21239,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.2
+      <t xml:space="preserve">2
+life</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
 radius</t>
     </r>
     <r>
@@ -20934,8 +21279,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">5
-decay</t>
+      <t xml:space="preserve">1.3
+max</t>
     </r>
     <r>
       <rPr>
@@ -20954,8 +21299,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.05
-sleep</t>
+      <t xml:space="preserve">2
+minFar</t>
     </r>
     <r>
       <rPr>
@@ -20974,121 +21319,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">補習班</t>
-  </si>
-  <si>
-    <t xml:space="preserve">放學後的補習班：題目又多又難，收穫也加倍。</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 敵人數量 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+{budget}%
-• </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">敵人生命 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+{hpUp}%
-• </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊倒分數 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">×{score}</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">• 清除所有敵人，而且不能受傷
-• 受傷就失敗，但仍可繼續打完</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">本頁加分：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1600
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">墨點：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">budget</t>
+      <t xml:space="preserve">3
+rangeX</t>
     </r>
     <r>
       <rPr>
@@ -21107,8 +21339,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.4
-hp</t>
+      <t xml:space="preserve">8
+rangeZ</t>
     </r>
     <r>
       <rPr>
@@ -21127,8 +21359,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.15
-score</t>
+      <t xml:space="preserve">4.5
+goal</t>
     </r>
     <r>
       <rPr>
@@ -21147,7 +21379,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2</t>
+      <t xml:space="preserve">5</t>
     </r>
   </si>
   <si>
@@ -24164,7 +24396,7 @@
       </c>
       <c r="P13" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="147.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="161.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>315</v>
       </c>
@@ -25433,7 +25665,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -26149,6 +26381,21 @@
         <v>3</v>
       </c>
       <c r="E47" s="10"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>572</v>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E48" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -26177,16 +26424,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>447</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -26194,31 +26441,31 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E3" s="10"/>
     </row>
@@ -26227,28 +26474,28 @@
         <v>394</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E5" s="10"/>
     </row>
@@ -26282,7 +26529,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>471</v>
@@ -26291,13 +26538,13 @@
         <v>342</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -26305,115 +26552,115 @@
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="G4" s="10"/>
     </row>
-    <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="G5" s="10"/>
     </row>
-    <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.9.40: choice pages need a second tap, ink tsunami damage 60 -> 75
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -6472,7 +6472,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">60
+      <t xml:space="preserve">75
 </t>
     </r>
     <r>
@@ -6531,7 +6531,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">60 </t>
+      <t xml:space="preserve">75 </t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
v0.9.44: dev-only debug panel, Paper Fortress ult, pen-sweep dodge tutorial, compass breaks props, sequential boss rewards, boss first-encounter page, resume interrupted runs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -19,7 +19,7 @@
     <sheet name="課程" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">卡牌!$A$1:$P$37</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">卡牌!$A$1:$P$38</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="626">
   <si>
     <r>
       <rPr>
@@ -6540,6 +6540,98 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">傷害並沖走敵彈。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">inkBarrier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">紙壘</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用一整圈紙牆把自己包住 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒：期間刀槍不入、不受任何傷害，敵彈會被紙牆擋下。</t>
     </r>
   </si>
   <si>
@@ -22088,7 +22180,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -23532,17 +23624,17 @@
         <v>214</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="F31" s="12" t="s">
         <v>52</v>
       </c>
       <c r="G31" s="13"/>
       <c r="H31" s="13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I31" s="13" t="n">
         <v>0</v>
@@ -23579,14 +23671,14 @@
         <v>111</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>231</v>
+        <v>112</v>
       </c>
       <c r="F32" s="12" t="s">
         <v>52</v>
       </c>
       <c r="G32" s="13"/>
       <c r="H32" s="13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I32" s="13" t="n">
         <v>0</v>
@@ -23598,50 +23690,48 @@
         <v>2</v>
       </c>
       <c r="L32" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="O32" s="12" t="s">
         <v>87</v>
       </c>
       <c r="P32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>234</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>235</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>214</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>36</v>
+        <v>111</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>90</v>
+        <v>235</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>12</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G33" s="13"/>
       <c r="H33" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I33" s="13" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K33" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L33" s="14" t="s">
         <v>236</v>
@@ -23655,7 +23745,7 @@
       </c>
       <c r="P33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
         <v>238</v>
       </c>
@@ -23669,29 +23759,31 @@
         <v>36</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="G34" s="13"/>
+        <v>60</v>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>12</v>
+      </c>
       <c r="H34" s="13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I34" s="13" t="n">
         <v>0</v>
       </c>
       <c r="J34" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K34" s="13" t="n">
         <v>4</v>
-      </c>
-      <c r="K34" s="13" t="n">
-        <v>3</v>
       </c>
       <c r="L34" s="14" t="s">
         <v>240</v>
       </c>
       <c r="M34" s="13"/>
-      <c r="N34" s="11" t="s">
+      <c r="N34" s="12" t="s">
         <v>241</v>
       </c>
       <c r="O34" s="12" t="s">
@@ -23699,7 +23791,7 @@
       </c>
       <c r="P34" s="10"/>
     </row>
-    <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
         <v>242</v>
       </c>
@@ -23713,16 +23805,14 @@
         <v>36</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>244</v>
+        <v>37</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>22</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G35" s="13"/>
       <c r="H35" s="13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I35" s="13" t="n">
         <v>0</v>
@@ -23734,11 +23824,11 @@
         <v>3</v>
       </c>
       <c r="L35" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="M35" s="13"/>
+      <c r="N35" s="11" t="s">
         <v>245</v>
-      </c>
-      <c r="M35" s="13"/>
-      <c r="N35" s="12" t="s">
-        <v>246</v>
       </c>
       <c r="O35" s="12" t="s">
         <v>87</v>
@@ -23747,26 +23837,28 @@
     </row>
     <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="B36" s="12" t="s">
         <v>247</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>248</v>
       </c>
       <c r="C36" s="12" t="s">
         <v>214</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>111</v>
+        <v>36</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>112</v>
+        <v>248</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="G36" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>22</v>
+      </c>
       <c r="H36" s="13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I36" s="13" t="n">
         <v>0</v>
@@ -23778,29 +23870,29 @@
         <v>3</v>
       </c>
       <c r="L36" s="14" t="s">
-        <v>114</v>
+        <v>249</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O36" s="12" t="s">
         <v>87</v>
       </c>
       <c r="P36" s="10"/>
     </row>
-    <row r="37" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>214</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>36</v>
+        <v>111</v>
       </c>
       <c r="E37" s="12" t="s">
         <v>112</v>
@@ -23822,7 +23914,7 @@
         <v>3</v>
       </c>
       <c r="L37" s="14" t="s">
-        <v>252</v>
+        <v>114</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="12" t="s">
@@ -23833,8 +23925,52 @@
       </c>
       <c r="P37" s="10"/>
     </row>
+    <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G38" s="13"/>
+      <c r="H38" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I38" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K38" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L38" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="M38" s="13"/>
+      <c r="N38" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="O38" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="P38" s="10"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P37"/>
+  <autoFilter ref="A1:P38"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -23870,13 +24006,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="B1" s="15" t="n">
         <v>2.5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="D1" s="15" t="n">
         <v>2</v>
@@ -23893,40 +24029,40 @@
         <v>20</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>32</v>
@@ -23934,13 +24070,13 @@
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>38</v>
@@ -23962,7 +24098,7 @@
         <v>10</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>1</v>
@@ -23975,22 +24111,22 @@
         <v>1</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="P4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>274</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>275</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>270</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>52</v>
@@ -24023,22 +24159,22 @@
         <v>2</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="P5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>46</v>
@@ -24060,7 +24196,7 @@
         <v>8.5</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="K6" s="8" t="n">
         <v>1.5</v>
@@ -24073,22 +24209,22 @@
         <v>2</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="P6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="270.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>64</v>
@@ -24121,22 +24257,22 @@
         <v>2</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="P7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>44</v>
@@ -24165,22 +24301,22 @@
         <v>2</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="P8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>293</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>289</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>26</v>
@@ -24209,22 +24345,22 @@
         <v>1</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="P9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>58</v>
@@ -24246,7 +24382,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="K10" s="8" t="n">
         <v>1.5</v>
@@ -24259,22 +24395,22 @@
         <v>2</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="P10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>90</v>
@@ -24303,22 +24439,22 @@
         <v>2</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="P11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>14</v>
@@ -24348,25 +24484,25 @@
       </c>
       <c r="N12" s="7"/>
       <c r="O12" s="6" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="P12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>900</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F13" s="13" t="n">
         <v>0.8</v>
@@ -24385,32 +24521,32 @@
         <v>4</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="12" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="P13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="161.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>2.2</v>
@@ -24429,32 +24565,32 @@
         <v>4</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="12" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="O14" s="11" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="P14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1300</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>0</v>
@@ -24473,32 +24609,32 @@
         <v>4</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="12" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="O15" s="11" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="P15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="331.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1100</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>1.4</v>
@@ -24517,32 +24653,32 @@
         <v>4</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="12" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="O16" s="11" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="P16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="252.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1400</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>0</v>
@@ -24561,26 +24697,26 @@
         <v>5</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="12" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="O17" s="11" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="P17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>45</v>
@@ -24610,7 +24746,7 @@
       </c>
       <c r="N18" s="7"/>
       <c r="O18" s="6" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="P18" s="10"/>
     </row>
@@ -24660,37 +24796,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -24698,16 +24834,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -24742,16 +24878,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -24786,16 +24922,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -24826,22 +24962,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -24872,22 +25008,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -24905,10 +25041,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -24918,22 +25054,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -24945,10 +25081,10 @@
         <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -24964,7 +25100,7 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="O7" s="10"/>
     </row>
@@ -24996,19 +25132,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -25016,289 +25152,289 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -25333,13 +25469,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -25347,13 +25483,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -25363,13 +25499,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -25379,13 +25515,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -25395,13 +25531,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -25411,13 +25547,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -25427,13 +25563,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -25443,13 +25579,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -25459,13 +25595,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -25475,13 +25611,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -25491,13 +25627,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -25507,13 +25643,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -25523,13 +25659,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -25539,13 +25675,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -25555,13 +25691,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -25571,13 +25707,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -25587,13 +25723,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -25603,13 +25739,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -25619,13 +25755,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -25635,13 +25771,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>
@@ -25677,16 +25813,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -25694,13 +25830,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -25709,13 +25845,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -25724,13 +25860,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
@@ -25739,13 +25875,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -25754,13 +25890,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -25769,13 +25905,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -25784,13 +25920,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -25799,13 +25935,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -25814,13 +25950,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -25829,13 +25965,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -25844,13 +25980,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -25859,28 +25995,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2</v>
@@ -25889,28 +26025,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>2</v>
@@ -25919,13 +26055,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>1</v>
@@ -25934,13 +26070,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>1</v>
@@ -25949,13 +26085,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>10</v>
@@ -25964,13 +26100,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>100</v>
@@ -25979,13 +26115,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="D21" s="8" t="n">
         <v>200</v>
@@ -25994,13 +26130,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>1</v>
@@ -26009,13 +26145,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>30</v>
@@ -26024,13 +26160,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>5</v>
@@ -26039,13 +26175,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>10</v>
@@ -26054,13 +26190,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10</v>
@@ -26069,13 +26205,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5</v>
@@ -26084,13 +26220,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>10</v>
@@ -26099,13 +26235,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>25</v>
@@ -26114,13 +26250,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>10</v>
@@ -26129,13 +26265,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>100</v>
@@ -26144,13 +26280,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>1</v>
@@ -26159,13 +26295,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>10</v>
@@ -26174,13 +26310,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>1</v>
@@ -26189,13 +26325,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="D35" s="8" t="n">
         <v>10</v>
@@ -26204,13 +26340,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>4</v>
@@ -26219,13 +26355,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="D37" s="8" t="n">
         <v>1000</v>
@@ -26234,13 +26370,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="D38" s="8" t="n">
         <v>1</v>
@@ -26249,13 +26385,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="D39" s="8" t="n">
         <v>10</v>
@@ -26264,13 +26400,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>1</v>
@@ -26279,13 +26415,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>13</v>
@@ -26294,13 +26430,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>1</v>
@@ -26309,13 +26445,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="D43" s="8" t="n">
         <v>1000</v>
@@ -26324,13 +26460,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="D44" s="8" t="n">
         <v>5</v>
@@ -26339,13 +26475,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="D45" s="8" t="n">
         <v>25</v>
@@ -26354,13 +26490,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="D46" s="8" t="n">
         <v>10</v>
@@ -26369,13 +26505,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="D47" s="8" t="n">
         <v>3</v>
@@ -26384,13 +26520,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="D48" s="8" t="n">
         <v>10</v>
@@ -26424,16 +26560,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -26441,61 +26577,61 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="E2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="E3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="E4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="E5" s="10"/>
     </row>
@@ -26529,22 +26665,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -26552,115 +26688,115 @@
     </row>
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.9.50: math course numbers pairs 1-5; music course 5 rings, spawn near player away from foes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -20634,17 +20634,92 @@
     <t xml:space="preserve">數學課</t>
   </si>
   <si>
-    <t xml:space="preserve">照編號順序打！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">• 敵人有編號，紅色的先打
-• 沒輪到的敵人，傷害 −</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">照數字順序打，從 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">數到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">！</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• 每次隨機 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">隻敵人頭上標同一個數字，打倒其中一隻就換下 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">隻標下一個數字
+• 沒標數字的敵人，傷害 −</t>
     </r>
     <r>
       <rPr>
@@ -20663,7 +20738,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">• 依序連續擊倒 </t>
+      <t xml:space="preserve">• 打倒標著 </t>
     </r>
     <r>
       <rPr>
@@ -20680,7 +20755,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">隻（打錯歸零）</t>
+      <t xml:space="preserve">的敵人，再清掉剩下的敵人就開門</t>
     </r>
   </si>
   <si>
@@ -20768,7 +20843,67 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">5</t>
+      <t xml:space="preserve">5
+tags</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+extra</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+extraDelay</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
     </r>
   </si>
   <si>
@@ -21582,7 +21717,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3.2
+      <t xml:space="preserve">2.6
 first</t>
     </r>
     <r>
@@ -21602,7 +21737,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2
+      <t xml:space="preserve">1.6
 life</t>
     </r>
     <r>
@@ -21682,8 +21817,68 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">2.2
+rangeX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5
+rangeZ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.6
+foeGap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">3
-rangeX</t>
+tries</t>
     </r>
     <r>
       <rPr>
@@ -21702,8 +21897,8 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8
-rangeZ</t>
+      <t xml:space="preserve">32
+goal</t>
     </r>
     <r>
       <rPr>
@@ -21722,27 +21917,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4.5
-goal</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
+      <t xml:space="preserve">5</t>
     </r>
   </si>
   <si>
@@ -27032,7 +27207,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
         <v>604</v>
       </c>
@@ -27116,7 +27291,7 @@
       </c>
       <c r="G5" s="10"/>
     </row>
-    <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>628</v>
       </c>

</xml_diff>

<commit_message>
v0.9.54: tiered grouped achievements, clickable level chests, 8 new accessories, weapon list view, crayon odds, smoother sketch leap, shorter ball preview
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="684">
   <si>
     <r>
       <rPr>
@@ -13048,7 +13048,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">30%</t>
+      <t xml:space="preserve">40%</t>
     </r>
     <r>
       <rPr>
@@ -13082,7 +13082,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">50%</t>
+      <t xml:space="preserve">40%</t>
     </r>
     <r>
       <rPr>
@@ -20572,22 +20572,1121 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">清潔工</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1000</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">菁英剋星</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個菁英敵人</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">首領退散</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗第一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">首領獵人</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊敗 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個首領</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">全員到齊</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗全部 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種首領</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">完美答卷</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷擊敗一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">一塵不染</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">無傷清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">千鈞一髮</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命時清除一頁</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">擦身而過</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">閃身步</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">一支穿雲劍</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">石油大亨</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個油桶</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">裡面是什麼？</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個箱子</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">易燃易爆炸</t>
+  </si>
+  <si>
+    <t xml:space="preserve">被油桶炸死一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">搖頭晃腦</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">連續原地旋轉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">圈（中間可停一下）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">出牌手感</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計使用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張卡牌</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1000</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">合而為一</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合成升級卡牌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">大招成癮</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計施放 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次大招卡</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">第一頁</t>
   </si>
   <si>
     <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
   </si>
   <si>
-    <t xml:space="preserve">擦身而過</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">衝刺閃過攻擊 </t>
+    <t xml:space="preserve">翻頁不停</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">寫完了！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完成整本筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">寫不完</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式抵達第 </t>
     </r>
     <r>
       <rPr>
@@ -20604,146 +21703,236 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">頁</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">課間高手</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">贏得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">場事件小遊戲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">熟客</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在商店購買 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">次</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">清潔工</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊倒 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">出牌手感</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計使用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">張卡牌</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">首領退散</t>
-  </si>
-  <si>
-    <t xml:space="preserve">擊敗第一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">翻頁不停</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">合而為一</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">合成升級卡牌 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">課間高手</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">贏得 </t>
+    <t xml:space="preserve">小有名氣</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「十」分完美</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">墨跡未乾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">用金幣復活一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">穿搭達人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">儲存一套自訂套組</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣櫃擴充</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">收集 </t>
     </r>
     <r>
       <rPr>
@@ -20760,378 +21949,88 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">場事件小遊戲</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">熟客</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在商店購買 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">小有名氣</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
+      <t xml:space="preserve">個新顏色或配飾</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">文具控</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種不同武器完成冒險</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">5</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">菁英剋星</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊倒 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個菁英敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">大招成癮</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計施放 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次大招卡</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">一塵不染</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">無傷清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">殘影</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">千鈞一髮</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">只剩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點生命時清除一頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">寫不完</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">課表模式抵達第 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">穿搭達人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">儲存一套自訂套組</t>
-  </si>
-  <si>
-    <t xml:space="preserve">衣櫃擴充</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">收集 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個新顏色或配飾</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">文具控</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種不同武器完成冒險</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">墨海</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊倒 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1000 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">寫完了！</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完成整本筆記本</t>
-  </si>
-  <si>
-    <t xml:space="preserve">首領獵人</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊敗 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個首領</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">完美答卷</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷擊敗一個首領</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">博物誌</t>
@@ -21164,317 +22063,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">墨跡未乾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">用金幣復活一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">牌桌老手</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計使用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1000 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">張卡牌</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">全員到齊</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗全部 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種首領</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">永無止境</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">課表模式抵達第 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「十」分完美</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">三本筆記</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">完成整本筆記本 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">搖頭晃腦</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">連續原地旋轉 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">圈（中間可停一下）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">石油大亨</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個油桶</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">裡面是什麼？</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個箱子</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">易燃易爆炸</t>
-  </si>
-  <si>
-    <t xml:space="preserve">被油桶炸死一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一支穿雲劍</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">閃身步</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
+    <t xml:space="preserve">13</t>
   </si>
   <si>
     <t xml:space="preserve">遺物</t>
@@ -27784,7 +28373,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -28118,7 +28707,7 @@
       </c>
       <c r="E22" s="10"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>553</v>
       </c>
@@ -28128,8 +28717,8 @@
       <c r="C23" s="7" t="s">
         <v>555</v>
       </c>
-      <c r="D23" s="8" t="n">
-        <v>1</v>
+      <c r="D23" s="8" t="s">
+        <v>556</v>
       </c>
       <c r="E23" s="10"/>
     </row>
@@ -28138,13 +28727,13 @@
         <v>553</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>557</v>
-      </c>
-      <c r="D24" s="8" t="n">
-        <v>10</v>
+        <v>558</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>559</v>
       </c>
       <c r="E24" s="10"/>
     </row>
@@ -28153,13 +28742,13 @@
         <v>553</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>559</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <v>100</v>
+        <v>561</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E25" s="10"/>
     </row>
@@ -28168,13 +28757,13 @@
         <v>553</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>561</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <v>200</v>
+        <v>564</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>565</v>
       </c>
       <c r="E26" s="10"/>
     </row>
@@ -28183,13 +28772,13 @@
         <v>553</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>563</v>
-      </c>
-      <c r="D27" s="8" t="n">
-        <v>1</v>
+        <v>567</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>568</v>
       </c>
       <c r="E27" s="10"/>
     </row>
@@ -28198,13 +28787,13 @@
         <v>553</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>565</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>30</v>
+        <v>570</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E28" s="10"/>
     </row>
@@ -28213,13 +28802,13 @@
         <v>553</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>567</v>
-      </c>
-      <c r="D29" s="8" t="n">
-        <v>20</v>
+        <v>572</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>573</v>
       </c>
       <c r="E29" s="10"/>
     </row>
@@ -28228,13 +28817,13 @@
         <v>553</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>569</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>10</v>
+        <v>575</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E30" s="10"/>
     </row>
@@ -28243,13 +28832,13 @@
         <v>553</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>571</v>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>10</v>
+        <v>577</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>578</v>
       </c>
       <c r="E31" s="10"/>
     </row>
@@ -28258,13 +28847,13 @@
         <v>553</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>572</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>573</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>5</v>
+        <v>579</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>581</v>
       </c>
       <c r="E32" s="10"/>
     </row>
@@ -28273,13 +28862,13 @@
         <v>553</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>574</v>
+        <v>582</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>575</v>
-      </c>
-      <c r="D33" s="8" t="n">
-        <v>10</v>
+        <v>583</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>581</v>
       </c>
       <c r="E33" s="10"/>
     </row>
@@ -28288,13 +28877,13 @@
         <v>553</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>576</v>
+        <v>584</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>577</v>
-      </c>
-      <c r="D34" s="8" t="n">
-        <v>50</v>
+        <v>585</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>586</v>
       </c>
       <c r="E34" s="10"/>
     </row>
@@ -28303,13 +28892,13 @@
         <v>553</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>578</v>
+        <v>587</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>579</v>
-      </c>
-      <c r="D35" s="8" t="n">
-        <v>10</v>
+        <v>588</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>586</v>
       </c>
       <c r="E35" s="10"/>
     </row>
@@ -28318,13 +28907,13 @@
         <v>553</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>580</v>
+        <v>589</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>581</v>
-      </c>
-      <c r="D36" s="8" t="n">
-        <v>100</v>
+        <v>590</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E36" s="10"/>
     </row>
@@ -28333,28 +28922,28 @@
         <v>553</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>582</v>
+        <v>591</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>583</v>
-      </c>
-      <c r="D37" s="8" t="n">
-        <v>1</v>
+        <v>592</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>593</v>
       </c>
       <c r="E37" s="10"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>553</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>584</v>
+        <v>594</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>585</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>10</v>
+        <v>595</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>596</v>
       </c>
       <c r="E38" s="10"/>
     </row>
@@ -28363,13 +28952,13 @@
         <v>553</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>587</v>
-      </c>
-      <c r="D39" s="8" t="n">
-        <v>1</v>
+        <v>598</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>599</v>
       </c>
       <c r="E39" s="10"/>
     </row>
@@ -28378,13 +28967,13 @@
         <v>553</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>589</v>
-      </c>
-      <c r="D40" s="8" t="n">
-        <v>10</v>
+        <v>601</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>602</v>
       </c>
       <c r="E40" s="10"/>
     </row>
@@ -28393,13 +28982,13 @@
         <v>553</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>590</v>
+        <v>603</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>591</v>
-      </c>
-      <c r="D41" s="8" t="n">
-        <v>4</v>
+        <v>604</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E41" s="10"/>
     </row>
@@ -28408,13 +28997,13 @@
         <v>553</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>592</v>
+        <v>605</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>593</v>
-      </c>
-      <c r="D42" s="8" t="n">
-        <v>1000</v>
+        <v>606</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>607</v>
       </c>
       <c r="E42" s="10"/>
     </row>
@@ -28423,13 +29012,13 @@
         <v>553</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>594</v>
+        <v>608</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>595</v>
-      </c>
-      <c r="D43" s="8" t="n">
-        <v>1</v>
+        <v>609</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>610</v>
       </c>
       <c r="E43" s="10"/>
     </row>
@@ -28438,13 +29027,13 @@
         <v>553</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>597</v>
-      </c>
-      <c r="D44" s="8" t="n">
-        <v>20</v>
+        <v>612</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>613</v>
       </c>
       <c r="E44" s="10"/>
     </row>
@@ -28453,13 +29042,13 @@
         <v>553</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>598</v>
+        <v>614</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>599</v>
-      </c>
-      <c r="D45" s="8" t="n">
-        <v>1</v>
+        <v>615</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>616</v>
       </c>
       <c r="E45" s="10"/>
     </row>
@@ -28468,13 +29057,13 @@
         <v>553</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>600</v>
+        <v>617</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>601</v>
-      </c>
-      <c r="D46" s="8" t="n">
-        <v>13</v>
+        <v>618</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>573</v>
       </c>
       <c r="E46" s="10"/>
     </row>
@@ -28483,13 +29072,13 @@
         <v>553</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>602</v>
+        <v>619</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>603</v>
-      </c>
-      <c r="D47" s="8" t="n">
-        <v>1</v>
+        <v>620</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>568</v>
       </c>
       <c r="E47" s="10"/>
     </row>
@@ -28498,13 +29087,13 @@
         <v>553</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>604</v>
+        <v>621</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>605</v>
-      </c>
-      <c r="D48" s="8" t="n">
-        <v>1000</v>
+        <v>622</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>593</v>
       </c>
       <c r="E48" s="10"/>
     </row>
@@ -28513,13 +29102,13 @@
         <v>553</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>606</v>
+        <v>623</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>607</v>
-      </c>
-      <c r="D49" s="8" t="n">
-        <v>5</v>
+        <v>624</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E49" s="10"/>
     </row>
@@ -28528,13 +29117,13 @@
         <v>553</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>608</v>
+        <v>625</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>609</v>
-      </c>
-      <c r="D50" s="8" t="n">
-        <v>25</v>
+        <v>626</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>562</v>
       </c>
       <c r="E50" s="10"/>
     </row>
@@ -28543,13 +29132,13 @@
         <v>553</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>610</v>
+        <v>627</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>611</v>
-      </c>
-      <c r="D51" s="8" t="n">
-        <v>10</v>
+        <v>628</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>573</v>
       </c>
       <c r="E51" s="10"/>
     </row>
@@ -28558,13 +29147,13 @@
         <v>553</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>612</v>
+        <v>629</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>613</v>
-      </c>
-      <c r="D52" s="8" t="n">
-        <v>3</v>
+        <v>630</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>631</v>
       </c>
       <c r="E52" s="10"/>
     </row>
@@ -28573,90 +29162,15 @@
         <v>553</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>614</v>
+        <v>632</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>615</v>
-      </c>
-      <c r="D53" s="8" t="n">
-        <v>10</v>
+        <v>633</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>634</v>
       </c>
       <c r="E53" s="10"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
-        <v>553</v>
-      </c>
-      <c r="B54" s="7" t="s">
-        <v>616</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>617</v>
-      </c>
-      <c r="D54" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E54" s="10"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7" t="s">
-        <v>553</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>618</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>619</v>
-      </c>
-      <c r="D55" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="E55" s="10"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
-        <v>553</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>620</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>621</v>
-      </c>
-      <c r="D56" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="10"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7" t="s">
-        <v>553</v>
-      </c>
-      <c r="B57" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>623</v>
-      </c>
-      <c r="D57" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E57" s="10"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
-        <v>553</v>
-      </c>
-      <c r="B58" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="D58" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E58" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -28685,16 +29199,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>626</v>
+        <v>635</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>483</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>627</v>
+        <v>636</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>628</v>
+        <v>637</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -28702,31 +29216,31 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>629</v>
+        <v>638</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>630</v>
+        <v>639</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>631</v>
+        <v>640</v>
       </c>
       <c r="E2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>632</v>
+        <v>641</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>633</v>
+        <v>642</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>634</v>
+        <v>643</v>
       </c>
       <c r="E3" s="10"/>
     </row>
@@ -28735,28 +29249,28 @@
         <v>430</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>635</v>
+        <v>644</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>636</v>
+        <v>645</v>
       </c>
       <c r="E4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>637</v>
+        <v>646</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>638</v>
+        <v>647</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>639</v>
+        <v>648</v>
       </c>
       <c r="E5" s="10"/>
     </row>
@@ -28790,7 +29304,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>640</v>
+        <v>649</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>507</v>
@@ -28799,13 +29313,13 @@
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>641</v>
+        <v>650</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>642</v>
+        <v>651</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>628</v>
+        <v>637</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -28813,115 +29327,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>643</v>
+        <v>652</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>644</v>
+        <v>653</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>645</v>
+        <v>654</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>646</v>
+        <v>655</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>647</v>
+        <v>656</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>648</v>
+        <v>657</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>649</v>
+        <v>658</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>650</v>
+        <v>659</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>651</v>
+        <v>660</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>652</v>
+        <v>661</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>653</v>
+        <v>662</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>654</v>
+        <v>663</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>655</v>
+        <v>664</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>656</v>
+        <v>665</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>657</v>
+        <v>666</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>658</v>
+        <v>667</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>659</v>
+        <v>668</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>660</v>
+        <v>669</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>661</v>
+        <v>670</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>662</v>
+        <v>671</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>663</v>
+        <v>672</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>664</v>
+        <v>673</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>665</v>
+        <v>674</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>666</v>
+        <v>675</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>667</v>
+        <v>676</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>668</v>
+        <v>677</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>669</v>
+        <v>678</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>670</v>
+        <v>679</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>671</v>
+        <v>680</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>672</v>
+        <v>681</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>673</v>
+        <v>682</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>674</v>
+        <v>683</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.9.56: in-run relics from a post-boss library, 18 new relics, relic capsule machine, S+ grade and grade coins, weapons merged into look editor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="757">
   <si>
     <r>
       <rPr>
@@ -20545,6 +20545,419 @@
     <t xml:space="preserve">等級寶箱：配飾</t>
   </si>
   <si>
+    <t xml:space="preserve">評分</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分數門檻（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">級結算獎勵 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分數門檻（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">級結算獎勵 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分數門檻（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">級結算獎勵 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分數門檻（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">級結算獎勵 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分數門檻（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">級結算獎勵 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">C</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -22069,7 +22482,10 @@
     <t xml:space="preserve">遺物</t>
   </si>
   <si>
-    <t xml:space="preserve">價格（墨點）</t>
+    <t xml:space="preserve">初始解鎖</t>
+  </si>
+  <si>
+    <t xml:space="preserve">扭蛋價格（金幣）</t>
   </si>
   <si>
     <t xml:space="preserve">參數</t>
@@ -22188,6 +22604,9 @@
       </rPr>
       <t xml:space="preserve">（圓規沒有彈匣，不受影響）。</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">★</t>
   </si>
   <si>
     <r>
@@ -22308,6 +22727,194 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">換彈時間縮短 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">reload</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.9</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">小墨水瓶</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每進入新的一頁，如果墨水不到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點，直接補到 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">min</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">止血貼</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">受傷後的無敵時間延長 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">invuln</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">立可白</t>
   </si>
   <si>
@@ -22360,13 +22967,558 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">換彈時間縮短 </t>
+    <t xml:space="preserve">急救貼布</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每通關 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁，回復 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回復：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">間隔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">運動鞋</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">閃避的無敵時間延長 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">iframe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">輕羽毛</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">移動速度提升 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">速度：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.06</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">橡皮屑</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每擊倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">隻敵人（小墨團不算）獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點墨水，計數會跨頁累積。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">間隔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">捲筆刀</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">離目標 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">公尺內時，武器傷害提升 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">距離：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">眼鏡</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">敵人與頭目攻擊前的紅色預警圈、預警線持續時間延長 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">減速：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.25</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">折價券</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">商店所有商品價格降低 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.85</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">完美節拍</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完美閃避後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內，射速提升 </t>
     </r>
     <r>
       <rPr>
@@ -22394,7 +23546,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">reload</t>
+      <t xml:space="preserve">time</t>
     </r>
     <r>
       <rPr>
@@ -22411,20 +23563,355 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.88</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">急救貼布</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">每擊敗一隻頭目，回復 </t>
+      <t xml:space="preserve">2
+rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.12</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">紅墨水契約</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">生命上限 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，但武器與卡牌傷害提升 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">耐久：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">複寫紙</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每使用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張一般卡（大招不算），下一張一般卡免費。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">間隔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">浴血重生</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">生命歸零時以 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命復活，並獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒無敵。每局一次，和金幣復活分開計算。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">耐久：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+invuln</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">大墨水瓶</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水上限 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">墨水滴漏</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">戰鬥中每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒獲得 </t>
     </r>
     <r>
       <rPr>
@@ -22441,17 +23928,56 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">點生命。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">回復：</t>
+      <t xml:space="preserve">點墨水（暫停與大招動畫時不計時）。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">護身紙</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">進入菁英頁與頭目頁時，獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">層紙盾。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">shields</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
     </r>
     <r>
       <rPr>
@@ -22461,6 +23987,321 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">背水一戰</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">生命 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點以下時，射速與移動速度提升 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">耐久：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">速度：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">賭徒心態</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在事件小遊戲、奇遇、休息區與寶箱頁，獲得的分數與回血 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，失去的分數與受到的傷害也 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（其他遺物造成的變化不算）。只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命時，加倍的傷害不會致死。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">受虐傾向</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每次被攻擊時獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點墨水（被紙盾、堡壘、立可白或其他遺物擋下也算）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">（取得方式）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每次擊敗頭目後進入圖書館，從已解鎖的遺物中隨機出 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件，免費選 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件；最多帶 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件，超過要丟棄 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件。</t>
     </r>
   </si>
   <si>
@@ -28373,7 +30214,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -28441,7 +30282,7 @@
         <v>515</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E4" s="10"/>
     </row>
@@ -28707,7 +30548,7 @@
       </c>
       <c r="E22" s="10"/>
     </row>
-    <row r="23" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>553</v>
       </c>
@@ -28717,8 +30558,8 @@
       <c r="C23" s="7" t="s">
         <v>555</v>
       </c>
-      <c r="D23" s="8" t="s">
-        <v>556</v>
+      <c r="D23" s="8" t="n">
+        <v>45000</v>
       </c>
       <c r="E23" s="10"/>
     </row>
@@ -28727,13 +30568,13 @@
         <v>553</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>556</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>557</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>558</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>559</v>
+      <c r="D24" s="8" t="n">
+        <v>35000</v>
       </c>
       <c r="E24" s="10"/>
     </row>
@@ -28742,13 +30583,13 @@
         <v>553</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>561</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>562</v>
+        <v>559</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>20000</v>
       </c>
       <c r="E25" s="10"/>
     </row>
@@ -28757,13 +30598,13 @@
         <v>553</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>564</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>565</v>
+        <v>561</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>10000</v>
       </c>
       <c r="E26" s="10"/>
     </row>
@@ -28772,13 +30613,13 @@
         <v>553</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>567</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>568</v>
+        <v>563</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>5000</v>
       </c>
       <c r="E27" s="10"/>
     </row>
@@ -28787,13 +30628,13 @@
         <v>553</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>570</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>562</v>
+        <v>555</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>80000</v>
       </c>
       <c r="E28" s="10"/>
     </row>
@@ -28802,13 +30643,13 @@
         <v>553</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>572</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>573</v>
+        <v>557</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>60000</v>
       </c>
       <c r="E29" s="10"/>
     </row>
@@ -28817,13 +30658,13 @@
         <v>553</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>574</v>
+        <v>566</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>575</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>562</v>
+        <v>559</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>30000</v>
       </c>
       <c r="E30" s="10"/>
     </row>
@@ -28832,13 +30673,13 @@
         <v>553</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>577</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>578</v>
+        <v>561</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>15000</v>
       </c>
       <c r="E31" s="10"/>
     </row>
@@ -28847,330 +30688,480 @@
         <v>553</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>579</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>580</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>581</v>
+        <v>568</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>563</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>5000</v>
       </c>
       <c r="E32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>582</v>
+        <v>570</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>583</v>
+        <v>571</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>581</v>
+        <v>572</v>
       </c>
       <c r="E33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>584</v>
+        <v>573</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>585</v>
+        <v>574</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>586</v>
+        <v>575</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>587</v>
+        <v>576</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>588</v>
+        <v>577</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>562</v>
+        <v>581</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>591</v>
+        <v>582</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>592</v>
+        <v>583</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>593</v>
+        <v>584</v>
       </c>
       <c r="E37" s="10"/>
     </row>
-    <row r="38" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>594</v>
+        <v>585</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>595</v>
+        <v>586</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>596</v>
+        <v>578</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>597</v>
+        <v>587</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>602</v>
+        <v>578</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>603</v>
+        <v>592</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>604</v>
+        <v>593</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>562</v>
+        <v>594</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>605</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>606</v>
+        <v>595</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>596</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>608</v>
+        <v>598</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>609</v>
+        <v>599</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>610</v>
+        <v>597</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>612</v>
+        <v>601</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>613</v>
+        <v>602</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>614</v>
+        <v>603</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>615</v>
+        <v>604</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>616</v>
+        <v>602</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>568</v>
+        <v>609</v>
       </c>
       <c r="E47" s="10"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>621</v>
+        <v>610</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>622</v>
+        <v>611</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>623</v>
+        <v>613</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>624</v>
+        <v>614</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>562</v>
+        <v>615</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>562</v>
+        <v>618</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>627</v>
+        <v>619</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>628</v>
+        <v>620</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>629</v>
+        <v>621</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>630</v>
+        <v>622</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>631</v>
+        <v>623</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>553</v>
+        <v>569</v>
       </c>
       <c r="B53" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>626</v>
+      </c>
+      <c r="E53" s="10"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>628</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>629</v>
+      </c>
+      <c r="E54" s="10"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="D55" s="8" t="s">
         <v>632</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="E55" s="10"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B56" s="7" t="s">
         <v>633</v>
       </c>
-      <c r="D53" s="8" t="s">
+      <c r="C56" s="7" t="s">
         <v>634</v>
       </c>
-      <c r="E53" s="10"/>
+      <c r="D56" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="E56" s="10"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>584</v>
+      </c>
+      <c r="E57" s="10"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>638</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>609</v>
+      </c>
+      <c r="E58" s="10"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="E59" s="10"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="D60" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="E60" s="10"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>643</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="D61" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="E61" s="10"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>645</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>647</v>
+      </c>
+      <c r="E62" s="10"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="D63" s="8" t="s">
+        <v>650</v>
+      </c>
+      <c r="E63" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -29188,91 +31179,409 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>635</v>
+        <v>651</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>483</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>636</v>
+        <v>652</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>637</v>
+        <v>653</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>638</v>
+        <v>655</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>639</v>
-      </c>
-      <c r="C2" s="8" t="n">
+        <v>656</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>640</v>
-      </c>
-      <c r="E2" s="10"/>
+      <c r="E2" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="F2" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>641</v>
+        <v>430</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>642</v>
-      </c>
-      <c r="C3" s="8" t="n">
+        <v>659</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>643</v>
-      </c>
-      <c r="E3" s="10"/>
+      <c r="E3" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>430</v>
+        <v>661</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>644</v>
-      </c>
-      <c r="C4" s="8" t="n">
+        <v>662</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>645</v>
-      </c>
-      <c r="E4" s="10"/>
+      <c r="E4" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>646</v>
+        <v>664</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>647</v>
-      </c>
-      <c r="C5" s="8" t="n">
+        <v>665</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>648</v>
-      </c>
-      <c r="E5" s="10"/>
+      <c r="E5" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="F5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>667</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>668</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="F6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>672</v>
+      </c>
+      <c r="F7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="F8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>676</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="F9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>680</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>681</v>
+      </c>
+      <c r="F10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="C11" s="7"/>
+      <c r="D11" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="F11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="C12" s="7"/>
+      <c r="D12" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="F12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>689</v>
+      </c>
+      <c r="C13" s="7"/>
+      <c r="D13" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="F13" s="10"/>
+    </row>
+    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>691</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>692</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="F14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>694</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="F15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>697</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="F16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>701</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>702</v>
+      </c>
+      <c r="F17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>703</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>705</v>
+      </c>
+      <c r="F18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>681</v>
+      </c>
+      <c r="F19" s="10"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="C20" s="7"/>
+      <c r="D20" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>710</v>
+      </c>
+      <c r="F20" s="10"/>
+    </row>
+    <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>711</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>712</v>
+      </c>
+      <c r="C21" s="7"/>
+      <c r="D21" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>713</v>
+      </c>
+      <c r="F21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>714</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>715</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="F22" s="10"/>
+    </row>
+    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>718</v>
+      </c>
+      <c r="C23" s="7"/>
+      <c r="D23" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="F23" s="10"/>
+    </row>
+    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E24" s="7"/>
+      <c r="F24" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -29304,7 +31613,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>649</v>
+        <v>722</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>507</v>
@@ -29313,13 +31622,13 @@
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>650</v>
+        <v>723</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>651</v>
+        <v>724</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>637</v>
+        <v>654</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -29327,115 +31636,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>652</v>
+        <v>725</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>653</v>
+        <v>726</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>654</v>
+        <v>727</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>655</v>
+        <v>728</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>656</v>
+        <v>729</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>657</v>
+        <v>730</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>658</v>
+        <v>731</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>659</v>
+        <v>732</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>660</v>
+        <v>733</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>661</v>
+        <v>734</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>662</v>
+        <v>735</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>663</v>
+        <v>736</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>664</v>
+        <v>737</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>665</v>
+        <v>738</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>666</v>
+        <v>739</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>667</v>
+        <v>740</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>668</v>
+        <v>741</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>669</v>
+        <v>742</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>670</v>
+        <v>743</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>671</v>
+        <v>744</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>672</v>
+        <v>745</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>673</v>
+        <v>746</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>674</v>
+        <v>747</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>675</v>
+        <v>748</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>676</v>
+        <v>749</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>677</v>
+        <v>750</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>678</v>
+        <v>751</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>679</v>
+        <v>752</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>680</v>
+        <v>753</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>681</v>
+        <v>754</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>682</v>
+        <v>755</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>683</v>
+        <v>756</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.10.06: three gacha achievements with capsule icon, animated dashed relic selection box
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1069" uniqueCount="765">
   <si>
     <r>
       <rPr>
@@ -22443,6 +22443,172 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">扭轉乾坤</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用遺物扭蛋機抽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">蛋定蛋定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">抽扭蛋把金幣花到一枚不剩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">遺物所有</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">解鎖 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件遺物</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22</t>
     </r>
   </si>
   <si>
@@ -30214,7 +30380,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -31162,6 +31328,51 @@
         <v>650</v>
       </c>
       <c r="E63" s="10"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>578</v>
+      </c>
+      <c r="E64" s="10"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>655</v>
+      </c>
+      <c r="E65" s="10"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="E66" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -31191,19 +31402,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>483</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -31211,19 +31422,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -31232,349 +31443,349 @@
         <v>430</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>665</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>657</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>717</v>
+        <v>725</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -31613,7 +31824,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>507</v>
@@ -31622,13 +31833,13 @@
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -31636,115 +31847,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>736</v>
+        <v>744</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>737</v>
+        <v>745</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>738</v>
+        <v>746</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>746</v>
+        <v>754</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>748</v>
+        <v>756</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>750</v>
+        <v>758</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>752</v>
+        <v>760</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>753</v>
+        <v>761</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>754</v>
+        <v>762</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>755</v>
+        <v>763</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>756</v>
+        <v>764</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.10.11: Simon Says minigame, scrollable training minigame chooser, single next-act library door
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1069" uniqueCount="765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="770">
   <si>
     <r>
       <rPr>
@@ -19899,6 +19899,1846 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">teacher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">老師說</t>
+  </si>
+  <si>
+    <t xml:space="preserve">老師</t>
+  </si>
+  <si>
+    <t xml:space="preserve">只有「老師說」開頭的指令才要照做，沒有說就站著別動！先站進中間的圈圈等指令：向左、向右就跑進那邊的圈圈，衝刺就按空白鍵或右鍵。</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">指令數：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">假指令機率：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">假指令最多連續：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">開頭必為真指令數：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">可失誤次數：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">真指令時限</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">先左後右時限</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.6
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">假指令需站住</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">間距：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.8
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">間隔隨機加成</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">連續指令機率：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">反向箭頭機率：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">近似開頭機率：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">總時間保險</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">56</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">中間圈位置：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[0, 2.6]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">中間圈半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">假指令離開判定半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">站穩速度上限：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">站穩時間</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">左右圈</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(x,z,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">半徑</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'x': 5, 'z': 0.6, 'r': 1.3}
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">紅叉顯示</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.9
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">對話框時間</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.6</t>
     </r>
   </si>
   <si>
@@ -29699,7 +31539,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -30016,6 +31856,24 @@
         <v>481</v>
       </c>
       <c r="F17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="297" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>485</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="F18" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -30048,13 +31906,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -30062,13 +31920,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -30078,13 +31936,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -30094,13 +31952,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -30110,13 +31968,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -30126,13 +31984,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -30142,13 +32000,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -30158,13 +32016,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -30174,13 +32032,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -30190,13 +32048,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -30206,13 +32064,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -30222,13 +32080,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -30238,13 +32096,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -30254,13 +32112,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -30270,13 +32128,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -30286,13 +32144,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -30302,13 +32160,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -30318,13 +32176,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -30334,13 +32192,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -30350,13 +32208,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>
@@ -30392,16 +32250,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -30409,13 +32267,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -30424,13 +32282,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -30439,13 +32297,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>25</v>
@@ -30454,13 +32312,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -30469,13 +32327,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -30484,13 +32342,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -30499,13 +32357,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -30514,13 +32372,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -30529,13 +32387,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -30544,13 +32402,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -30559,13 +32417,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -30574,28 +32432,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2</v>
@@ -30604,28 +32462,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>2</v>
@@ -30634,13 +32492,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>1</v>
@@ -30649,10 +32507,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
@@ -30662,13 +32520,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>5</v>
@@ -30677,10 +32535,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
@@ -30690,10 +32548,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -30703,10 +32561,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
@@ -30716,13 +32574,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>45000</v>
@@ -30731,13 +32589,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>35000</v>
@@ -30746,13 +32604,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>20000</v>
@@ -30761,13 +32619,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10000</v>
@@ -30776,13 +32634,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5000</v>
@@ -30791,13 +32649,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>80000</v>
@@ -30806,13 +32664,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>60000</v>
@@ -30821,13 +32679,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>30000</v>
@@ -30836,13 +32694,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>15000</v>
@@ -30851,13 +32709,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>568</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>563</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>5000</v>
@@ -30866,511 +32724,511 @@
     </row>
     <row r="33" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="E33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="E66" s="10"/>
     </row>
@@ -31402,19 +33260,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -31422,19 +33280,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -31443,349 +33301,349 @@
         <v>430</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>675</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>670</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>665</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>709</v>
+        <v>714</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -31824,22 +33682,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -31847,115 +33705,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>747</v>
+        <v>752</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.10.12: Inner Clock minigame, training settings home button, single minigame door in training
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="770">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="775">
   <si>
     <r>
       <rPr>
@@ -21739,6 +21739,597 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.6</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">心中有數</t>
+  </si>
+  <si>
+    <t xml:space="preserve">沙漏</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">我會告訴你一個秒數。倒數 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">之後碼錶開始跑，跑沒幾秒螢幕就會暗掉，你得在心裡默數，覺得時間到了就按互動鍵停下碼錶！誤差 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內算完美，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內也算過關。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒數範圍</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">整數</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[6, 11]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倒數秒數：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">開始變暗</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[3, 4]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">變暗過程</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完美誤差</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">過關誤差</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">超時判定</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">結果展示</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.6
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">碼錶位置：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[0, -1.2]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">玩家距碼錶：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">碼錶半徑：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.75</t>
     </r>
   </si>
   <si>
@@ -31539,7 +32130,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -31874,6 +32465,24 @@
         <v>486</v>
       </c>
       <c r="F18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>488</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>489</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>490</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="F19" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -31906,13 +32515,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -31920,13 +32529,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -31936,13 +32545,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -31952,13 +32561,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -31968,13 +32577,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -31984,13 +32593,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -32000,13 +32609,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -32016,13 +32625,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -32032,13 +32641,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -32048,13 +32657,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -32064,13 +32673,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -32080,13 +32689,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -32096,13 +32705,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -32112,13 +32721,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -32128,13 +32737,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -32144,13 +32753,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -32160,13 +32769,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -32176,13 +32785,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -32192,13 +32801,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -32208,13 +32817,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>
@@ -32250,16 +32859,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -32267,13 +32876,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -32282,13 +32891,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -32297,13 +32906,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>25</v>
@@ -32312,13 +32921,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -32327,13 +32936,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -32342,13 +32951,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -32357,13 +32966,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -32372,13 +32981,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -32387,13 +32996,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -32402,13 +33011,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -32417,13 +33026,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>536</v>
+        <v>541</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -32432,28 +33041,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2</v>
@@ -32462,28 +33071,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>2</v>
@@ -32492,13 +33101,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>1</v>
@@ -32507,10 +33116,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
@@ -32520,13 +33129,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>5</v>
@@ -32535,10 +33144,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
@@ -32548,10 +33157,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -32561,10 +33170,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
@@ -32574,13 +33183,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>45000</v>
@@ -32589,13 +33198,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>35000</v>
@@ -32604,13 +33213,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>20000</v>
@@ -32619,13 +33228,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10000</v>
@@ -32634,13 +33243,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5000</v>
@@ -32649,13 +33258,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>80000</v>
@@ -32664,13 +33273,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>60000</v>
@@ -32679,13 +33288,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>30000</v>
@@ -32694,13 +33303,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>15000</v>
@@ -32709,13 +33318,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>573</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>568</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>5000</v>
@@ -32724,511 +33333,511 @@
     </row>
     <row r="33" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>575</v>
+        <v>580</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="E33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>574</v>
+        <v>579</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="E66" s="10"/>
     </row>
@@ -33260,19 +33869,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -33280,19 +33889,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -33301,349 +33910,349 @@
         <v>430</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>680</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>675</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>670</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>709</v>
+        <v>714</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -33682,22 +34291,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -33705,115 +34314,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>747</v>
+        <v>752</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.10.13: perfect count bonus reward, solid stopwatch, clearer Simon Says decoys and feedback, version on rotate screen, harder pun-named achievements
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="773">
   <si>
     <r>
       <rPr>
@@ -20065,7 +20065,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.3</t>
+      <t xml:space="preserve">0.5</t>
     </r>
     <r>
       <rPr>
@@ -20103,7 +20103,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.35</t>
+      <t xml:space="preserve">0.55</t>
     </r>
     <r>
       <rPr>
@@ -20141,7 +20141,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.4
+      <t xml:space="preserve">0.6
 </t>
     </r>
     <r>
@@ -20181,6 +20181,121 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">可失誤次數：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">2
 </t>
     </r>
@@ -20191,121 +20306,6 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">可失誤次數：第</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">幕 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／第</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">幕 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／第</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">幕 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">真指令時限</t>
     </r>
     <r>
@@ -21197,6 +21197,121 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">0.6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.8
+nearHard</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">幕 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">0</t>
     </r>
     <r>
@@ -21235,7 +21350,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0</t>
+      <t xml:space="preserve">0.4</t>
     </r>
     <r>
       <rPr>
@@ -21273,7 +21388,47 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.5
+      <t xml:space="preserve">0.6
+nearEasyKeys</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1, 2, 3, 4]
+nearHardKeys</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[5, 6, 7, 8]
 </t>
     </r>
     <r>
@@ -21680,7 +21835,67 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.9
+      <t xml:space="preserve">1
+markSize</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.4
+flashTime</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.8
+wrongShake</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35
 </t>
     </r>
     <r>
@@ -21825,16 +22040,16 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒內算完美，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">0.5 </t>
+      <t xml:space="preserve">秒內算完美（多拿一項獎勵），</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6 </t>
     </r>
     <r>
       <rPr>
@@ -22153,7 +22368,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.5
+      <t xml:space="preserve">0.6
+depth</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
 </t>
     </r>
     <r>
@@ -23416,7 +23651,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">清潔工</t>
+    <t xml:space="preserve">「擊」不可失</t>
   </si>
   <si>
     <r>
@@ -23434,7 +23669,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">100 </t>
+      <t xml:space="preserve">300 </t>
     </r>
     <r>
       <rPr>
@@ -23454,7 +23689,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">100</t>
+      <t xml:space="preserve">300</t>
     </r>
     <r>
       <rPr>
@@ -23473,8 +23708,539 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">1500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4000</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「精」益求精</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個菁英敵人</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「頭」頭是道</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗第一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「目」不暇給</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊敗 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個首領</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「首」屈一指</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗全部 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種首領</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「目」中無人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷擊敗一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「無傷」大雅</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">無傷清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">120</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「血」中送炭</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命時清除一頁</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「閃」亮登場</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">500</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「一閃」一閃亮晶晶</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「穿」流不息</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「桶」快淋漓</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個油桶</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -23492,20 +24258,75 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1000</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">菁英剋星</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊倒 </t>
+      <t xml:space="preserve">150</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">300</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「箱」當然耳</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個箱子</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「桶」歸於盡</t>
+  </si>
+  <si>
+    <t xml:space="preserve">被油桶炸死一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「暈」籌帷幄</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">連續原地旋轉 </t>
     </r>
     <r>
       <rPr>
@@ -23522,10 +24343,357 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">個菁英敵人</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">圈（中間可停一下）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「牌」山倒海</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計使用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">500 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張卡牌</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4000</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「合」家歡樂</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合成升級卡牌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">150</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「招」搖過市</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計施放 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次大招卡</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">600</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「頁」不容辭</t>
+  </si>
+  <si>
+    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「翻」天覆地</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「筆」到成功</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完成整本筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -23536,6 +24704,48 @@
       </rPr>
       <t xml:space="preserve">10</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「課」不容緩</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式抵達第 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -23553,7 +24763,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">30</t>
+      <t xml:space="preserve">25</t>
     </r>
     <r>
       <rPr>
@@ -23572,59 +24782,246 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">60</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">首領退散</t>
-  </si>
-  <si>
-    <t xml:space="preserve">擊敗第一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">首領獵人</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊敗 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個首領</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
+      <t xml:space="preserve">40</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「遊」刃有餘</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">贏得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">場事件小遊戲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「買」力十足</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在商店購買 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「級」不可待</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">5</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「十」分完美</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「金」蟬脫殼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">用金幣復活一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「衣」見鍾情</t>
+  </si>
+  <si>
+    <t xml:space="preserve">儲存一套自訂套組</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「衣衣」不捨</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">收集 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個新顏色或配飾</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「筆」上梁山</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種不同武器完成冒險</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -23642,7 +25039,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">10</t>
+      <t xml:space="preserve">5</t>
     </r>
     <r>
       <rPr>
@@ -23661,88 +25058,85 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">全員到齊</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗全部 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種首領</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完美答卷</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷擊敗一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一塵不染</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">無傷清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
+      <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「扭」轉乾坤</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用遺物扭蛋機抽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「蛋」定蛋定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">抽扭蛋把金幣花到一枚不剩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「遺物」所有</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">解鎖 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件遺物</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
     </r>
     <r>
       <rPr>
@@ -23761,7 +25155,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">25</t>
+      <t xml:space="preserve">15</t>
     </r>
     <r>
       <rPr>
@@ -23780,1270 +25174,11 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">千鈞一髮</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">只剩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點生命時清除一頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">擦身而過</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">閃身步</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一支穿雲劍</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">石油大亨</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個油桶</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">裡面是什麼？</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個箱子</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">易燃易爆炸</t>
-  </si>
-  <si>
-    <t xml:space="preserve">被油桶炸死一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">搖頭晃腦</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">連續原地旋轉 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">圈（中間可停一下）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">出牌手感</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計使用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">張卡牌</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">500</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1000</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">合而為一</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">合成升級卡牌 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">大招成癮</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計施放 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次大招卡</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">第一頁</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">翻頁不停</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">90</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">寫完了！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">完成整本筆記本 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">寫不完</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">課表模式抵達第 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">課間高手</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">贏得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">場事件小遊戲</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">熟客</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在商店購買 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">小有名氣</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「十」分完美</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">墨跡未乾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">用金幣復活一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">穿搭達人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">儲存一套自訂套組</t>
-  </si>
-  <si>
-    <t xml:space="preserve">衣櫃擴充</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">收集 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個新顏色或配飾</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">文具控</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種不同武器完成冒險</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">扭轉乾坤</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用遺物扭蛋機抽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">蛋定蛋定</t>
-  </si>
-  <si>
-    <t xml:space="preserve">抽扭蛋把金幣花到一枚不剩</t>
-  </si>
-  <si>
-    <t xml:space="preserve">遺物所有</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">解鎖 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">件遺物</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">22</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">博物誌</t>
+    <t xml:space="preserve">「鑑」多識廣</t>
   </si>
   <si>
     <r>
@@ -32448,7 +32583,7 @@
       </c>
       <c r="F17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="297" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="377.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
         <v>482</v>
       </c>
@@ -32466,7 +32601,7 @@
       </c>
       <c r="F18" s="10"/>
     </row>
-    <row r="19" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
         <v>487</v>
       </c>
@@ -33477,7 +33612,7 @@
         <v>606</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>607</v>
+        <v>594</v>
       </c>
       <c r="E42" s="10"/>
     </row>
@@ -33486,13 +33621,13 @@
         <v>579</v>
       </c>
       <c r="B43" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>608</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="D43" s="8" t="s">
         <v>609</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>607</v>
       </c>
       <c r="E43" s="10"/>
     </row>
@@ -33627,7 +33762,7 @@
         <v>632</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>633</v>
+        <v>612</v>
       </c>
       <c r="E52" s="10"/>
     </row>
@@ -33636,13 +33771,13 @@
         <v>579</v>
       </c>
       <c r="B53" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="C53" s="7" t="s">
         <v>634</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="D53" s="8" t="s">
         <v>635</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>636</v>
       </c>
       <c r="E53" s="10"/>
     </row>
@@ -33651,13 +33786,13 @@
         <v>579</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="C54" s="7" t="s">
         <v>637</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="D54" s="8" t="s">
         <v>638</v>
-      </c>
-      <c r="D54" s="8" t="s">
-        <v>639</v>
       </c>
       <c r="E54" s="10"/>
     </row>
@@ -33666,13 +33801,13 @@
         <v>579</v>
       </c>
       <c r="B55" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="C55" s="7" t="s">
         <v>640</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="D55" s="8" t="s">
         <v>641</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>642</v>
       </c>
       <c r="E55" s="10"/>
     </row>
@@ -33681,10 +33816,10 @@
         <v>579</v>
       </c>
       <c r="B56" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="C56" s="7" t="s">
         <v>643</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>644</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>599</v>
@@ -33696,10 +33831,10 @@
         <v>579</v>
       </c>
       <c r="B57" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="C57" s="7" t="s">
         <v>645</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>646</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>594</v>
@@ -33711,10 +33846,10 @@
         <v>579</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="C58" s="7" t="s">
         <v>647</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>648</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>619</v>
@@ -33726,10 +33861,10 @@
         <v>579</v>
       </c>
       <c r="B59" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="C59" s="7" t="s">
         <v>649</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>650</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>588</v>
@@ -33741,10 +33876,10 @@
         <v>579</v>
       </c>
       <c r="B60" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="C60" s="7" t="s">
         <v>651</v>
-      </c>
-      <c r="C60" s="7" t="s">
-        <v>652</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>588</v>
@@ -33756,13 +33891,13 @@
         <v>579</v>
       </c>
       <c r="B61" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="C61" s="7" t="s">
         <v>653</v>
       </c>
-      <c r="C61" s="7" t="s">
-        <v>654</v>
-      </c>
       <c r="D61" s="8" t="s">
-        <v>599</v>
+        <v>591</v>
       </c>
       <c r="E61" s="10"/>
     </row>
@@ -33771,13 +33906,13 @@
         <v>579</v>
       </c>
       <c r="B62" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="C62" s="7" t="s">
         <v>655</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="D62" s="8" t="s">
         <v>656</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>657</v>
       </c>
       <c r="E62" s="10"/>
     </row>
@@ -33786,13 +33921,13 @@
         <v>579</v>
       </c>
       <c r="B63" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="C63" s="7" t="s">
         <v>658</v>
       </c>
-      <c r="C63" s="7" t="s">
-        <v>659</v>
-      </c>
       <c r="D63" s="8" t="s">
-        <v>660</v>
+        <v>635</v>
       </c>
       <c r="E63" s="10"/>
     </row>
@@ -33801,10 +33936,10 @@
         <v>579</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>588</v>
@@ -33816,13 +33951,13 @@
         <v>579</v>
       </c>
       <c r="B65" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="D65" s="8" t="s">
         <v>663</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>664</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>665</v>
       </c>
       <c r="E65" s="10"/>
     </row>
@@ -33831,13 +33966,13 @@
         <v>579</v>
       </c>
       <c r="B66" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="D66" s="8" t="s">
         <v>666</v>
-      </c>
-      <c r="C66" s="7" t="s">
-        <v>667</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>668</v>
       </c>
       <c r="E66" s="10"/>
     </row>
@@ -33869,19 +34004,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>493</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>668</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>670</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>671</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>672</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -33889,19 +34024,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>672</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>673</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>674</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>675</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -33910,349 +34045,349 @@
         <v>430</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -34291,7 +34426,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>517</v>
@@ -34300,13 +34435,13 @@
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -34314,115 +34449,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>742</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>743</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>744</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>745</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="F2" s="8" t="s">
         <v>746</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>747</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>748</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>748</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>749</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>750</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>751</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="8" t="s">
         <v>752</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>753</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>754</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>753</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>754</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>755</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>756</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>757</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>758</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>759</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>760</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>760</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>761</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>762</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>763</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>764</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>765</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>766</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>767</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>768</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>769</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>770</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>771</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>772</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.10.14: black correct mark in Simon Says, milder achievement goals, selective pun names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="773">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="776">
   <si>
     <r>
       <rPr>
@@ -23651,7 +23651,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">「擊」不可失</t>
+    <t xml:space="preserve">擊不可失</t>
   </si>
   <si>
     <r>
@@ -23669,7 +23669,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">300 </t>
+      <t xml:space="preserve">150 </t>
     </r>
     <r>
       <rPr>
@@ -23689,7 +23689,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">300</t>
+      <t xml:space="preserve">150</t>
     </r>
     <r>
       <rPr>
@@ -23708,7 +23708,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1500</t>
+      <t xml:space="preserve">600</t>
     </r>
     <r>
       <rPr>
@@ -23727,11 +23727,11 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4000</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「精」益求精</t>
+      <t xml:space="preserve">1200</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">精益求精</t>
   </si>
   <si>
     <r>
@@ -23749,6 +23749,708 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個菁英敵人</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">首領退散</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗第一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">首領獵人</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊敗 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個首領</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">全員到齊</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗全部 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種首領</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">目中無人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷擊敗一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷大雅</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">無傷清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">千鈞一髮</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命時清除一頁</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">閃亮登場</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">150</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">一閃一閃亮晶晶</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">一支穿雲劍</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">石油大亨</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個油桶</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">120</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">箱當然耳</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個箱子</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">桶歸於盡</t>
+  </si>
+  <si>
+    <t xml:space="preserve">被油桶炸死一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">暈籌帷幄</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">連續原地旋轉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">圈（中間可停一下）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">牌山倒海</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計使用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張卡牌</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">600</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1200</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">合而為一</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合成升級卡牌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">25 </t>
     </r>
     <r>
@@ -23757,7 +24459,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">個菁英敵人</t>
+      <t xml:space="preserve">次</t>
     </r>
   </si>
   <si>
@@ -23788,7 +24490,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">80</t>
+      <t xml:space="preserve">50</t>
     </r>
     <r>
       <rPr>
@@ -23807,29 +24509,216 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">200</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「頭」頭是道</t>
-  </si>
-  <si>
-    <t xml:space="preserve">擊敗第一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「目」不暇給</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊敗 </t>
+      <t xml:space="preserve">100</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">招搖過市</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計施放 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次大招卡</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">120</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">第一頁</t>
+  </si>
+  <si>
+    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">翻頁不停</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">寫完了！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完成整本筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">課不容緩</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式抵達第 </t>
     </r>
     <r>
       <rPr>
@@ -23846,7 +24735,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">個首領</t>
+      <t xml:space="preserve">頁</t>
     </r>
   </si>
   <si>
@@ -23896,88 +24785,295 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">遊刃有餘</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">贏得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">場事件小遊戲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">買力十足</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在商店購買 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">小有名氣</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">「十」分完美</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">墨跡未乾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">用金幣復活一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣見鍾情</t>
+  </si>
+  <si>
+    <t xml:space="preserve">儲存一套自訂套組</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣衣不捨</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">收集 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個新顏色或配飾</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">50</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">「首」屈一指</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗全部 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種首領</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「目」中無人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷擊敗一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「無傷」大雅</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">無傷清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
+    <t xml:space="preserve">文具控</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種不同武器完成冒險</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
     </r>
     <r>
       <rPr>
@@ -23996,7 +25092,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">60</t>
+      <t xml:space="preserve">5</t>
     </r>
     <r>
       <rPr>
@@ -24015,20 +25111,20 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">120</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「血」中送炭</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">只剩 </t>
+      <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">扭轉乾坤</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用遺物扭蛋機抽 </t>
     </r>
     <r>
       <rPr>
@@ -24045,36 +25141,6 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">點生命時清除一頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「閃」亮登場</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">次</t>
     </r>
   </si>
@@ -24087,7 +25153,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">50</t>
+      <t xml:space="preserve">1</t>
     </r>
     <r>
       <rPr>
@@ -24106,7 +25172,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">200</t>
+      <t xml:space="preserve">5</t>
     </r>
     <r>
       <rPr>
@@ -24125,121 +25191,55 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">500</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「一閃」一閃亮晶晶</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「穿」流不息</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「桶」快淋漓</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個油桶</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">蛋定蛋定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">抽扭蛋把金幣花到一枚不剩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">遺物所有</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">解鎖 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">件遺物</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
     </r>
     <r>
       <rPr>
@@ -24258,7 +25258,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150</t>
+      <t xml:space="preserve">15</t>
     </r>
     <r>
       <rPr>
@@ -24277,908 +25277,11 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">300</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「箱」當然耳</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個箱子</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「桶」歸於盡</t>
-  </si>
-  <si>
-    <t xml:space="preserve">被油桶炸死一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「暈」籌帷幄</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">連續原地旋轉 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">圈（中間可停一下）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「牌」山倒海</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計使用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">500 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">張卡牌</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">500</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1500</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4000</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「合」家歡樂</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">合成升級卡牌 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">150</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「招」搖過市</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計施放 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次大招卡</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">250</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">600</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「頁」不容辭</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「翻」天覆地</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「筆」到成功</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">完成整本筆記本 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「課」不容緩</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">課表模式抵達第 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「遊」刃有餘</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">贏得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">場事件小遊戲</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「買」力十足</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在商店購買 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「級」不可待</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「十」分完美</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「金」蟬脫殼</t>
-  </si>
-  <si>
-    <t xml:space="preserve">用金幣復活一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「衣」見鍾情</t>
-  </si>
-  <si>
-    <t xml:space="preserve">儲存一套自訂套組</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「衣衣」不捨</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">收集 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個新顏色或配飾</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「筆」上梁山</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種不同武器完成冒險</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「扭」轉乾坤</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用遺物扭蛋機抽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">「蛋」定蛋定</t>
-  </si>
-  <si>
-    <t xml:space="preserve">抽扭蛋把金幣花到一枚不剩</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「遺物」所有</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">解鎖 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">件遺物</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">22</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">「鑑」多識廣</t>
+    <t xml:space="preserve">鑑多識廣</t>
   </si>
   <si>
     <r>
@@ -33612,7 +33715,7 @@
         <v>606</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>594</v>
+        <v>607</v>
       </c>
       <c r="E42" s="10"/>
     </row>
@@ -33621,13 +33724,13 @@
         <v>579</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E43" s="10"/>
     </row>
@@ -33636,13 +33739,13 @@
         <v>579</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E44" s="10"/>
     </row>
@@ -33651,13 +33754,13 @@
         <v>579</v>
       </c>
       <c r="B45" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>613</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>614</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>612</v>
       </c>
       <c r="E45" s="10"/>
     </row>
@@ -33666,10 +33769,10 @@
         <v>579</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>588</v>
@@ -33681,13 +33784,13 @@
         <v>579</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E47" s="10"/>
     </row>
@@ -33696,13 +33799,13 @@
         <v>579</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="E48" s="10"/>
     </row>
@@ -33711,13 +33814,13 @@
         <v>579</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E49" s="10"/>
     </row>
@@ -33726,13 +33829,13 @@
         <v>579</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E50" s="10"/>
     </row>
@@ -33741,10 +33844,10 @@
         <v>579</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>588</v>
@@ -33756,13 +33859,13 @@
         <v>579</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E52" s="10"/>
     </row>
@@ -33771,13 +33874,13 @@
         <v>579</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E53" s="10"/>
     </row>
@@ -33786,13 +33889,13 @@
         <v>579</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E54" s="10"/>
     </row>
@@ -33801,13 +33904,13 @@
         <v>579</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E55" s="10"/>
     </row>
@@ -33816,10 +33919,10 @@
         <v>579</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>599</v>
@@ -33831,10 +33934,10 @@
         <v>579</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>594</v>
@@ -33846,13 +33949,13 @@
         <v>579</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E58" s="10"/>
     </row>
@@ -33861,10 +33964,10 @@
         <v>579</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>588</v>
@@ -33876,10 +33979,10 @@
         <v>579</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>588</v>
@@ -33891,13 +33994,13 @@
         <v>579</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>591</v>
+        <v>655</v>
       </c>
       <c r="E61" s="10"/>
     </row>
@@ -33906,13 +34009,13 @@
         <v>579</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="E62" s="10"/>
     </row>
@@ -33921,13 +34024,13 @@
         <v>579</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>635</v>
+        <v>661</v>
       </c>
       <c r="E63" s="10"/>
     </row>
@@ -33936,10 +34039,10 @@
         <v>579</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>588</v>
@@ -33951,13 +34054,13 @@
         <v>579</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="E65" s="10"/>
     </row>
@@ -33966,13 +34069,13 @@
         <v>579</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="E66" s="10"/>
     </row>
@@ -34004,19 +34107,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>493</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -34024,19 +34127,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -34045,349 +34148,349 @@
         <v>430</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -34426,7 +34529,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>517</v>
@@ -34435,13 +34538,13 @@
         <v>374</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -34449,115 +34552,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
Alarm boss: black second hand, single warned bell wave, pad direction arrow, pressed pad vanishes (beta v0.10.25)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -12419,7 +12419,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【秒針掃射】先畫出紅色預警線，接著細紅雷射繞著它轉一整圈（約 </t>
+      <t xml:space="preserve">【秒針掃射】先畫出紅色預警線，接著細黑雷射繞著它轉一整圈（約 </t>
     </r>
     <r>
       <rPr>
@@ -12473,7 +12473,7 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">秒後時針與分針指著的方向各射出一道光束，先看預警線再躲。
-【鈴鐺響】兩個鈴鐺先後敲響，各發出一圈往外擴散的衝擊波，用衝刺跨過去就不會受傷。
+【鈴鐺響】鈴鐺晃動時，從它身上一圈圈往外淡出的紅環是預警；接著兩個鈴鐺一起敲響，發出一圈往外擴散的衝擊波，用衝刺跨過去就不會受傷。
 【鈴聲爆發】鈴聲條滿了還沒按掉就會爆發：先一圈大衝擊波，接著 </t>
     </r>
     <r>
@@ -12833,7 +12833,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'r': 1.4, 'hold': 0.8, 'hold2': 0.6, 'decay': 0.5, 'inset': 2.4, 'minDist': 5, 'window': 6, 'avoid': 0.45}
+      <t xml:space="preserve">{'r': 1.4, 'hold': 0.8, 'hold2': 0.6, 'decay': 0.5, 'inset': 2.4, 'minDist': 5, 'window': 6, 'avoid': 0.45, 'vanish': 0.3}
 snooze</t>
     </r>
     <r>
@@ -12923,7 +12923,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'tele': 0.7, 'delay': 0.4, 'speed': 6.5, 'max': 18, 'width': 0.45, 'sets': 1, 'sets2': 2, 'setGap': 1.1}
+      <t xml:space="preserve">{'tele': 1.1, 'speed': 6.5, 'max': 18, 'width': 0.45, 'warnCycle': 0.55, 'warnRings': 3, 'warnReach': 6, 'warnWidth': 0.35, 'warnAlpha': 0.7}
 burst</t>
     </r>
     <r>
@@ -32487,7 +32487,7 @@
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="317.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="342.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>363</v>
       </c>

</xml_diff>

<commit_message>
Alarm boss: safe inside pad, single pad in both forms, burst beams delayed, pad hint; smaller text-scaled page banner (beta v0.10.26)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -12474,7 +12474,24 @@
       </rPr>
       <t xml:space="preserve">秒後時針與分針指著的方向各射出一道光束，先看預警線再躲。
 【鈴鐺響】鈴鐺晃動時，從它身上一圈圈往外淡出的紅環是預警；接著兩個鈴鐺一起敲響，發出一圈往外擴散的衝擊波，用衝刺跨過去就不會受傷。
-【鈴聲爆發】鈴聲條滿了還沒按掉就會爆發：先一圈大衝擊波，接著 </t>
+【鈴聲爆發】鈴聲條滿了還沒按掉就會爆發：先一圈大衝擊波，等波過去約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒後，光束才變成三倍旋轉 </t>
     </r>
     <r>
       <rPr>
@@ -12491,7 +12508,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒內光束變成三倍。每次命中 </t>
+      <t xml:space="preserve">秒。每次命中 </t>
     </r>
     <r>
       <rPr>
@@ -12560,7 +12577,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">時，角落會亮起紅色閃動的鬧鐘圈。站進圈內約 </t>
+      <t xml:space="preserve">時，角落會亮起紅色閃動的鬧鐘圈。站在圈內不會受到任何傷害；待約 </t>
     </r>
     <r>
       <rPr>
@@ -12629,24 +12646,24 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">墨水。離開圈子進度會慢慢倒退。
-【雙重鬧鐘（第二型態）】血量剩一半時進化：鈴聲條漲更快，一次亮對角兩個圈，要在 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內兩個都按掉才會貪睡 </t>
+【急躁鬧鐘（第二型態）】血量剩一半時進化：鈴聲條漲更快，鬧鐘圈只要站 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒就能按掉，貪睡變成 </t>
     </r>
     <r>
       <rPr>
@@ -12656,23 +12673,6 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒；只按一個鈴聲條減半、貪睡 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1.5 </t>
     </r>
     <r>
       <rPr>
@@ -12833,7 +12833,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'r': 1.4, 'hold': 0.8, 'hold2': 0.6, 'decay': 0.5, 'inset': 2.4, 'minDist': 5, 'window': 6, 'avoid': 0.45, 'vanish': 0.3}
+      <t xml:space="preserve">{'r': 1.4, 'hold': 0.8, 'hold2': 0.6, 'decay': 0.5, 'inset': 2.4, 'minDist': 5, 'avoid': 0.45, 'vanish': 0.3, 'safe': 0.15}
 snooze</t>
     </r>
     <r>
@@ -12851,7 +12851,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'time': 3.5, 'time2': 4, 'half': 1.5, 'ink': 1}
+      <t xml:space="preserve">{'time': 3.5, 'time2': 4, 'ink': 1}
 second</t>
     </r>
     <r>
@@ -12923,7 +12923,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'tele': 1.1, 'speed': 6.5, 'max': 18, 'width': 0.45, 'warnCycle': 0.55, 'warnRings': 3, 'warnReach': 6, 'warnWidth': 0.35, 'warnAlpha': 0.7}
+      <t xml:space="preserve">{'tele': 1.1, 'rest': 0.9, 'speed': 6.5, 'max': 18, 'width': 0.45, 'warnCycle': 0.55, 'warnRings': 3, 'warnReach': 6, 'warnWidth': 0.35, 'warnAlpha': 0.7}
 burst</t>
     </r>
     <r>
@@ -12941,7 +12941,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'warn': 0.9, 'speed': 9, 'max': 22, 'width': 0.8, 'time': 4, 'mult': 3, 'cap': 2, 'spin': 0.45, 'width2': 0.4, 'len': 24, 'inner': 1.9}
+      <t xml:space="preserve">{'warn': 0.9, 'beamDelay': 1.6, 'speed': 9, 'max': 22, 'width': 0.8, 'time': 4, 'mult': 3, 'cap': 2, 'spin': 0.45, 'width2': 0.4, 'len': 24, 'inner': 1.9}
 p2</t>
     </r>
     <r>

</xml_diff>

<commit_message>
Alarm boss: 1500 HP, hop slam, persistent snooze reminder; boss summons capped at two live waves, slower scissors summons (beta v0.10.28)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -11261,7 +11261,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.9
+      <t xml:space="preserve">2.6
 knockMult</t>
     </r>
     <r>
@@ -12419,7 +12419,42 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【秒針掃射】先畫出紅色預警線，接著細黑雷射繞著它轉一整圈（約 </t>
+      <t xml:space="preserve">【跳躍砸地】先在你的位置畫出紅圈，接著大鬧鐘跳過來砸下，落地時圈內受傷並發出一小圈衝擊波。連跳 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次（第二型態 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次）後跳回原位。
+【秒針掃射】先畫出紅色預警線，接著細黑雷射繞著它轉一整圈（約 </t>
     </r>
     <r>
       <rPr>
@@ -12798,6 +12833,24 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2.2
+hop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{'tele': 0.9, 'homeTele': 0.6, 'air': 0.6, 'height': 3.5, 'r': 2.4, 'count': 2, 'count2': 3, 'margin': 3, 'wave': {'speed': 7, 'max': 6, 'width': 0.4}}
 bar</t>
     </r>
     <r>
@@ -32487,7 +32540,7 @@
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="342.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="381.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>363</v>
       </c>
@@ -32498,7 +32551,7 @@
         <v>342</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>343</v>

</xml_diff>

<commit_message>
Sketch leap from current spot with take-off and landing rings, bounce ball 15, per-boss achievements, faster alarm boss with phase-2 burst and wider gap, wall telegraph matches bullet sheet (beta v0.10.29)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="781">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="793">
   <si>
     <r>
       <rPr>
@@ -3307,7 +3307,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12
+      <t xml:space="preserve">15
 bounces</t>
     </r>
     <r>
@@ -3348,7 +3348,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12
+      <t xml:space="preserve">15
 bounces</t>
     </r>
     <r>
@@ -3387,7 +3387,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
+      <t xml:space="preserve">15</t>
     </r>
     <r>
       <rPr>
@@ -3431,7 +3431,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
+      <t xml:space="preserve">15</t>
     </r>
     <r>
       <rPr>
@@ -5489,7 +5489,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">先向四周射出 </t>
+      <t xml:space="preserve">從目前位置跳到目標位置，起跳與落地時各向四周射出 </t>
     </r>
     <r>
       <rPr>
@@ -5523,17 +5523,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">），再跳到目標位置，跳躍中不會受傷。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">先向四周射出 </t>
+      <t xml:space="preserve">），跳躍中不會受傷。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">從目前位置跳到目標位置，起跳與落地時各向四周射出 </t>
     </r>
     <r>
       <rPr>
@@ -5567,7 +5567,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">），再跳到目標位置，跳躍中不會受傷。</t>
+      <t xml:space="preserve">），跳躍中不會受傷。</t>
     </r>
   </si>
   <si>
@@ -12681,7 +12681,7 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">墨水。離開圈子進度會慢慢倒退。
-【急躁鬧鐘（第二型態）】血量剩一半時進化：鈴聲條漲更快，鬧鐘圈只要站 </t>
+【急躁鬧鐘（第二型態）】血量剩一半時進化，一進化就立刻鈴聲爆發！之後鈴聲條漲更快，鬧鐘圈只要站 </t>
     </r>
     <r>
       <rPr>
@@ -12814,7 +12814,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[1, 1.5]
+      <t xml:space="preserve">[0.45, 0.8]
 first</t>
     </r>
     <r>
@@ -12832,7 +12832,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2.2
+      <t xml:space="preserve">1.2
 hop</t>
     </r>
     <r>
@@ -12940,7 +12940,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'warn': 1.1, 'dur': 6, 'speeds': [0.36, 0.78, -0.6], 'width': 0.42, 'gap': [5.5, 8.5], 'gapW': 2.6, 'len': 24, 'inner': 1.9}
+      <t xml:space="preserve">{'warn': 1.1, 'dur': 5, 'speeds': [0.36, 0.78, -0.6], 'width': 0.42, 'gap': [5.5, 8.5], 'gapW': 3.3, 'len': 24, 'inner': 1.9}
 chime</t>
     </r>
     <r>
@@ -12976,7 +12976,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'tele': 1.1, 'rest': 0.9, 'speed': 6.5, 'max': 18, 'width': 0.45, 'warnCycle': 0.55, 'warnRings': 3, 'warnReach': 6, 'warnWidth': 0.35, 'warnAlpha': 0.7}
+      <t xml:space="preserve">{'tele': 1.1, 'rest': 0.5, 'speed': 6.5, 'max': 18, 'width': 0.45, 'warnCycle': 0.55, 'warnRings': 3, 'warnReach': 6, 'warnWidth': 0.35, 'warnAlpha': 0.7}
 burst</t>
     </r>
     <r>
@@ -24558,6 +24558,42 @@
   </si>
   <si>
     <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">瓶安歸來</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗巨型墨瓶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">剪單明瞭</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗剪刀魔</t>
+  </si>
+  <si>
+    <t xml:space="preserve">書途同歸</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗墨跡之書</t>
+  </si>
+  <si>
+    <t xml:space="preserve">金榜題名</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗考卷魔王</t>
+  </si>
+  <si>
+    <t xml:space="preserve">妙筆生花</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗巨筆暴君</t>
+  </si>
+  <si>
+    <t xml:space="preserve">鐘於解脫</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗大鬧鐘</t>
   </si>
   <si>
     <t xml:space="preserve">目中無人</t>
@@ -33757,7 +33793,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -34342,7 +34378,7 @@
         <v>602</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>603</v>
+        <v>592</v>
       </c>
       <c r="E39" s="10"/>
     </row>
@@ -34351,10 +34387,10 @@
         <v>583</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>604</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>605</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>592</v>
@@ -34366,13 +34402,13 @@
         <v>583</v>
       </c>
       <c r="B41" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>606</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>607</v>
-      </c>
       <c r="D41" s="8" t="s">
-        <v>608</v>
+        <v>592</v>
       </c>
       <c r="E41" s="10"/>
     </row>
@@ -34381,13 +34417,13 @@
         <v>583</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>609</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>610</v>
+        <v>607</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>608</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>611</v>
+        <v>592</v>
       </c>
       <c r="E42" s="10"/>
     </row>
@@ -34396,13 +34432,13 @@
         <v>583</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>614</v>
+        <v>592</v>
       </c>
       <c r="E43" s="10"/>
     </row>
@@ -34411,13 +34447,13 @@
         <v>583</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>617</v>
+        <v>592</v>
       </c>
       <c r="E44" s="10"/>
     </row>
@@ -34426,13 +34462,13 @@
         <v>583</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E45" s="10"/>
     </row>
@@ -34441,10 +34477,10 @@
         <v>583</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>592</v>
@@ -34456,28 +34492,28 @@
         <v>583</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>624</v>
+        <v>620</v>
       </c>
       <c r="E47" s="10"/>
     </row>
-    <row r="48" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>583</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>625</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>626</v>
+        <v>621</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>622</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="E48" s="10"/>
     </row>
@@ -34486,13 +34522,13 @@
         <v>583</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="E49" s="10"/>
     </row>
@@ -34501,13 +34537,13 @@
         <v>583</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>632</v>
+        <v>628</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="E50" s="10"/>
     </row>
@@ -34516,13 +34552,13 @@
         <v>583</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>634</v>
+        <v>630</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>635</v>
+        <v>631</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>592</v>
+        <v>629</v>
       </c>
       <c r="E51" s="10"/>
     </row>
@@ -34531,13 +34567,13 @@
         <v>583</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>617</v>
+        <v>592</v>
       </c>
       <c r="E52" s="10"/>
     </row>
@@ -34546,28 +34582,28 @@
         <v>583</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>638</v>
+        <v>634</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>640</v>
+        <v>636</v>
       </c>
       <c r="E53" s="10"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
         <v>583</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>641</v>
+        <v>637</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="E54" s="10"/>
     </row>
@@ -34576,13 +34612,13 @@
         <v>583</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="E55" s="10"/>
     </row>
@@ -34591,13 +34627,13 @@
         <v>583</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>603</v>
+        <v>645</v>
       </c>
       <c r="E56" s="10"/>
     </row>
@@ -34606,13 +34642,13 @@
         <v>583</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>651</v>
+        <v>592</v>
       </c>
       <c r="E57" s="10"/>
     </row>
@@ -34621,13 +34657,13 @@
         <v>583</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>652</v>
+        <v>648</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>653</v>
+        <v>649</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="E58" s="10"/>
     </row>
@@ -34636,13 +34672,13 @@
         <v>583</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>655</v>
+        <v>651</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>592</v>
+        <v>652</v>
       </c>
       <c r="E59" s="10"/>
     </row>
@@ -34651,13 +34687,13 @@
         <v>583</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>592</v>
+        <v>655</v>
       </c>
       <c r="E60" s="10"/>
     </row>
@@ -34666,13 +34702,13 @@
         <v>583</v>
       </c>
       <c r="B61" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="D61" s="8" t="s">
         <v>658</v>
-      </c>
-      <c r="C61" s="7" t="s">
-        <v>659</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>660</v>
       </c>
       <c r="E61" s="10"/>
     </row>
@@ -34681,13 +34717,13 @@
         <v>583</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>663</v>
+        <v>615</v>
       </c>
       <c r="E62" s="10"/>
     </row>
@@ -34696,13 +34732,13 @@
         <v>583</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="E63" s="10"/>
     </row>
@@ -34711,13 +34747,13 @@
         <v>583</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>592</v>
+        <v>636</v>
       </c>
       <c r="E64" s="10"/>
     </row>
@@ -34726,13 +34762,13 @@
         <v>583</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>671</v>
+        <v>592</v>
       </c>
       <c r="E65" s="10"/>
     </row>
@@ -34741,15 +34777,105 @@
         <v>583</v>
       </c>
       <c r="B66" s="7" t="s">
+        <v>668</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="D66" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="E66" s="10"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="D67" s="8" t="s">
         <v>672</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="E67" s="10"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B68" s="7" t="s">
         <v>673</v>
       </c>
-      <c r="D66" s="8" t="s">
+      <c r="C68" s="7" t="s">
         <v>674</v>
       </c>
-      <c r="E66" s="10"/>
+      <c r="D68" s="8" t="s">
+        <v>675</v>
+      </c>
+      <c r="E68" s="10"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>676</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="D69" s="8" t="s">
+        <v>678</v>
+      </c>
+      <c r="E69" s="10"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>680</v>
+      </c>
+      <c r="D70" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="E70" s="10"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>681</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="D71" s="8" t="s">
+        <v>683</v>
+      </c>
+      <c r="E71" s="10"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>684</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="D72" s="8" t="s">
+        <v>686</v>
+      </c>
+      <c r="E72" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -34779,19 +34905,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>675</v>
+        <v>687</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>497</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>676</v>
+        <v>688</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>677</v>
+        <v>689</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>678</v>
+        <v>690</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -34799,19 +34925,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>679</v>
+        <v>691</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>680</v>
+        <v>692</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>681</v>
+        <v>693</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>682</v>
+        <v>694</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -34820,349 +34946,349 @@
         <v>434</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>683</v>
+        <v>695</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>681</v>
+        <v>693</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>684</v>
+        <v>696</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>685</v>
+        <v>697</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>686</v>
+        <v>698</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>681</v>
+        <v>693</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>687</v>
+        <v>699</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>688</v>
+        <v>700</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>689</v>
+        <v>701</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>681</v>
+        <v>693</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>690</v>
+        <v>702</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>691</v>
+        <v>703</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>692</v>
+        <v>704</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>693</v>
+        <v>705</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>694</v>
+        <v>706</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>695</v>
+        <v>707</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>696</v>
+        <v>708</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>697</v>
+        <v>709</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>698</v>
+        <v>710</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>699</v>
+        <v>711</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>700</v>
+        <v>712</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>701</v>
+        <v>713</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>702</v>
+        <v>714</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>703</v>
+        <v>715</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>704</v>
+        <v>716</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>705</v>
+        <v>717</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>706</v>
+        <v>718</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>707</v>
+        <v>719</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>708</v>
+        <v>720</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>709</v>
+        <v>721</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>710</v>
+        <v>722</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>711</v>
+        <v>723</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>712</v>
+        <v>724</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>713</v>
+        <v>725</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>714</v>
+        <v>726</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>715</v>
+        <v>727</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>716</v>
+        <v>728</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>717</v>
+        <v>729</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>718</v>
+        <v>730</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>719</v>
+        <v>731</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>720</v>
+        <v>732</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>721</v>
+        <v>733</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>722</v>
+        <v>734</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>723</v>
+        <v>735</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>724</v>
+        <v>736</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>725</v>
+        <v>737</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>726</v>
+        <v>738</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>727</v>
+        <v>739</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>728</v>
+        <v>740</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>729</v>
+        <v>741</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>730</v>
+        <v>742</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>731</v>
+        <v>743</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>705</v>
+        <v>717</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>732</v>
+        <v>744</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>733</v>
+        <v>745</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>734</v>
+        <v>746</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>735</v>
+        <v>747</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>736</v>
+        <v>748</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>737</v>
+        <v>749</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>738</v>
+        <v>750</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>739</v>
+        <v>751</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>740</v>
+        <v>752</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>741</v>
+        <v>753</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>742</v>
+        <v>754</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>743</v>
+        <v>755</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>744</v>
+        <v>756</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>745</v>
+        <v>757</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -35201,7 +35327,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>746</v>
+        <v>758</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>521</v>
@@ -35210,13 +35336,13 @@
         <v>378</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>747</v>
+        <v>759</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>748</v>
+        <v>760</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>678</v>
+        <v>690</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -35224,115 +35350,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>749</v>
+        <v>761</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>750</v>
+        <v>762</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>751</v>
+        <v>763</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>752</v>
+        <v>764</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>753</v>
+        <v>765</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>754</v>
+        <v>766</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>755</v>
+        <v>767</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>756</v>
+        <v>768</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>757</v>
+        <v>769</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>758</v>
+        <v>770</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>759</v>
+        <v>771</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>760</v>
+        <v>772</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>761</v>
+        <v>773</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>762</v>
+        <v>774</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>763</v>
+        <v>775</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>764</v>
+        <v>776</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>765</v>
+        <v>777</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>766</v>
+        <v>778</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>767</v>
+        <v>779</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>768</v>
+        <v>780</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>769</v>
+        <v>781</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>770</v>
+        <v>782</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>771</v>
+        <v>783</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>772</v>
+        <v>784</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>773</v>
+        <v>785</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>774</v>
+        <v>786</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>775</v>
+        <v>787</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>776</v>
+        <v>788</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>777</v>
+        <v>789</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>778</v>
+        <v>790</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>779</v>
+        <v>791</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>780</v>
+        <v>792</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
Per-boss achievements become 10/20/30 defeat tiers (beta v0.10.30)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="793">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="794">
   <si>
     <r>
       <rPr>
@@ -24563,37 +24563,231 @@
     <t xml:space="preserve">瓶安歸來</t>
   </si>
   <si>
-    <t xml:space="preserve">擊敗巨型墨瓶</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗巨型墨瓶 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">剪單明瞭</t>
   </si>
   <si>
-    <t xml:space="preserve">擊敗剪刀魔</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗剪刀魔 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">書途同歸</t>
   </si>
   <si>
-    <t xml:space="preserve">擊敗墨跡之書</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗墨跡之書 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">金榜題名</t>
   </si>
   <si>
-    <t xml:space="preserve">擊敗考卷魔王</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗考卷魔王 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">妙筆生花</t>
   </si>
   <si>
-    <t xml:space="preserve">擊敗巨筆暴君</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗巨筆暴君 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">鐘於解脫</t>
   </si>
   <si>
-    <t xml:space="preserve">擊敗大鬧鐘</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗大鬧鐘 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">目中無人</t>
@@ -34363,7 +34557,7 @@
         <v>600</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E38" s="10"/>
     </row>
@@ -34372,13 +34566,13 @@
         <v>583</v>
       </c>
       <c r="B39" s="7" t="s">
+        <v>602</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>601</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>602</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>592</v>
       </c>
       <c r="E39" s="10"/>
     </row>
@@ -34387,13 +34581,13 @@
         <v>583</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E40" s="10"/>
     </row>
@@ -34402,13 +34596,13 @@
         <v>583</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E41" s="10"/>
     </row>
@@ -34417,13 +34611,13 @@
         <v>583</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E42" s="10"/>
     </row>
@@ -34432,13 +34626,13 @@
         <v>583</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>592</v>
+        <v>601</v>
       </c>
       <c r="E43" s="10"/>
     </row>
@@ -34447,10 +34641,10 @@
         <v>583</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>592</v>
@@ -34462,13 +34656,13 @@
         <v>583</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E45" s="10"/>
     </row>
@@ -34477,10 +34671,10 @@
         <v>583</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>592</v>
@@ -34492,13 +34686,13 @@
         <v>583</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E47" s="10"/>
     </row>
@@ -34507,13 +34701,13 @@
         <v>583</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E48" s="10"/>
     </row>
@@ -34522,13 +34716,13 @@
         <v>583</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E49" s="10"/>
     </row>
@@ -34537,13 +34731,13 @@
         <v>583</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E50" s="10"/>
     </row>
@@ -34552,13 +34746,13 @@
         <v>583</v>
       </c>
       <c r="B51" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="D51" s="8" t="s">
         <v>630</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>631</v>
-      </c>
-      <c r="D51" s="8" t="s">
-        <v>629</v>
       </c>
       <c r="E51" s="10"/>
     </row>
@@ -34567,10 +34761,10 @@
         <v>583</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>592</v>
@@ -34582,13 +34776,13 @@
         <v>583</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E53" s="10"/>
     </row>
@@ -34597,13 +34791,13 @@
         <v>583</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E54" s="10"/>
     </row>
@@ -34612,13 +34806,13 @@
         <v>583</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E55" s="10"/>
     </row>
@@ -34627,13 +34821,13 @@
         <v>583</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E56" s="10"/>
     </row>
@@ -34642,10 +34836,10 @@
         <v>583</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>592</v>
@@ -34657,13 +34851,13 @@
         <v>583</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E58" s="10"/>
     </row>
@@ -34672,13 +34866,13 @@
         <v>583</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E59" s="10"/>
     </row>
@@ -34687,13 +34881,13 @@
         <v>583</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="E60" s="10"/>
     </row>
@@ -34702,13 +34896,13 @@
         <v>583</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="E61" s="10"/>
     </row>
@@ -34717,13 +34911,13 @@
         <v>583</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E62" s="10"/>
     </row>
@@ -34732,13 +34926,13 @@
         <v>583</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E63" s="10"/>
     </row>
@@ -34747,13 +34941,13 @@
         <v>583</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E64" s="10"/>
     </row>
@@ -34762,10 +34956,10 @@
         <v>583</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>592</v>
@@ -34777,10 +34971,10 @@
         <v>583</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>592</v>
@@ -34792,13 +34986,13 @@
         <v>583</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="E67" s="10"/>
     </row>
@@ -34807,13 +35001,13 @@
         <v>583</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="E68" s="10"/>
     </row>
@@ -34822,13 +35016,13 @@
         <v>583</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="E69" s="10"/>
     </row>
@@ -34837,10 +35031,10 @@
         <v>583</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D70" s="8" t="s">
         <v>592</v>
@@ -34852,13 +35046,13 @@
         <v>583</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="E71" s="10"/>
     </row>
@@ -34867,13 +35061,13 @@
         <v>583</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E72" s="10"/>
     </row>
@@ -34905,19 +35099,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>497</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -34925,19 +35119,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -34946,349 +35140,349 @@
         <v>434</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -35327,7 +35521,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>521</v>
@@ -35336,13 +35530,13 @@
         <v>378</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -35350,115 +35544,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
Touch reload button, achievement list top padding, no boss coin drop, alarm snoozes in place, line-plus-fade telegraphs for walls and rotating beams (beta v0.10.32)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="794">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="792">
   <si>
     <r>
       <rPr>
@@ -12850,7 +12850,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'tele': 0.9, 'homeTele': 0.6, 'air': 0.6, 'height': 3.5, 'r': 2.4, 'count': 2, 'count2': 3, 'margin': 3, 'wave': {'speed': 7, 'max': 6, 'width': 0.4}}
+      <t xml:space="preserve">{'tele': 0.9, 'homeTele': 0.6, 'air': 0.6, 'height': 3.5, 'fall': 14, 'r': 2.4, 'count': 2, 'count2': 3, 'margin': 3, 'wave': {'speed': 7, 'max': 6, 'width': 0.4}}
 bar</t>
     </r>
     <r>
@@ -23721,12 +23721,6 @@
       </rPr>
       <t xml:space="preserve">3</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">擊敗頭目獲得墨點</t>
-  </si>
-  <si>
-    <t xml:space="preserve">筆記本與課表模式</t>
   </si>
   <si>
     <t xml:space="preserve">等級獎勵</t>
@@ -33987,7 +33981,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -34226,7 +34220,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>550</v>
+        <v>537</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>556</v>
@@ -34235,48 +34229,46 @@
         <v>557</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>537</v>
+        <v>558</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>558</v>
-      </c>
-      <c r="C17" s="7" t="s">
         <v>559</v>
       </c>
+      <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>558</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>560</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>561</v>
       </c>
-      <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>562</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>563</v>
-      </c>
+      <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>5</v>
       </c>
@@ -34284,23 +34276,23 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -34310,20 +34302,22 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>566</v>
       </c>
-      <c r="C22" s="7"/>
+      <c r="C22" s="7" t="s">
+        <v>567</v>
+      </c>
       <c r="D22" s="8" t="n">
-        <v>1</v>
+        <v>45000</v>
       </c>
       <c r="E22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>568</v>
@@ -34332,13 +34326,13 @@
         <v>569</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>45000</v>
+        <v>35000</v>
       </c>
       <c r="E23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>570</v>
@@ -34347,13 +34341,13 @@
         <v>571</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>35000</v>
+        <v>20000</v>
       </c>
       <c r="E24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>572</v>
@@ -34362,13 +34356,13 @@
         <v>573</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>20000</v>
+        <v>10000</v>
       </c>
       <c r="E25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>574</v>
@@ -34377,193 +34371,193 @@
         <v>575</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="E26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>576</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>577</v>
+        <v>567</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>5000</v>
+        <v>80000</v>
       </c>
       <c r="E27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>569</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>80000</v>
+        <v>60000</v>
       </c>
       <c r="E28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>571</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="E29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>573</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="E30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>575</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="E31" s="10"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>567</v>
+        <v>581</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>582</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>577</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>5000</v>
+        <v>583</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>584</v>
       </c>
       <c r="E32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E33" s="10"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B38" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>599</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>600</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>601</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>602</v>
@@ -34572,13 +34566,13 @@
         <v>603</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>604</v>
@@ -34587,13 +34581,13 @@
         <v>605</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>606</v>
@@ -34602,13 +34596,13 @@
         <v>607</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>608</v>
@@ -34617,13 +34611,13 @@
         <v>609</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>610</v>
@@ -34632,13 +34626,13 @@
         <v>611</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>601</v>
+        <v>590</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>612</v>
@@ -34647,28 +34641,28 @@
         <v>613</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>592</v>
+        <v>614</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>616</v>
+        <v>590</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>617</v>
@@ -34677,73 +34671,73 @@
         <v>618</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>592</v>
+        <v>619</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>619</v>
-      </c>
-      <c r="C47" s="7" t="s">
         <v>620</v>
       </c>
+      <c r="C47" s="6" t="s">
+        <v>621</v>
+      </c>
       <c r="D47" s="8" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C48" s="6" t="s">
         <v>623</v>
       </c>
+      <c r="C48" s="7" t="s">
+        <v>624</v>
+      </c>
       <c r="D48" s="8" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B50" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="D50" s="8" t="s">
         <v>628</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>629</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>630</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>631</v>
@@ -34752,13 +34746,13 @@
         <v>632</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>630</v>
+        <v>590</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>633</v>
@@ -34767,73 +34761,73 @@
         <v>634</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>592</v>
+        <v>635</v>
       </c>
       <c r="E52" s="10"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E53" s="10"/>
     </row>
-    <row r="54" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>646</v>
+        <v>590</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B57" s="7" t="s">
         <v>647</v>
@@ -34842,13 +34836,13 @@
         <v>648</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>592</v>
+        <v>628</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B58" s="7" t="s">
         <v>649</v>
@@ -34857,58 +34851,58 @@
         <v>650</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>630</v>
+        <v>651</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>659</v>
+        <v>614</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B62" s="7" t="s">
         <v>660</v>
@@ -34917,28 +34911,28 @@
         <v>661</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>616</v>
+        <v>662</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>664</v>
+        <v>635</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B64" s="7" t="s">
         <v>665</v>
@@ -34947,13 +34941,13 @@
         <v>666</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>637</v>
+        <v>590</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B65" s="7" t="s">
         <v>667</v>
@@ -34962,13 +34956,13 @@
         <v>668</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B66" s="7" t="s">
         <v>669</v>
@@ -34977,58 +34971,58 @@
         <v>670</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>592</v>
+        <v>671</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>679</v>
+        <v>590</v>
       </c>
       <c r="E69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B70" s="7" t="s">
         <v>680</v>
@@ -35037,39 +35031,24 @@
         <v>681</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>592</v>
+        <v>682</v>
       </c>
       <c r="E70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E71" s="10"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="7" t="s">
-        <v>583</v>
-      </c>
-      <c r="B72" s="7" t="s">
-        <v>685</v>
-      </c>
-      <c r="C72" s="7" t="s">
-        <v>686</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>687</v>
-      </c>
-      <c r="E72" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -35099,19 +35078,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>497</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>689</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>690</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>691</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -35119,19 +35098,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>691</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>692</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>693</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>694</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -35140,349 +35119,349 @@
         <v>434</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -35521,7 +35500,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>521</v>
@@ -35530,13 +35509,13 @@
         <v>378</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -35544,115 +35523,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>760</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>762</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>763</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>764</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="F2" s="8" t="s">
         <v>765</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>766</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>767</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>767</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>768</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>769</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>770</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="8" t="s">
         <v>771</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>772</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>773</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>772</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>773</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>774</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>775</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>776</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>777</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>778</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>779</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>778</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>779</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>780</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>781</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>782</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>783</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>784</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>785</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>785</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>786</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>787</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>788</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>789</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>790</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>791</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
Puppet ult rework, portal art, gacha no-skip and punchier pull sounds, relic info button, tutorial reminders and deck hints, release-to-cast instant skills (beta v0.10.33)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -7998,37 +7998,17 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">5
-shields</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">放出不會攻擊的傀儡，</t>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">放出不會攻擊的傀儡（從天而降砸在目標位置），</t>
     </r>
     <r>
       <rPr>
@@ -8045,24 +8025,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒內吸引所有敵人；同時紙盾補到 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">片，時間到收回這次補的紙盾。</t>
+      <t xml:space="preserve">秒內所有敵人都會被吸引、往傀儡移動；這段時間你不會受到任何子彈（遠程攻擊）的傷害，被子彈打中也不會扣紙盾。衝撞、砸地等近身攻擊仍會受傷。</t>
     </r>
   </si>
   <si>
@@ -26223,7 +26186,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">、刷子 </t>
+      <t xml:space="preserve">、毛筆 </t>
     </r>
     <r>
       <rPr>
@@ -31801,7 +31764,7 @@
       </c>
       <c r="P38" s="10"/>
     </row>
-    <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
         <v>266</v>
       </c>

</xml_diff>

<commit_message>
beta v0.10.34: accessory clip, reload button, late dodge, tutorial remind tweaks, taller back wall, alarm boss tuning
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -12417,16 +12417,16 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">次）後跳回原位。
-【秒針掃射】先畫出紅色預警線，接著細黑雷射繞著它轉一整圈（約 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
+【秒針掃射】先畫出紅色預警線，接著細黑雷射繞著它轉一圈多（約 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5 </t>
     </r>
     <r>
       <rPr>
@@ -12644,7 +12644,7 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">墨水。離開圈子進度會慢慢倒退。
-【急躁鬧鐘（第二型態）】血量剩一半時進化，一進化就立刻鈴聲爆發！之後鈴聲條漲更快，鬧鐘圈只要站 </t>
+【急躁鬧鐘（第二型態）】血量剩一半時進化，一進化就立刻鈴聲爆發！之後鈴聲條漲更快，會同時亮起兩個相鄰（不會在對角）的鬧鐘圈，各站 </t>
     </r>
     <r>
       <rPr>
@@ -12661,7 +12661,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒就能按掉，貪睡變成 </t>
+      <t xml:space="preserve">秒、兩個都按掉才會貪睡，貪睡變成 </t>
     </r>
     <r>
       <rPr>
@@ -12777,7 +12777,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[0.45, 0.8]
+      <t xml:space="preserve">[0.3, 0.6]
 first</t>
     </r>
     <r>
@@ -12795,7 +12795,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.2
+      <t xml:space="preserve">1
 hop</t>
     </r>
     <r>
@@ -12885,7 +12885,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'warn': 1, 'period': 6, 'turns': 1, 'width': 0.14, 'len': 24, 'inner': 1.9}
+      <t xml:space="preserve">{'warn': 1, 'period': 5, 'turns': 1.2, 'width': 0.14, 'len': 24, 'inner': 1.9}
 hands</t>
     </r>
     <r>
@@ -12903,7 +12903,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'warn': 1.1, 'dur': 5, 'speeds': [0.36, 0.78, -0.6], 'width': 0.42, 'gap': [5.5, 8.5], 'gapW': 3.3, 'len': 24, 'inner': 1.9}
+      <t xml:space="preserve">{'warn': 1.1, 'dur': 5.5, 'speeds': [0.44, 0.92, -0.72], 'width': 0.42, 'gap': [5.5, 8.5], 'gapW': 3.3, 'len': 24, 'inner': 1.9}
 chime</t>
     </r>
     <r>
@@ -32738,7 +32738,7 @@
         <v>342</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1500</v>
+        <v>1300</v>
       </c>
       <c r="E18" s="12" t="s">
         <v>343</v>

</xml_diff>

<commit_message>
beta v0.10.35: calculator boss, revert late dodge, mask fit, arena-clipped attacks, alarm edge glow, door wall, achievements, S++ grade, remove dev overlay
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="792">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="798">
   <si>
     <r>
       <rPr>
@@ -23813,6 +23813,69 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">S++</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分數門檻（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S++ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">級結算獎勵 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">金幣）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">S+</t>
     </r>
   </si>
@@ -24128,6 +24191,25 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">S++</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">S+</t>
     </r>
   </si>
@@ -24747,6 +24829,36 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">精打細算</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗計算機魔王 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">目中無人</t>
   </si>
   <si>
@@ -24943,7 +25055,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">一閃一閃亮晶晶</t>
+    <t xml:space="preserve">閃身步</t>
   </si>
   <si>
     <r>
@@ -25018,7 +25130,7 @@
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">石油大亨</t>
+    <t xml:space="preserve">易燃易爆炸</t>
   </si>
   <si>
     <r>
@@ -25143,7 +25255,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">連續原地旋轉 </t>
+      <t xml:space="preserve">移動或瞄準方向連續轉 </t>
     </r>
     <r>
       <rPr>
@@ -25160,7 +25272,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">圈（中間可停一下）</t>
+      <t xml:space="preserve">圈（左右搖桿都可以，中間可停一下）</t>
     </r>
   </si>
   <si>
@@ -25353,7 +25465,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">次大招卡</t>
+      <t xml:space="preserve">次特殊卡</t>
     </r>
   </si>
   <si>
@@ -25769,7 +25881,34 @@
     <t xml:space="preserve">衣見鍾情</t>
   </si>
   <si>
-    <t xml:space="preserve">儲存一套自訂套組</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">儲存 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">套自訂套組</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
   </si>
   <si>
     <t xml:space="preserve">衣衣不捨</t>
@@ -33944,7 +34083,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -34274,7 +34413,7 @@
         <v>567</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="E22" s="10"/>
     </row>
@@ -34289,7 +34428,7 @@
         <v>569</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>35000</v>
+        <v>45000</v>
       </c>
       <c r="E23" s="10"/>
     </row>
@@ -34304,7 +34443,7 @@
         <v>571</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>20000</v>
+        <v>35000</v>
       </c>
       <c r="E24" s="10"/>
     </row>
@@ -34319,7 +34458,7 @@
         <v>573</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>10000</v>
+        <v>20000</v>
       </c>
       <c r="E25" s="10"/>
     </row>
@@ -34334,7 +34473,7 @@
         <v>575</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="E26" s="10"/>
     </row>
@@ -34346,10 +34485,10 @@
         <v>576</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>567</v>
+        <v>577</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>80000</v>
+        <v>5000</v>
       </c>
       <c r="E27" s="10"/>
     </row>
@@ -34358,13 +34497,13 @@
         <v>565</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>60000</v>
+        <v>110000</v>
       </c>
       <c r="E28" s="10"/>
     </row>
@@ -34373,13 +34512,13 @@
         <v>565</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="E29" s="10"/>
     </row>
@@ -34388,13 +34527,13 @@
         <v>565</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>15000</v>
+        <v>60000</v>
       </c>
       <c r="E30" s="10"/>
     </row>
@@ -34403,115 +34542,115 @@
         <v>565</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>5000</v>
+        <v>30000</v>
       </c>
       <c r="E31" s="10"/>
     </row>
-    <row r="32" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>581</v>
+        <v>565</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>582</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>583</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>584</v>
+        <v>575</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>15000</v>
       </c>
       <c r="E32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>581</v>
+        <v>565</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>586</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>587</v>
+        <v>577</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>5000</v>
       </c>
       <c r="E33" s="10"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="D38" s="8" t="s">
         <v>599</v>
@@ -34520,498 +34659,543 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B39" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>602</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>603</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>599</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>603</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>604</v>
       </c>
-      <c r="C40" s="7" t="s">
-        <v>605</v>
-      </c>
       <c r="D40" s="8" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B41" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>606</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>607</v>
-      </c>
       <c r="D41" s="8" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>607</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>608</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>609</v>
-      </c>
       <c r="D42" s="8" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B43" s="7" t="s">
+        <v>609</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>610</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>611</v>
-      </c>
       <c r="D43" s="8" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B44" s="7" t="s">
+        <v>611</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>612</v>
       </c>
-      <c r="C44" s="7" t="s">
-        <v>613</v>
-      </c>
       <c r="D44" s="8" t="s">
-        <v>614</v>
+        <v>602</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>619</v>
+        <v>593</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>620</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>621</v>
+        <v>617</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>618</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>625</v>
+        <v>593</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>628</v>
+        <v>624</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>629</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>630</v>
+        <v>625</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>626</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>590</v>
+        <v>630</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B52" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="D52" s="8" t="s">
         <v>633</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>634</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>635</v>
       </c>
       <c r="E52" s="10"/>
     </row>
-    <row r="53" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>641</v>
+        <v>593</v>
       </c>
       <c r="E54" s="10"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>644</v>
+        <v>640</v>
       </c>
       <c r="E55" s="10"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>645</v>
+        <v>641</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>590</v>
+        <v>643</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>628</v>
+        <v>646</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="D58" s="8" t="s">
         <v>649</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>650</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>651</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>654</v>
+        <v>593</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>657</v>
+        <v>633</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>614</v>
+        <v>656</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>635</v>
+        <v>662</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>590</v>
+        <v>619</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B65" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>666</v>
+      </c>
+      <c r="D65" s="8" t="s">
         <v>667</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>668</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>590</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B66" s="7" t="s">
+        <v>668</v>
+      </c>
+      <c r="C66" s="7" t="s">
         <v>669</v>
       </c>
-      <c r="C66" s="7" t="s">
-        <v>670</v>
-      </c>
       <c r="D66" s="8" t="s">
-        <v>671</v>
+        <v>640</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>674</v>
+        <v>593</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>590</v>
+        <v>677</v>
       </c>
       <c r="E69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B70" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="D70" s="8" t="s">
         <v>680</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>681</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>682</v>
       </c>
       <c r="E70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B71" s="7" t="s">
+        <v>681</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="D71" s="8" t="s">
         <v>683</v>
       </c>
-      <c r="C71" s="7" t="s">
+      <c r="E71" s="10"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="B72" s="7" t="s">
         <v>684</v>
       </c>
-      <c r="D71" s="8" t="s">
+      <c r="C72" s="7" t="s">
         <v>685</v>
       </c>
-      <c r="E71" s="10"/>
+      <c r="D72" s="8" t="s">
+        <v>593</v>
+      </c>
+      <c r="E72" s="10"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>687</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>688</v>
+      </c>
+      <c r="E73" s="10"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>689</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>690</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>691</v>
+      </c>
+      <c r="E74" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -35041,19 +35225,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>497</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -35061,19 +35245,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -35082,349 +35266,349 @@
         <v>434</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -35463,7 +35647,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>521</v>
@@ -35472,13 +35656,13 @@
         <v>378</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -35486,115 +35670,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>782</v>
+        <v>788</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
beta v0.10.36: real acts after act 3 with routes, summary act/page, late boss caps, card cap 4, card/relic tuning, alarm pad grace, Arithmagistrate key quiz, portal occlusion, codex clip, equal grades
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="798">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="797">
   <si>
     <r>
       <rPr>
@@ -2629,7 +2629,65 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3</t>
+      <t xml:space="preserve">2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
     </r>
   </si>
   <si>
@@ -2650,7 +2708,65 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4</t>
+      <t xml:space="preserve">3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
     </r>
   </si>
   <si>
@@ -2669,6 +2785,50 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">片環繞的紙盾，每片可抵擋一次攻擊，持續 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">召喚 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">3 </t>
     </r>
     <r>
@@ -2677,34 +2837,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">片環繞的紙盾，每片可抵擋一次攻擊。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">召喚 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">片環繞的紙盾，每片可抵擋一次攻擊。</t>
+      <t xml:space="preserve">片環繞的紙盾，每片可抵擋一次攻擊，持續 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒。</t>
     </r>
   </si>
   <si>
@@ -2986,6 +3136,27 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回復：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">2</t>
     </r>
   </si>
@@ -2993,27 +3164,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">回復：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -3026,34 +3176,34 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">塗上修正液，回復 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點生命。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">塗上修正液，回復 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
     </r>
     <r>
       <rPr>
@@ -7537,7 +7687,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4</t>
+      <t xml:space="preserve">5</t>
     </r>
   </si>
   <si>
@@ -7556,7 +7706,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4 </t>
+      <t xml:space="preserve">5 </t>
     </r>
     <r>
       <rPr>
@@ -7941,65 +8091,6 @@
   </si>
   <si>
     <t xml:space="preserve">傀儡</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
   </si>
   <si>
     <r>
@@ -12575,7 +12666,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">時，角落會亮起紅色閃動的鬧鐘圈。站在圈內不會受到任何傷害；待約 </t>
+      <t xml:space="preserve">時，角落會亮起紅色閃動的鬧鐘圈。站在圈內不會受到任何傷害（圈消失後 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內也是）；待約 </t>
     </r>
     <r>
       <rPr>
@@ -12849,7 +12957,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{'r': 1.4, 'hold': 0.8, 'hold2': 0.6, 'decay': 0.5, 'inset': 2.4, 'minDist': 5, 'avoid': 0.45, 'vanish': 0.3, 'safe': 0.15}
+      <t xml:space="preserve">{'r': 1.4, 'hold': 0.8, 'hold2': 0.6, 'decay': 0.5, 'inset': 2.4, 'minDist': 5, 'avoid': 0.45, 'vanish': 0.3, 'safe': 0.15, 'linger': 0.6}
 snooze</t>
     </r>
     <r>
@@ -24838,7 +24946,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">擊敗計算機魔王 </t>
+      <t xml:space="preserve">擊敗加減法官 </t>
     </r>
     <r>
       <rPr>
@@ -30551,7 +30659,7 @@
       </c>
       <c r="P9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>95</v>
       </c>
@@ -31938,11 +32046,11 @@
         <v>3</v>
       </c>
       <c r="L39" s="14" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="O39" s="12" t="s">
         <v>87</v>
@@ -31951,10 +32059,10 @@
     </row>
     <row r="40" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="B40" s="12" t="s">
         <v>270</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>271</v>
       </c>
       <c r="C40" s="12" t="s">
         <v>238</v>
@@ -31982,11 +32090,11 @@
         <v>3</v>
       </c>
       <c r="L40" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="M40" s="13"/>
       <c r="N40" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="O40" s="12" t="s">
         <v>87</v>
@@ -31995,10 +32103,10 @@
     </row>
     <row r="41" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B41" s="12" t="s">
         <v>274</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>275</v>
       </c>
       <c r="C41" s="12" t="s">
         <v>238</v>
@@ -32007,7 +32115,7 @@
         <v>36</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F41" s="12" t="s">
         <v>38</v>
@@ -32028,11 +32136,11 @@
         <v>3</v>
       </c>
       <c r="L41" s="14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="M41" s="13"/>
       <c r="N41" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="O41" s="12" t="s">
         <v>87</v>
@@ -32041,10 +32149,10 @@
     </row>
     <row r="42" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="B42" s="12" t="s">
         <v>279</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>280</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>238</v>
@@ -32076,7 +32184,7 @@
       </c>
       <c r="M42" s="13"/>
       <c r="N42" s="12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="O42" s="12" t="s">
         <v>87</v>
@@ -32085,10 +32193,10 @@
     </row>
     <row r="43" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>282</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>283</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>238</v>
@@ -32116,11 +32224,11 @@
         <v>3</v>
       </c>
       <c r="L43" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="M43" s="13"/>
       <c r="N43" s="12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O43" s="12" t="s">
         <v>87</v>
@@ -32164,13 +32272,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B1" s="15" t="n">
         <v>2.5</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D1" s="15" t="n">
         <v>2</v>
@@ -32187,40 +32295,40 @@
         <v>20</v>
       </c>
       <c r="D3" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="J3" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="K3" s="5" t="s">
         <v>294</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="L3" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="M3" s="5" t="s">
         <v>296</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="N3" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="O3" s="5" t="s">
         <v>298</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>299</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>32</v>
@@ -32228,13 +32336,13 @@
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>301</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>302</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>38</v>
@@ -32256,7 +32364,7 @@
         <v>10</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>1</v>
@@ -32269,22 +32377,22 @@
         <v>1</v>
       </c>
       <c r="N4" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>304</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>305</v>
       </c>
       <c r="P4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>306</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>307</v>
-      </c>
       <c r="C5" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>52</v>
@@ -32317,22 +32425,22 @@
         <v>2</v>
       </c>
       <c r="N5" s="7" t="s">
+        <v>307</v>
+      </c>
+      <c r="O5" s="6" t="s">
         <v>308</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>309</v>
       </c>
       <c r="P5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>310</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>311</v>
-      </c>
       <c r="C6" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>46</v>
@@ -32354,7 +32462,7 @@
         <v>8.5</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="K6" s="8" t="n">
         <v>1.5</v>
@@ -32367,22 +32475,22 @@
         <v>2</v>
       </c>
       <c r="N6" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="O6" s="6" t="s">
         <v>313</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>314</v>
       </c>
       <c r="P6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="270.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>315</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>316</v>
-      </c>
       <c r="C7" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>64</v>
@@ -32415,22 +32523,22 @@
         <v>2</v>
       </c>
       <c r="N7" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>317</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>318</v>
       </c>
       <c r="P7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="243.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>319</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>320</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>321</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>44</v>
@@ -32459,22 +32567,22 @@
         <v>2</v>
       </c>
       <c r="N8" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="O8" s="6" t="s">
         <v>322</v>
-      </c>
-      <c r="O8" s="6" t="s">
-        <v>323</v>
       </c>
       <c r="P8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>325</v>
-      </c>
       <c r="C9" s="7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>26</v>
@@ -32503,22 +32611,22 @@
         <v>1</v>
       </c>
       <c r="N9" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="O9" s="6" t="s">
         <v>326</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>327</v>
       </c>
       <c r="P9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>328</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>329</v>
-      </c>
       <c r="C10" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>58</v>
@@ -32540,7 +32648,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K10" s="8" t="n">
         <v>1.5</v>
@@ -32553,22 +32661,22 @@
         <v>2</v>
       </c>
       <c r="N10" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="O10" s="6" t="s">
         <v>331</v>
-      </c>
-      <c r="O10" s="6" t="s">
-        <v>332</v>
       </c>
       <c r="P10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>334</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>90</v>
@@ -32597,22 +32705,22 @@
         <v>2</v>
       </c>
       <c r="N11" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="O11" s="6" t="s">
         <v>335</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>336</v>
       </c>
       <c r="P11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>337</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>338</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>14</v>
@@ -32642,25 +32750,25 @@
       </c>
       <c r="N12" s="7"/>
       <c r="O12" s="6" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="P12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
+        <v>339</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>340</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="C13" s="12" t="s">
         <v>341</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>342</v>
       </c>
       <c r="D13" s="13" t="n">
         <v>900</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F13" s="13" t="n">
         <v>0.8</v>
@@ -32679,32 +32787,32 @@
         <v>4</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="O13" s="11" t="s">
         <v>345</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>346</v>
       </c>
       <c r="P13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="161.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>347</v>
       </c>
-      <c r="B14" s="12" t="s">
-        <v>348</v>
-      </c>
       <c r="C14" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>1000</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F14" s="13" t="n">
         <v>2.2</v>
@@ -32723,32 +32831,32 @@
         <v>4</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="O14" s="11" t="s">
         <v>349</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>350</v>
       </c>
       <c r="P14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>351</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>352</v>
-      </c>
       <c r="C15" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1300</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F15" s="13" t="n">
         <v>0</v>
@@ -32767,32 +32875,32 @@
         <v>4</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="O15" s="11" t="s">
         <v>353</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>354</v>
       </c>
       <c r="P15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="331.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>355</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>356</v>
-      </c>
       <c r="C16" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1100</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>1.4</v>
@@ -32811,32 +32919,32 @@
         <v>4</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="12" t="s">
+        <v>356</v>
+      </c>
+      <c r="O16" s="11" t="s">
         <v>357</v>
-      </c>
-      <c r="O16" s="11" t="s">
-        <v>358</v>
       </c>
       <c r="P16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="252.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>359</v>
       </c>
-      <c r="B17" s="12" t="s">
-        <v>360</v>
-      </c>
       <c r="C17" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1400</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>0</v>
@@ -32855,32 +32963,32 @@
         <v>5</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="O17" s="11" t="s">
         <v>361</v>
-      </c>
-      <c r="O17" s="11" t="s">
-        <v>362</v>
       </c>
       <c r="P17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="381.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
+        <v>362</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>363</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>364</v>
-      </c>
       <c r="C18" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D18" s="13" t="n">
         <v>1300</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F18" s="13" t="n">
         <v>0</v>
@@ -32897,26 +33005,26 @@
         <v>4</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="M18" s="13"/>
       <c r="N18" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="O18" s="11" t="s">
         <v>365</v>
-      </c>
-      <c r="O18" s="11" t="s">
-        <v>366</v>
       </c>
       <c r="P18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>367</v>
       </c>
-      <c r="B19" s="7" t="s">
-        <v>368</v>
-      </c>
       <c r="C19" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>45</v>
@@ -32946,7 +33054,7 @@
       </c>
       <c r="N19" s="7"/>
       <c r="O19" s="6" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P19" s="10"/>
     </row>
@@ -32996,37 +33104,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>372</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>373</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>377</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>378</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -33034,16 +33142,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>379</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>380</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -33078,16 +33186,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>382</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>383</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -33122,16 +33230,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>385</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>386</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -33162,22 +33270,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>389</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>390</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -33208,22 +33316,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>393</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>394</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>8</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -33241,10 +33349,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -33254,22 +33362,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -33281,10 +33389,10 @@
         <v>1.8</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -33300,22 +33408,22 @@
         <v>11.1</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="O7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>400</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>401</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>13</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>5</v>
@@ -33346,7 +33454,7 @@
         <v>33.3</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="O8" s="10"/>
     </row>
@@ -33378,19 +33486,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>406</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>407</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -33398,325 +33506,325 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>408</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>411</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>412</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>413</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>416</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>417</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="9" t="s">
         <v>421</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>422</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>423</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>424</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>425</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>426</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>427</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>428</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="9" t="s">
         <v>430</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>431</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>431</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>432</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>433</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>434</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="9" t="s">
         <v>435</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>436</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>437</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>438</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="9" t="s">
         <v>440</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>441</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>442</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="7" t="s">
         <v>443</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="7" t="s">
         <v>444</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="9" t="s">
         <v>445</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>446</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>447</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>448</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>449</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="9" t="s">
         <v>450</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>451</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>452</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>453</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>454</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="E11" s="9" t="s">
         <v>455</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>456</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>458</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="E12" s="9" t="s">
         <v>459</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>460</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>461</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="C13" s="7" t="s">
         <v>462</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>463</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="9" t="s">
         <v>464</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>465</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>466</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>467</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>468</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="9" t="s">
         <v>469</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>470</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>471</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="C15" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="9" t="s">
         <v>474</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>475</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="C16" s="7" t="s">
         <v>477</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>478</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="9" t="s">
         <v>479</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>480</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="7" t="s">
         <v>483</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="8" t="s">
         <v>484</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>485</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="377.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>486</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>487</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>488</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E18" s="9" t="s">
         <v>489</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>490</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>491</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="7" t="s">
         <v>492</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>493</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="9" t="s">
         <v>494</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>495</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -33751,13 +33859,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>496</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>497</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>498</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -33765,13 +33873,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
@@ -33781,13 +33889,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
@@ -33797,13 +33905,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
@@ -33813,13 +33921,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
@@ -33829,13 +33937,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
@@ -33845,13 +33953,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
@@ -33861,13 +33969,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
@@ -33877,13 +33985,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
@@ -33893,13 +34001,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
@@ -33909,13 +34017,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
@@ -33925,13 +34033,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
@@ -33941,13 +34049,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
@@ -33957,13 +34065,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
@@ -33973,13 +34081,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
@@ -33989,13 +34097,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
@@ -34005,13 +34113,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
@@ -34021,13 +34129,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
@@ -34037,13 +34145,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
@@ -34053,13 +34161,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>
@@ -34095,16 +34203,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>521</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>522</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -34112,13 +34220,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>522</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>523</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>524</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>525</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -34127,13 +34235,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>525</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>526</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>527</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -34142,13 +34250,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>527</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>528</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>529</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>25</v>
@@ -34157,13 +34265,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>529</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>530</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>531</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>532</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -34172,13 +34280,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -34187,13 +34295,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>535</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>536</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -34202,13 +34310,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>536</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>537</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>538</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>539</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -34217,13 +34325,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>540</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>541</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -34232,13 +34340,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>542</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>543</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -34247,13 +34355,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>544</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>545</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -34262,13 +34370,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -34277,28 +34385,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>547</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="8" t="s">
         <v>548</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>549</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>549</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>550</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="C14" s="7" t="s">
         <v>551</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>552</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2</v>
@@ -34307,28 +34415,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>552</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>553</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>554</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>555</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>556</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>557</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>1</v>
@@ -34337,10 +34445,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>557</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>558</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>559</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
@@ -34350,13 +34458,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>559</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>560</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>561</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>5</v>
@@ -34365,10 +34473,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
@@ -34378,10 +34486,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
@@ -34391,10 +34499,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -34404,13 +34512,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
+        <v>564</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>565</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="C22" s="7" t="s">
         <v>566</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>567</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>60000</v>
@@ -34419,13 +34527,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>567</v>
+      </c>
+      <c r="C23" s="7" t="s">
         <v>568</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>569</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>45000</v>
@@ -34434,13 +34542,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>569</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>570</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>571</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>35000</v>
@@ -34449,13 +34557,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>571</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>572</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>573</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>20000</v>
@@ -34464,13 +34572,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>574</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>575</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10000</v>
@@ -34479,13 +34587,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>575</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>576</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>577</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5000</v>
@@ -34494,88 +34602,88 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>110000</v>
+        <v>60000</v>
       </c>
       <c r="E28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>80000</v>
+        <v>45000</v>
       </c>
       <c r="E29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>60000</v>
+        <v>35000</v>
       </c>
       <c r="E30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="E31" s="10"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="E32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>5000</v>
@@ -34584,616 +34692,616 @@
     </row>
     <row r="34" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B34" s="7" t="s">
         <v>584</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="C34" s="7" t="s">
         <v>585</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="D34" s="8" t="s">
         <v>586</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>587</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B35" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>588</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="D35" s="8" t="s">
         <v>589</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>590</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>591</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D36" s="8" t="s">
         <v>592</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>593</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B37" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>594</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="D37" s="8" t="s">
         <v>595</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>596</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B38" s="7" t="s">
+        <v>596</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>597</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="D38" s="8" t="s">
         <v>598</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>599</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B39" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>600</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="D39" s="8" t="s">
         <v>601</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>602</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>602</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>603</v>
       </c>
-      <c r="C40" s="7" t="s">
-        <v>604</v>
-      </c>
       <c r="D40" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B41" s="7" t="s">
+        <v>604</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>605</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>606</v>
-      </c>
       <c r="D41" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>606</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>607</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>608</v>
-      </c>
       <c r="D42" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B43" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="C43" s="7" t="s">
         <v>609</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>610</v>
-      </c>
       <c r="D43" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B44" s="7" t="s">
+        <v>610</v>
+      </c>
+      <c r="C44" s="7" t="s">
         <v>611</v>
       </c>
-      <c r="C44" s="7" t="s">
-        <v>612</v>
-      </c>
       <c r="D44" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B45" s="7" t="s">
+        <v>612</v>
+      </c>
+      <c r="C45" s="7" t="s">
         <v>613</v>
       </c>
-      <c r="C45" s="7" t="s">
-        <v>614</v>
-      </c>
       <c r="D45" s="8" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B46" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="C46" s="7" t="s">
         <v>615</v>
       </c>
-      <c r="C46" s="7" t="s">
-        <v>616</v>
-      </c>
       <c r="D46" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B47" s="7" t="s">
+        <v>616</v>
+      </c>
+      <c r="C47" s="7" t="s">
         <v>617</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="D47" s="8" t="s">
         <v>618</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>619</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="C48" s="7" t="s">
         <v>620</v>
       </c>
-      <c r="C48" s="7" t="s">
-        <v>621</v>
-      </c>
       <c r="D48" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B49" s="7" t="s">
+        <v>621</v>
+      </c>
+      <c r="C49" s="7" t="s">
         <v>622</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="D49" s="8" t="s">
         <v>623</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>624</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B50" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="C50" s="6" t="s">
         <v>625</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="D50" s="8" t="s">
         <v>626</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>627</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B51" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="C51" s="7" t="s">
         <v>628</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="D51" s="8" t="s">
         <v>629</v>
-      </c>
-      <c r="D51" s="8" t="s">
-        <v>630</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B52" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="C52" s="7" t="s">
         <v>631</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="D52" s="8" t="s">
         <v>632</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>633</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B53" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="C53" s="7" t="s">
         <v>634</v>
       </c>
-      <c r="C53" s="7" t="s">
-        <v>635</v>
-      </c>
       <c r="D53" s="8" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B54" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="C54" s="7" t="s">
         <v>636</v>
       </c>
-      <c r="C54" s="7" t="s">
-        <v>637</v>
-      </c>
       <c r="D54" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B55" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="C55" s="7" t="s">
         <v>638</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="D55" s="8" t="s">
         <v>639</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>640</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B56" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="C56" s="7" t="s">
         <v>641</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="D56" s="8" t="s">
         <v>642</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>643</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B57" s="7" t="s">
+        <v>643</v>
+      </c>
+      <c r="C57" s="7" t="s">
         <v>644</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="D57" s="8" t="s">
         <v>645</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>646</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B58" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="C58" s="7" t="s">
         <v>647</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="D58" s="8" t="s">
         <v>648</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>649</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B59" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="C59" s="7" t="s">
         <v>650</v>
       </c>
-      <c r="C59" s="7" t="s">
-        <v>651</v>
-      </c>
       <c r="D59" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B60" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="C60" s="7" t="s">
         <v>652</v>
       </c>
-      <c r="C60" s="7" t="s">
-        <v>653</v>
-      </c>
       <c r="D60" s="8" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B61" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="C61" s="7" t="s">
         <v>654</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="D61" s="8" t="s">
         <v>655</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>656</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B62" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="C62" s="7" t="s">
         <v>657</v>
       </c>
-      <c r="C62" s="7" t="s">
+      <c r="D62" s="8" t="s">
         <v>658</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>659</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B63" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="C63" s="7" t="s">
         <v>660</v>
       </c>
-      <c r="C63" s="7" t="s">
+      <c r="D63" s="8" t="s">
         <v>661</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>662</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B64" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="C64" s="7" t="s">
         <v>663</v>
       </c>
-      <c r="C64" s="7" t="s">
-        <v>664</v>
-      </c>
       <c r="D64" s="8" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B65" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="C65" s="7" t="s">
         <v>665</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="D65" s="8" t="s">
         <v>666</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>667</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B66" s="7" t="s">
+        <v>667</v>
+      </c>
+      <c r="C66" s="7" t="s">
         <v>668</v>
       </c>
-      <c r="C66" s="7" t="s">
-        <v>669</v>
-      </c>
       <c r="D66" s="8" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B67" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="C67" s="7" t="s">
         <v>670</v>
       </c>
-      <c r="C67" s="7" t="s">
-        <v>671</v>
-      </c>
       <c r="D67" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B68" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="C68" s="7" t="s">
         <v>672</v>
       </c>
-      <c r="C68" s="7" t="s">
+      <c r="D68" s="8" t="s">
         <v>673</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>674</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B69" s="7" t="s">
+        <v>674</v>
+      </c>
+      <c r="C69" s="7" t="s">
         <v>675</v>
       </c>
-      <c r="C69" s="7" t="s">
+      <c r="D69" s="8" t="s">
         <v>676</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>677</v>
       </c>
       <c r="E69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B70" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="C70" s="7" t="s">
         <v>678</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="D70" s="8" t="s">
         <v>679</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>680</v>
       </c>
       <c r="E70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B71" s="7" t="s">
+        <v>680</v>
+      </c>
+      <c r="C71" s="7" t="s">
         <v>681</v>
       </c>
-      <c r="C71" s="7" t="s">
+      <c r="D71" s="8" t="s">
         <v>682</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>683</v>
       </c>
       <c r="E71" s="10"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B72" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="C72" s="7" t="s">
         <v>684</v>
       </c>
-      <c r="C72" s="7" t="s">
-        <v>685</v>
-      </c>
       <c r="D72" s="8" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B73" s="7" t="s">
+        <v>685</v>
+      </c>
+      <c r="C73" s="7" t="s">
         <v>686</v>
       </c>
-      <c r="C73" s="7" t="s">
+      <c r="D73" s="8" t="s">
         <v>687</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>688</v>
       </c>
       <c r="E73" s="10"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B74" s="7" t="s">
+        <v>688</v>
+      </c>
+      <c r="C74" s="7" t="s">
         <v>689</v>
       </c>
-      <c r="C74" s="7" t="s">
+      <c r="D74" s="8" t="s">
         <v>690</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>691</v>
       </c>
       <c r="E74" s="10"/>
     </row>
@@ -35225,19 +35333,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
+        <v>691</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>692</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>497</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>693</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>694</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>695</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -35245,370 +35353,370 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>696</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>697</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>698</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>701</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>702</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>703</v>
-      </c>
       <c r="C4" s="6" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>705</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>706</v>
-      </c>
       <c r="C5" s="6" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>708</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>709</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>710</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>711</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>712</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
+        <v>713</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>714</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>715</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>717</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>718</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>720</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>721</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
+        <v>722</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>723</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>724</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>726</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>727</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>728</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>729</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>730</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>731</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>732</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>733</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
+        <v>734</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>735</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>736</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>737</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>738</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>739</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>741</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>742</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>744</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>745</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>746</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>747</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>748</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
+        <v>748</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>749</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>750</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
+        <v>751</v>
+      </c>
+      <c r="B21" s="7" t="s">
         <v>752</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>753</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
+        <v>754</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>755</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>756</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>757</v>
+      </c>
+      <c r="B23" s="7" t="s">
         <v>758</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>759</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
+        <v>760</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>761</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>762</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -35647,22 +35755,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
+        <v>762</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>763</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>521</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>764</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>765</v>
-      </c>
       <c r="F1" s="5" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -35670,115 +35778,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>766</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>767</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>768</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>769</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="8" t="s">
         <v>770</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>771</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>771</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>772</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="C3" s="7" t="s">
         <v>773</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>774</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="7" t="s">
         <v>775</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="8" t="s">
         <v>776</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>777</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>777</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>778</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
         <v>779</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>780</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>781</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>782</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>783</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>783</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>784</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>785</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>786</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>787</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>788</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>789</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>790</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>791</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>792</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>793</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="8" t="s">
         <v>794</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>795</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>795</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>796</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>797</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
beta v0.10.37: late summons capped, Arithmagistrate fixes (no interact on keys, 9/8s, sweep edge warning, wider gap), kill ink, event balance with max HP/ink 8-12, shield icon, achievement fling scroll
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1117" uniqueCount="797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="799">
   <si>
     <r>
       <rPr>
@@ -23355,16 +23355,77 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">墨水 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">+4</t>
+      <t xml:space="preserve">墨水上限 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、墨水 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">生命上限 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、回復 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">生命</t>
     </r>
   </si>
   <si>
@@ -23533,6 +23594,25 @@
   </si>
   <si>
     <t xml:space="preserve">下一場一般戰變精英戰</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水上限 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-1</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">觸發伏擊戰</t>
@@ -32651,11 +32731,11 @@
         <v>329</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">K10*$D$1</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M10" s="8" t="n">
         <v>2</v>
@@ -32695,11 +32775,11 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
       <c r="K11" s="8" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">K11*$D$1</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M11" s="8" t="n">
         <v>2</v>
@@ -33844,7 +33924,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -33882,7 +33962,7 @@
         <v>499</v>
       </c>
       <c r="D2" s="16" t="n">
-        <f aca="false">ROUND(B2/SUM(B$2:B$12),3)</f>
+        <f aca="false">ROUND(B2/SUM(B$2:B$13),3)</f>
         <v>0.15</v>
       </c>
       <c r="E2" s="10"/>
@@ -33898,7 +33978,7 @@
         <v>500</v>
       </c>
       <c r="D3" s="16" t="n">
-        <f aca="false">ROUND(B3/SUM(B$2:B$12),3)</f>
+        <f aca="false">ROUND(B3/SUM(B$2:B$13),3)</f>
         <v>0.1</v>
       </c>
       <c r="E3" s="10"/>
@@ -33914,7 +33994,7 @@
         <v>501</v>
       </c>
       <c r="D4" s="16" t="n">
-        <f aca="false">ROUND(B4/SUM(B$2:B$12),3)</f>
+        <f aca="false">ROUND(B4/SUM(B$2:B$13),3)</f>
         <v>0.15</v>
       </c>
       <c r="E4" s="10"/>
@@ -33930,7 +34010,7 @@
         <v>502</v>
       </c>
       <c r="D5" s="16" t="n">
-        <f aca="false">ROUND(B5/SUM(B$2:B$12),3)</f>
+        <f aca="false">ROUND(B5/SUM(B$2:B$13),3)</f>
         <v>0.05</v>
       </c>
       <c r="E5" s="10"/>
@@ -33946,7 +34026,7 @@
         <v>503</v>
       </c>
       <c r="D6" s="16" t="n">
-        <f aca="false">ROUND(B6/SUM(B$2:B$12),3)</f>
+        <f aca="false">ROUND(B6/SUM(B$2:B$13),3)</f>
         <v>0.1</v>
       </c>
       <c r="E6" s="10"/>
@@ -33956,14 +34036,14 @@
         <v>498</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>504</v>
       </c>
       <c r="D7" s="16" t="n">
-        <f aca="false">ROUND(B7/SUM(B$2:B$12),3)</f>
-        <v>0.1</v>
+        <f aca="false">ROUND(B7/SUM(B$2:B$13),3)</f>
+        <v>0.05</v>
       </c>
       <c r="E7" s="10"/>
     </row>
@@ -33972,14 +34052,14 @@
         <v>498</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>505</v>
       </c>
       <c r="D8" s="16" t="n">
-        <f aca="false">ROUND(B8/SUM(B$2:B$12),3)</f>
-        <v>0.1</v>
+        <f aca="false">ROUND(B8/SUM(B$2:B$13),3)</f>
+        <v>0.05</v>
       </c>
       <c r="E8" s="10"/>
     </row>
@@ -33988,14 +34068,14 @@
         <v>498</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>506</v>
       </c>
       <c r="D9" s="16" t="n">
-        <f aca="false">ROUND(B9/SUM(B$2:B$12),3)</f>
-        <v>0.05</v>
+        <f aca="false">ROUND(B9/SUM(B$2:B$13),3)</f>
+        <v>0.1</v>
       </c>
       <c r="E9" s="10"/>
     </row>
@@ -34004,14 +34084,14 @@
         <v>498</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>507</v>
       </c>
       <c r="D10" s="16" t="n">
-        <f aca="false">ROUND(B10/SUM(B$2:B$12),3)</f>
-        <v>0.1</v>
+        <f aca="false">ROUND(B10/SUM(B$2:B$13),3)</f>
+        <v>0.05</v>
       </c>
       <c r="E10" s="10"/>
     </row>
@@ -34020,14 +34100,14 @@
         <v>498</v>
       </c>
       <c r="B11" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>508</v>
       </c>
       <c r="D11" s="16" t="n">
-        <f aca="false">ROUND(B11/SUM(B$2:B$12),3)</f>
-        <v>0.05</v>
+        <f aca="false">ROUND(B11/SUM(B$2:B$13),3)</f>
+        <v>0.1</v>
       </c>
       <c r="E11" s="10"/>
     </row>
@@ -34042,78 +34122,78 @@
         <v>509</v>
       </c>
       <c r="D12" s="16" t="n">
-        <f aca="false">ROUND(B12/SUM(B$2:B$12),3)</f>
+        <f aca="false">ROUND(B12/SUM(B$2:B$13),3)</f>
         <v>0.05</v>
       </c>
       <c r="E12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>510</v>
       </c>
-      <c r="B13" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>511</v>
-      </c>
       <c r="D13" s="16" t="n">
-        <f aca="false">ROUND(B13/SUM(B$13:B$20),3)</f>
-        <v>0.2</v>
+        <f aca="false">ROUND(B13/SUM(B$2:B$13),3)</f>
+        <v>0.05</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B14" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>512</v>
       </c>
       <c r="D14" s="16" t="n">
-        <f aca="false">ROUND(B14/SUM(B$13:B$20),3)</f>
-        <v>0.067</v>
+        <f aca="false">ROUND(B14/SUM(B$14:B$22),3)</f>
+        <v>0.188</v>
       </c>
       <c r="E14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B15" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>513</v>
       </c>
       <c r="D15" s="16" t="n">
-        <f aca="false">ROUND(B15/SUM(B$13:B$20),3)</f>
-        <v>0.2</v>
+        <f aca="false">ROUND(B15/SUM(B$14:B$22),3)</f>
+        <v>0.063</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B16" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>514</v>
       </c>
       <c r="D16" s="16" t="n">
-        <f aca="false">ROUND(B16/SUM(B$13:B$20),3)</f>
-        <v>0.133</v>
+        <f aca="false">ROUND(B16/SUM(B$14:B$22),3)</f>
+        <v>0.188</v>
       </c>
       <c r="E16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
@@ -34122,14 +34202,14 @@
         <v>515</v>
       </c>
       <c r="D17" s="16" t="n">
-        <f aca="false">ROUND(B17/SUM(B$13:B$20),3)</f>
-        <v>0.133</v>
+        <f aca="false">ROUND(B17/SUM(B$14:B$22),3)</f>
+        <v>0.125</v>
       </c>
       <c r="E17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
@@ -34138,30 +34218,30 @@
         <v>516</v>
       </c>
       <c r="D18" s="16" t="n">
-        <f aca="false">ROUND(B18/SUM(B$13:B$20),3)</f>
-        <v>0.133</v>
+        <f aca="false">ROUND(B18/SUM(B$14:B$22),3)</f>
+        <v>0.125</v>
       </c>
       <c r="E18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B19" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>517</v>
       </c>
       <c r="D19" s="16" t="n">
-        <f aca="false">ROUND(B19/SUM(B$13:B$20),3)</f>
-        <v>0.067</v>
+        <f aca="false">ROUND(B19/SUM(B$14:B$22),3)</f>
+        <v>0.125</v>
       </c>
       <c r="E19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
@@ -34170,10 +34250,42 @@
         <v>518</v>
       </c>
       <c r="D20" s="16" t="n">
-        <f aca="false">ROUND(B20/SUM(B$13:B$20),3)</f>
-        <v>0.067</v>
+        <f aca="false">ROUND(B20/SUM(B$14:B$22),3)</f>
+        <v>0.063</v>
       </c>
       <c r="E20" s="10"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>519</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <f aca="false">ROUND(B21/SUM(B$14:B$22),3)</f>
+        <v>0.063</v>
+      </c>
+      <c r="E21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>511</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>520</v>
+      </c>
+      <c r="D22" s="16" t="n">
+        <f aca="false">ROUND(B22/SUM(B$14:B$22),3)</f>
+        <v>0.063</v>
+      </c>
+      <c r="E22" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -34203,16 +34315,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -34220,13 +34332,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -34235,13 +34347,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -34250,13 +34362,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>25</v>
@@ -34265,13 +34377,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -34280,13 +34392,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -34295,13 +34407,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -34310,13 +34422,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -34325,13 +34437,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -34340,13 +34452,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -34355,13 +34467,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -34370,13 +34482,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -34385,28 +34497,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2</v>
@@ -34415,28 +34527,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>1</v>
@@ -34445,10 +34557,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
@@ -34458,13 +34570,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>5</v>
@@ -34473,10 +34585,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
@@ -34486,10 +34598,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
@@ -34499,10 +34611,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -34512,13 +34624,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>60000</v>
@@ -34527,13 +34639,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>45000</v>
@@ -34542,13 +34654,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>35000</v>
@@ -34557,13 +34669,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>20000</v>
@@ -34572,13 +34684,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10000</v>
@@ -34587,13 +34699,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5000</v>
@@ -34602,13 +34714,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>60000</v>
@@ -34617,13 +34729,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>45000</v>
@@ -34632,13 +34744,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>35000</v>
@@ -34647,13 +34759,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>20000</v>
@@ -34662,13 +34774,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>10000</v>
@@ -34677,13 +34789,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>5000</v>
@@ -34692,616 +34804,616 @@
     </row>
     <row r="34" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="C40" s="7" t="s">
+        <v>605</v>
+      </c>
+      <c r="D40" s="8" t="s">
         <v>603</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>601</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C53" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="D53" s="8" t="s">
         <v>634</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>632</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="E69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="E70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="E71" s="10"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="E73" s="10"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="E74" s="10"/>
     </row>
@@ -35333,19 +35445,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>496</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -35353,19 +35465,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -35374,349 +35486,349 @@
         <v>433</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>701</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>699</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>697</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -35755,22 +35867,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>377</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -35778,115 +35890,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>